<commit_message>
Integrate 4.0.4: commit #f24eca9, 1/23/25, Add policy lever for policy lever additions and load in data to swap in IRA repeal for agricultural incentives, repeal EPA methane rules, and repeal AIM Act
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C977ABCA-1BB2-4D89-9B53-88D4D882D946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B01FBE4-3B6E-4E45-A6AB-63D6C15D47FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1466" uniqueCount="848">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2564,6 +2564,18 @@
   </si>
   <si>
     <t>You plan on using a policy mandated change in distributed solar capacity additions</t>
+  </si>
+  <si>
+    <t>PEAAC</t>
+  </si>
+  <si>
+    <t>Process Emissions Additions and Costs</t>
+  </si>
+  <si>
+    <t>Process Emissions Additions and Costs, Marginal Cost Definitions</t>
+  </si>
+  <si>
+    <t>You want to test the addition rather than the reduction of process emissions for select industries</t>
   </si>
 </sst>
 </file>
@@ -3375,7 +3387,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G308"/>
+  <dimension ref="A1:G309"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
@@ -6462,44 +6474,50 @@
         <v>63</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>65</v>
+        <v>844</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>67</v>
+        <v>845</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="F199" s="14" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
+        <v>846</v>
+      </c>
+      <c r="F199" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G199" s="2" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>188</v>
+        <v>65</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="F200" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="201" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+      <c r="D200" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="F200" s="14" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>554</v>
+        <v>188</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>555</v>
-      </c>
-      <c r="F201" s="5" t="s">
-        <v>99</v>
+        <v>189</v>
+      </c>
+      <c r="F201" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="202" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6507,38 +6525,38 @@
         <v>63</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>815</v>
+        <v>554</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>816</v>
-      </c>
-      <c r="F202" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.35">
+        <v>555</v>
+      </c>
+      <c r="F202" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>464</v>
+        <v>815</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>463</v>
+        <v>816</v>
       </c>
       <c r="F203" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="204" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>480</v>
+        <v>464</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>481</v>
+        <v>463</v>
       </c>
       <c r="F204" s="4" t="s">
         <v>98</v>
@@ -6549,13 +6567,13 @@
         <v>63</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>822</v>
+        <v>480</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>823</v>
-      </c>
-      <c r="F205" s="5" t="s">
-        <v>99</v>
+        <v>481</v>
+      </c>
+      <c r="F205" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="206" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6563,75 +6581,72 @@
         <v>63</v>
       </c>
       <c r="B206" s="2" t="s">
+        <v>822</v>
+      </c>
+      <c r="C206" s="2" t="s">
+        <v>823</v>
+      </c>
+      <c r="F206" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A207" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B207" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="C206" s="2" t="s">
+      <c r="C207" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="F206" s="4" t="s">
+      <c r="F207" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="207" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A207" s="17" t="s">
+    <row r="208" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A208" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B207" s="17" t="s">
+      <c r="B208" s="17" t="s">
         <v>832</v>
       </c>
-      <c r="C207" s="17" t="s">
+      <c r="C208" s="17" t="s">
         <v>833</v>
       </c>
-      <c r="D207" s="17"/>
-      <c r="E207" s="17"/>
-      <c r="F207" s="19" t="s">
+      <c r="D208" s="17"/>
+      <c r="E208" s="17"/>
+      <c r="F208" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="G207" s="17"/>
-    </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A208" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="B208" s="2" t="s">
-        <v>788</v>
-      </c>
-      <c r="C208" s="2" t="s">
-        <v>789</v>
-      </c>
-      <c r="F208" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="209" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="G208" s="17"/>
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>546</v>
+        <v>788</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>547</v>
-      </c>
-      <c r="D209" s="2" t="s">
-        <v>548</v>
+        <v>789</v>
       </c>
       <c r="F209" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>697</v>
+        <v>546</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>698</v>
+        <v>547</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>696</v>
+        <v>548</v>
       </c>
       <c r="F210" s="3" t="s">
         <v>97</v>
@@ -6642,10 +6657,13 @@
         <v>407</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>415</v>
+        <v>697</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>416</v>
+        <v>698</v>
+      </c>
+      <c r="D211" s="2" t="s">
+        <v>696</v>
       </c>
       <c r="F211" s="3" t="s">
         <v>97</v>
@@ -6656,10 +6674,10 @@
         <v>407</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="F212" s="3" t="s">
         <v>97</v>
@@ -6670,10 +6688,10 @@
         <v>407</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>388</v>
+        <v>417</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>389</v>
+        <v>418</v>
       </c>
       <c r="F213" s="3" t="s">
         <v>97</v>
@@ -6684,44 +6702,44 @@
         <v>407</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>419</v>
+        <v>388</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>420</v>
+        <v>389</v>
       </c>
       <c r="F214" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="215" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A215" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>600</v>
+        <v>419</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>602</v>
-      </c>
-      <c r="D215" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="E215" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="F215" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B216" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="C216" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="D216" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="E216" s="2" t="s">
         <v>421</v>
-      </c>
-      <c r="C216" s="2" t="s">
-        <v>422</v>
       </c>
       <c r="F216" s="3" t="s">
         <v>97</v>
@@ -6732,30 +6750,27 @@
         <v>407</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>411</v>
+        <v>422</v>
       </c>
       <c r="F217" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="218" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>517</v>
+        <v>409</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="F218" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G218" s="2" t="s">
-        <v>519</v>
+        <v>411</v>
+      </c>
+      <c r="F218" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="219" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6763,48 +6778,48 @@
         <v>407</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>467</v>
+        <v>517</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="D219" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="F219" s="3"/>
-    </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
+        <v>518</v>
+      </c>
+      <c r="F219" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G219" s="2" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>515</v>
+        <v>467</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="F220" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G220" s="2" t="s">
-        <v>520</v>
-      </c>
+        <v>468</v>
+      </c>
+      <c r="D220" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="F220" s="3"/>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>490</v>
+        <v>515</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>491</v>
-      </c>
-      <c r="E221" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="F221" s="3" t="s">
-        <v>97</v>
+        <v>516</v>
+      </c>
+      <c r="F221" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G221" s="2" t="s">
+        <v>520</v>
       </c>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.35">
@@ -6812,13 +6827,16 @@
         <v>407</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>489</v>
-      </c>
-      <c r="F222" s="5" t="s">
-        <v>99</v>
+        <v>491</v>
+      </c>
+      <c r="E222" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F222" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.35">
@@ -6826,10 +6844,10 @@
         <v>407</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>454</v>
+        <v>488</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>455</v>
+        <v>489</v>
       </c>
       <c r="F223" s="5" t="s">
         <v>99</v>
@@ -6840,10 +6858,10 @@
         <v>407</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>410</v>
+        <v>454</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>412</v>
+        <v>455</v>
       </c>
       <c r="F224" s="5" t="s">
         <v>99</v>
@@ -6854,10 +6872,10 @@
         <v>407</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>456</v>
+        <v>410</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>457</v>
+        <v>412</v>
       </c>
       <c r="F225" s="5" t="s">
         <v>99</v>
@@ -6868,106 +6886,106 @@
         <v>407</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>528</v>
+        <v>456</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>529</v>
-      </c>
-      <c r="F226" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="227" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>457</v>
+      </c>
+      <c r="F226" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A227" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>413</v>
+        <v>528</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="F227" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G227" s="2" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="228" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>529</v>
+      </c>
+      <c r="F227" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B228" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F228" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G228" s="2" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A229" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B229" s="2" t="s">
         <v>556</v>
       </c>
-      <c r="C228" s="2" t="s">
+      <c r="C229" s="2" t="s">
         <v>557</v>
       </c>
-      <c r="F228" s="19" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="229" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A229" s="17" t="s">
-        <v>407</v>
-      </c>
-      <c r="B229" s="17" t="s">
-        <v>478</v>
-      </c>
-      <c r="C229" s="17" t="s">
-        <v>479</v>
-      </c>
-      <c r="D229" s="17"/>
-      <c r="E229" s="17"/>
       <c r="F229" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="G229" s="17"/>
-    </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A230" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B230" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="C230" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="F230" s="5" t="s">
-        <v>99</v>
-      </c>
+    </row>
+    <row r="230" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A230" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="B230" s="17" t="s">
+        <v>478</v>
+      </c>
+      <c r="C230" s="17" t="s">
+        <v>479</v>
+      </c>
+      <c r="D230" s="17"/>
+      <c r="E230" s="17"/>
+      <c r="F230" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="G230" s="17"/>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A231" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>292</v>
+        <v>203</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="E231" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F231" s="12" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="232" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>204</v>
+      </c>
+      <c r="F231" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A232" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>205</v>
+        <v>292</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="F232" s="5" t="s">
-        <v>99</v>
+        <v>293</v>
+      </c>
+      <c r="E232" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F232" s="12" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="233" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6975,30 +6993,30 @@
         <v>91</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="F233" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G233" s="2" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
+        <v>206</v>
+      </c>
+      <c r="F233" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A234" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="F234" s="5" t="s">
-        <v>99</v>
+        <v>208</v>
+      </c>
+      <c r="F234" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G234" s="2" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.35">
@@ -7006,10 +7024,10 @@
         <v>91</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>92</v>
+        <v>209</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>95</v>
+        <v>214</v>
       </c>
       <c r="F235" s="5" t="s">
         <v>99</v>
@@ -7020,128 +7038,128 @@
         <v>91</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>210</v>
+        <v>92</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="F236" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="237" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+      <c r="F236" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A237" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B237" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C237" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F237" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A238" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B238" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="C237" s="2" t="s">
+      <c r="C238" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="F237" s="12" t="s">
+      <c r="F238" s="12" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="238" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A238" s="17" t="s">
+    <row r="239" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A239" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="B238" s="17" t="s">
+      <c r="B239" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="C238" s="17" t="s">
+      <c r="C239" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D238" s="17"/>
-      <c r="E238" s="17"/>
-      <c r="F238" s="20" t="s">
+      <c r="D239" s="17"/>
+      <c r="E239" s="17"/>
+      <c r="F239" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="G238" s="17"/>
-    </row>
-    <row r="239" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A239" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B239" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C239" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F239" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G239" s="2" t="s">
-        <v>319</v>
-      </c>
+      <c r="G239" s="17"/>
     </row>
     <row r="240" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A240" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>190</v>
+        <v>69</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>192</v>
+        <v>70</v>
       </c>
       <c r="F240" s="6" t="s">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="G240" s="2" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.35">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A241" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>731</v>
+        <v>190</v>
       </c>
       <c r="C241" s="2" t="s">
-        <v>732</v>
+        <v>192</v>
       </c>
       <c r="F241" s="6" t="s">
         <v>140</v>
       </c>
       <c r="G241" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A242" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B242" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="C242" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="F242" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G242" s="2" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="242" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A242" s="17" t="s">
+    <row r="243" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A243" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="B242" s="17" t="s">
+      <c r="B243" s="17" t="s">
         <v>191</v>
       </c>
-      <c r="C242" s="17" t="s">
+      <c r="C243" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="D242" s="17"/>
-      <c r="E242" s="17"/>
-      <c r="F242" s="22" t="s">
+      <c r="D243" s="17"/>
+      <c r="E243" s="17"/>
+      <c r="F243" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="G242" s="17" t="s">
+      <c r="G243" s="17" t="s">
         <v>324</v>
-      </c>
-    </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A243" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B243" s="2" t="s">
-        <v>619</v>
-      </c>
-      <c r="C243" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="F243" s="4" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.35">
@@ -7149,13 +7167,13 @@
         <v>71</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>537</v>
+        <v>619</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>538</v>
-      </c>
-      <c r="F244" s="5" t="s">
-        <v>99</v>
+        <v>620</v>
+      </c>
+      <c r="F244" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="245" spans="1:7" x14ac:dyDescent="0.35">
@@ -7163,13 +7181,13 @@
         <v>71</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>72</v>
+        <v>537</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F245" s="4" t="s">
-        <v>98</v>
+        <v>538</v>
+      </c>
+      <c r="F245" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="246" spans="1:7" x14ac:dyDescent="0.35">
@@ -7177,41 +7195,41 @@
         <v>71</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="F246" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="247" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+      <c r="F246" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A247" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>541</v>
+        <v>73</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>542</v>
+        <v>81</v>
       </c>
       <c r="F247" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A248" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>398</v>
+        <v>541</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="F248" s="4" t="s">
-        <v>98</v>
+        <v>542</v>
+      </c>
+      <c r="F248" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="249" spans="1:7" x14ac:dyDescent="0.35">
@@ -7219,10 +7237,10 @@
         <v>71</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>663</v>
+        <v>398</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>664</v>
+        <v>399</v>
       </c>
       <c r="F249" s="4" t="s">
         <v>98</v>
@@ -7233,13 +7251,13 @@
         <v>71</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>539</v>
+        <v>663</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>540</v>
-      </c>
-      <c r="F250" s="5" t="s">
-        <v>99</v>
+        <v>664</v>
+      </c>
+      <c r="F250" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="251" spans="1:7" x14ac:dyDescent="0.35">
@@ -7247,13 +7265,13 @@
         <v>71</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>271</v>
+        <v>539</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="F251" s="3" t="s">
-        <v>97</v>
+        <v>540</v>
+      </c>
+      <c r="F251" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.35">
@@ -7261,44 +7279,44 @@
         <v>71</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>250</v>
+        <v>271</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="F252" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="253" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A253" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E253" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="F253" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.35">
+        <v>251</v>
+      </c>
+      <c r="F253" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A254" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>790</v>
+        <v>230</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>791</v>
-      </c>
-      <c r="F254" s="3" t="s">
-        <v>97</v>
+        <v>231</v>
+      </c>
+      <c r="E254" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="F254" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.35">
@@ -7306,13 +7324,13 @@
         <v>71</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>605</v>
+        <v>790</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="F255" s="5" t="s">
-        <v>99</v>
+        <v>791</v>
+      </c>
+      <c r="F255" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="256" spans="1:7" x14ac:dyDescent="0.35">
@@ -7320,10 +7338,10 @@
         <v>71</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="F256" s="5" t="s">
         <v>99</v>
@@ -7334,10 +7352,10 @@
         <v>71</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>226</v>
+        <v>607</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>227</v>
+        <v>608</v>
       </c>
       <c r="F257" s="5" t="s">
         <v>99</v>
@@ -7348,10 +7366,10 @@
         <v>71</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="F258" s="5" t="s">
         <v>99</v>
@@ -7362,13 +7380,10 @@
         <v>71</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>621</v>
+        <v>222</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="D259" s="2" t="s">
-        <v>623</v>
+        <v>223</v>
       </c>
       <c r="F259" s="5" t="s">
         <v>99</v>
@@ -7379,10 +7394,13 @@
         <v>71</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>609</v>
+        <v>621</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>610</v>
+        <v>622</v>
+      </c>
+      <c r="D260" s="2" t="s">
+        <v>623</v>
       </c>
       <c r="F260" s="5" t="s">
         <v>99</v>
@@ -7393,13 +7411,13 @@
         <v>71</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>694</v>
+        <v>609</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>695</v>
-      </c>
-      <c r="F261" s="3" t="s">
-        <v>97</v>
+        <v>610</v>
+      </c>
+      <c r="F261" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.35">
@@ -7407,10 +7425,10 @@
         <v>71</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>624</v>
+        <v>694</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>625</v>
+        <v>695</v>
       </c>
       <c r="F262" s="3" t="s">
         <v>97</v>
@@ -7421,10 +7439,10 @@
         <v>71</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>596</v>
+        <v>624</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>597</v>
+        <v>625</v>
       </c>
       <c r="F263" s="3" t="s">
         <v>97</v>
@@ -7435,13 +7453,13 @@
         <v>71</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>576</v>
+        <v>596</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>577</v>
-      </c>
-      <c r="F264" s="4" t="s">
-        <v>98</v>
+        <v>597</v>
+      </c>
+      <c r="F264" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.35">
@@ -7449,44 +7467,44 @@
         <v>71</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>235</v>
+        <v>576</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>236</v>
+        <v>577</v>
       </c>
       <c r="F265" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="266" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A266" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>273</v>
+        <v>235</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="F266" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="G266" s="2" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
+        <v>236</v>
+      </c>
+      <c r="F266" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A267" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>74</v>
+        <v>273</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F267" s="5" t="s">
-        <v>99</v>
+        <v>274</v>
+      </c>
+      <c r="F267" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G267" s="2" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.35">
@@ -7494,10 +7512,10 @@
         <v>71</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F268" s="5" t="s">
         <v>99</v>
@@ -7508,10 +7526,10 @@
         <v>71</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F269" s="5" t="s">
         <v>99</v>
@@ -7522,13 +7540,13 @@
         <v>71</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F270" s="4" t="s">
-        <v>98</v>
+        <v>84</v>
+      </c>
+      <c r="F270" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="271" spans="1:7" x14ac:dyDescent="0.35">
@@ -7536,16 +7554,13 @@
         <v>71</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>611</v>
+        <v>77</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>612</v>
-      </c>
-      <c r="D271" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="F271" s="5" t="s">
-        <v>99</v>
+        <v>85</v>
+      </c>
+      <c r="F271" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="272" spans="1:7" x14ac:dyDescent="0.35">
@@ -7553,13 +7568,16 @@
         <v>71</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>435</v>
+        <v>611</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="F272" s="4" t="s">
-        <v>98</v>
+        <v>612</v>
+      </c>
+      <c r="D272" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="F272" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.35">
@@ -7567,41 +7585,41 @@
         <v>71</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>465</v>
+        <v>435</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>466</v>
+        <v>436</v>
       </c>
       <c r="F273" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="274" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A274" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>626</v>
+        <v>465</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="F274" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
+        <v>466</v>
+      </c>
+      <c r="F274" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A275" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>725</v>
+        <v>626</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>726</v>
-      </c>
-      <c r="F275" s="3" t="s">
-        <v>97</v>
+        <v>627</v>
+      </c>
+      <c r="F275" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="276" spans="1:7" x14ac:dyDescent="0.35">
@@ -7609,10 +7627,10 @@
         <v>71</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>78</v>
+        <v>725</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>86</v>
+        <v>726</v>
       </c>
       <c r="F276" s="3" t="s">
         <v>97</v>
@@ -7623,30 +7641,27 @@
         <v>71</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>535</v>
+        <v>78</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="F277" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="278" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+      <c r="F277" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A278" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>281</v>
+        <v>535</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="F278" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G278" s="2" t="s">
-        <v>323</v>
+        <v>536</v>
+      </c>
+      <c r="F278" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="279" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -7654,10 +7669,10 @@
         <v>71</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="F279" s="16" t="s">
         <v>291</v>
@@ -7671,10 +7686,10 @@
         <v>71</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>233</v>
+        <v>283</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>234</v>
+        <v>284</v>
       </c>
       <c r="F280" s="16" t="s">
         <v>291</v>
@@ -7683,35 +7698,38 @@
         <v>323</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A281" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E281" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="F281" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="282" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+      <c r="F281" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G281" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A282" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>677</v>
+        <v>224</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="F282" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
+      </c>
+      <c r="E282" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F282" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="283" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7719,58 +7737,58 @@
         <v>71</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>79</v>
+        <v>677</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F283" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.35">
+        <v>678</v>
+      </c>
+      <c r="F283" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A284" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>729</v>
+        <v>79</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>730</v>
+        <v>87</v>
       </c>
       <c r="F284" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="285" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A285" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>430</v>
+        <v>729</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="F285" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G285" s="2" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.35">
+        <v>730</v>
+      </c>
+      <c r="F285" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A286" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>628</v>
+        <v>430</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>629</v>
-      </c>
-      <c r="F286" s="5" t="s">
-        <v>99</v>
+        <v>431</v>
+      </c>
+      <c r="F286" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G286" s="2" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.35">
@@ -7778,44 +7796,44 @@
         <v>71</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>494</v>
+        <v>628</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>495</v>
+        <v>629</v>
       </c>
       <c r="F287" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="288" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A288" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>762</v>
+        <v>494</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>763</v>
-      </c>
-      <c r="F288" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G288" s="2" t="s">
-        <v>764</v>
-      </c>
-    </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.35">
+        <v>495</v>
+      </c>
+      <c r="F288" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A289" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>239</v>
+        <v>762</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="F289" s="14" t="s">
-        <v>252</v>
+        <v>763</v>
+      </c>
+      <c r="F289" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G289" s="2" t="s">
+        <v>764</v>
       </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.35">
@@ -7823,13 +7841,13 @@
         <v>71</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>286</v>
+        <v>239</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="F290" s="5" t="s">
-        <v>99</v>
+        <v>240</v>
+      </c>
+      <c r="F290" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.35">
@@ -7837,13 +7855,13 @@
         <v>71</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>630</v>
+        <v>286</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>631</v>
-      </c>
-      <c r="F291" s="4" t="s">
-        <v>98</v>
+        <v>285</v>
+      </c>
+      <c r="F291" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.35">
@@ -7851,13 +7869,13 @@
         <v>71</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>228</v>
+        <v>630</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="F292" s="5" t="s">
-        <v>99</v>
+        <v>631</v>
+      </c>
+      <c r="F292" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.35">
@@ -7865,10 +7883,10 @@
         <v>71</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>614</v>
+        <v>228</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>615</v>
+        <v>229</v>
       </c>
       <c r="F293" s="5" t="s">
         <v>99</v>
@@ -7879,13 +7897,13 @@
         <v>71</v>
       </c>
       <c r="B294" s="2" t="s">
-        <v>220</v>
+        <v>614</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F294" s="12" t="s">
-        <v>244</v>
+        <v>615</v>
+      </c>
+      <c r="F294" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="295" spans="1:7" x14ac:dyDescent="0.35">
@@ -7893,13 +7911,13 @@
         <v>71</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>511</v>
+        <v>220</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="F295" s="14" t="s">
-        <v>252</v>
+        <v>221</v>
+      </c>
+      <c r="F295" s="12" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="296" spans="1:7" x14ac:dyDescent="0.35">
@@ -7907,16 +7925,13 @@
         <v>71</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>510</v>
-      </c>
-      <c r="E296" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="F296" s="5" t="s">
-        <v>99</v>
+        <v>512</v>
+      </c>
+      <c r="F296" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="297" spans="1:7" x14ac:dyDescent="0.35">
@@ -7924,44 +7939,44 @@
         <v>71</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>218</v>
+        <v>509</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>219</v>
+        <v>510</v>
+      </c>
+      <c r="E297" s="2" t="s">
+        <v>220</v>
       </c>
       <c r="F297" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="298" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A298" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>632</v>
+        <v>218</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>633</v>
-      </c>
-      <c r="F298" s="20" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="299" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>219</v>
+      </c>
+      <c r="F298" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A299" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>571</v>
+        <v>632</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>573</v>
-      </c>
-      <c r="F299" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="G299" s="2" t="s">
-        <v>574</v>
+        <v>633</v>
+      </c>
+      <c r="F299" s="20" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="300" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7969,81 +7984,81 @@
         <v>71</v>
       </c>
       <c r="B300" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="C300" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="F300" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G300" s="2" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A301" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B301" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="C300" s="2" t="s">
+      <c r="C301" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="F300" s="16" t="s">
+      <c r="F301" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G300" s="2" t="s">
+      <c r="G301" s="2" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="301" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A301" s="17" t="s">
+    <row r="302" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A302" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B301" s="17" t="s">
+      <c r="B302" s="17" t="s">
         <v>294</v>
       </c>
-      <c r="C301" s="17" t="s">
+      <c r="C302" s="17" t="s">
         <v>295</v>
       </c>
-      <c r="D301" s="17"/>
-      <c r="E301" s="17"/>
-      <c r="F301" s="20" t="s">
+      <c r="D302" s="17"/>
+      <c r="E302" s="17"/>
+      <c r="F302" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="G301" s="17"/>
-    </row>
-    <row r="302" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A302" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B302" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C302" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D302" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="F302" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G302" s="17"/>
+    </row>
+    <row r="303" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A303" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>216</v>
+        <v>89</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>215</v>
+        <v>90</v>
       </c>
       <c r="D303" s="2" t="s">
-        <v>390</v>
+        <v>303</v>
       </c>
       <c r="F303" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="304" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A304" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>242</v>
+        <v>215</v>
       </c>
       <c r="D304" s="2" t="s">
-        <v>243</v>
+        <v>390</v>
       </c>
       <c r="F304" s="5" t="s">
         <v>99</v>
@@ -8054,27 +8069,30 @@
         <v>88</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>792</v>
+        <v>241</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>793</v>
-      </c>
-      <c r="F305" s="25" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+      <c r="D305" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F305" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="306" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A306" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>338</v>
+        <v>792</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="F306" s="4" t="s">
-        <v>98</v>
+        <v>793</v>
+      </c>
+      <c r="F306" s="25" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="307" spans="1:7" x14ac:dyDescent="0.35">
@@ -8082,36 +8100,50 @@
         <v>88</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>551</v>
+        <v>338</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="D307" s="2" t="s">
-        <v>553</v>
+        <v>339</v>
       </c>
       <c r="F307" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="308" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A308" s="17" t="s">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A308" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B308" s="17" t="s">
+      <c r="B308" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="C308" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="D308" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="F308" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="309" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A309" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B309" s="17" t="s">
         <v>279</v>
       </c>
-      <c r="C308" s="17" t="s">
+      <c r="C309" s="17" t="s">
         <v>280</v>
       </c>
-      <c r="D308" s="17" t="s">
+      <c r="D309" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="E308" s="17"/>
-      <c r="F308" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="G308" s="17"/>
+      <c r="E309" s="17"/>
+      <c r="F309" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="G309" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Integrate 4.0.4: commit #71ad922, 1/28/25, Modify ZEV levers to split options for federal and subnational ZEV requirements
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B01FBE4-3B6E-4E45-A6AB-63D6C15D47FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{693EE7FF-73B1-464B-8372-BD3A2CB5CA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1466" uniqueCount="848">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1470" uniqueCount="850">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2576,6 +2576,12 @@
   </si>
   <si>
     <t>You want to test the addition rather than the reduction of process emissions for select industries</t>
+  </si>
+  <si>
+    <t>BRZSPbMR</t>
+  </si>
+  <si>
+    <t>BAU Required ZEV Sales Perc by Model Region</t>
   </si>
 </sst>
 </file>
@@ -3387,7 +3393,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G309"/>
+  <dimension ref="A1:G310"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
@@ -7425,10 +7431,10 @@
         <v>71</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>694</v>
+        <v>848</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>695</v>
+        <v>849</v>
       </c>
       <c r="F262" s="3" t="s">
         <v>97</v>
@@ -7439,10 +7445,10 @@
         <v>71</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>624</v>
+        <v>694</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>625</v>
+        <v>695</v>
       </c>
       <c r="F263" s="3" t="s">
         <v>97</v>
@@ -7453,10 +7459,10 @@
         <v>71</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>596</v>
+        <v>624</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>597</v>
+        <v>625</v>
       </c>
       <c r="F264" s="3" t="s">
         <v>97</v>
@@ -7467,13 +7473,13 @@
         <v>71</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>576</v>
+        <v>596</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>577</v>
-      </c>
-      <c r="F265" s="4" t="s">
-        <v>98</v>
+        <v>597</v>
+      </c>
+      <c r="F265" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.35">
@@ -7481,44 +7487,44 @@
         <v>71</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>235</v>
+        <v>576</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>236</v>
+        <v>577</v>
       </c>
       <c r="F266" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="267" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A267" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>273</v>
+        <v>235</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="F267" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="G267" s="2" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
+        <v>236</v>
+      </c>
+      <c r="F267" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A268" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>74</v>
+        <v>273</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F268" s="5" t="s">
-        <v>99</v>
+        <v>274</v>
+      </c>
+      <c r="F268" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G268" s="2" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.35">
@@ -7526,10 +7532,10 @@
         <v>71</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F269" s="5" t="s">
         <v>99</v>
@@ -7540,10 +7546,10 @@
         <v>71</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F270" s="5" t="s">
         <v>99</v>
@@ -7554,13 +7560,13 @@
         <v>71</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F271" s="4" t="s">
-        <v>98</v>
+        <v>84</v>
+      </c>
+      <c r="F271" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="272" spans="1:7" x14ac:dyDescent="0.35">
@@ -7568,16 +7574,13 @@
         <v>71</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>611</v>
+        <v>77</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>612</v>
-      </c>
-      <c r="D272" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="F272" s="5" t="s">
-        <v>99</v>
+        <v>85</v>
+      </c>
+      <c r="F272" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.35">
@@ -7585,13 +7588,16 @@
         <v>71</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>435</v>
+        <v>611</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="F273" s="4" t="s">
-        <v>98</v>
+        <v>612</v>
+      </c>
+      <c r="D273" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="F273" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="274" spans="1:7" x14ac:dyDescent="0.35">
@@ -7599,41 +7605,41 @@
         <v>71</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>465</v>
+        <v>435</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>466</v>
+        <v>436</v>
       </c>
       <c r="F274" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="275" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A275" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>626</v>
+        <v>465</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="F275" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.35">
+        <v>466</v>
+      </c>
+      <c r="F275" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="276" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A276" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>725</v>
+        <v>626</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>726</v>
-      </c>
-      <c r="F276" s="3" t="s">
-        <v>97</v>
+        <v>627</v>
+      </c>
+      <c r="F276" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.35">
@@ -7641,10 +7647,10 @@
         <v>71</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>78</v>
+        <v>725</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>86</v>
+        <v>726</v>
       </c>
       <c r="F277" s="3" t="s">
         <v>97</v>
@@ -7655,30 +7661,27 @@
         <v>71</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>535</v>
+        <v>78</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="F278" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="279" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+      <c r="F278" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A279" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>281</v>
+        <v>535</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="F279" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G279" s="2" t="s">
-        <v>323</v>
+        <v>536</v>
+      </c>
+      <c r="F279" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="280" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -7686,10 +7689,10 @@
         <v>71</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="F280" s="16" t="s">
         <v>291</v>
@@ -7703,10 +7706,10 @@
         <v>71</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>233</v>
+        <v>283</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>234</v>
+        <v>284</v>
       </c>
       <c r="F281" s="16" t="s">
         <v>291</v>
@@ -7715,35 +7718,38 @@
         <v>323</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A282" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E282" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="F282" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="283" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+      <c r="F282" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G282" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A283" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>677</v>
+        <v>224</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="F283" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
+      </c>
+      <c r="E283" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F283" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="284" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7751,58 +7757,58 @@
         <v>71</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>79</v>
+        <v>677</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F284" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
+        <v>678</v>
+      </c>
+      <c r="F284" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="285" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A285" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>729</v>
+        <v>79</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>730</v>
+        <v>87</v>
       </c>
       <c r="F285" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="286" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A286" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>430</v>
+        <v>729</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="F286" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G286" s="2" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.35">
+        <v>730</v>
+      </c>
+      <c r="F286" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A287" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>628</v>
+        <v>430</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>629</v>
-      </c>
-      <c r="F287" s="5" t="s">
-        <v>99</v>
+        <v>431</v>
+      </c>
+      <c r="F287" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G287" s="2" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.35">
@@ -7810,44 +7816,44 @@
         <v>71</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>494</v>
+        <v>628</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>495</v>
+        <v>629</v>
       </c>
       <c r="F288" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="289" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A289" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>762</v>
+        <v>494</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>763</v>
-      </c>
-      <c r="F289" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G289" s="2" t="s">
-        <v>764</v>
-      </c>
-    </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.35">
+        <v>495</v>
+      </c>
+      <c r="F289" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A290" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>239</v>
+        <v>762</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="F290" s="14" t="s">
-        <v>252</v>
+        <v>763</v>
+      </c>
+      <c r="F290" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G290" s="2" t="s">
+        <v>764</v>
       </c>
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.35">
@@ -7855,13 +7861,13 @@
         <v>71</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>286</v>
+        <v>239</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="F291" s="5" t="s">
-        <v>99</v>
+        <v>240</v>
+      </c>
+      <c r="F291" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.35">
@@ -7869,13 +7875,13 @@
         <v>71</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>630</v>
+        <v>286</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>631</v>
-      </c>
-      <c r="F292" s="4" t="s">
-        <v>98</v>
+        <v>285</v>
+      </c>
+      <c r="F292" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.35">
@@ -7883,13 +7889,13 @@
         <v>71</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>228</v>
+        <v>630</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="F293" s="5" t="s">
-        <v>99</v>
+        <v>631</v>
+      </c>
+      <c r="F293" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="294" spans="1:7" x14ac:dyDescent="0.35">
@@ -7897,10 +7903,10 @@
         <v>71</v>
       </c>
       <c r="B294" s="2" t="s">
-        <v>614</v>
+        <v>228</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>615</v>
+        <v>229</v>
       </c>
       <c r="F294" s="5" t="s">
         <v>99</v>
@@ -7911,13 +7917,13 @@
         <v>71</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>220</v>
+        <v>614</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F295" s="12" t="s">
-        <v>244</v>
+        <v>615</v>
+      </c>
+      <c r="F295" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="296" spans="1:7" x14ac:dyDescent="0.35">
@@ -7925,13 +7931,13 @@
         <v>71</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>511</v>
+        <v>220</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="F296" s="14" t="s">
-        <v>252</v>
+        <v>221</v>
+      </c>
+      <c r="F296" s="12" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="297" spans="1:7" x14ac:dyDescent="0.35">
@@ -7939,16 +7945,13 @@
         <v>71</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>510</v>
-      </c>
-      <c r="E297" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="F297" s="5" t="s">
-        <v>99</v>
+        <v>512</v>
+      </c>
+      <c r="F297" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="298" spans="1:7" x14ac:dyDescent="0.35">
@@ -7956,44 +7959,44 @@
         <v>71</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>218</v>
+        <v>509</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>219</v>
+        <v>510</v>
+      </c>
+      <c r="E298" s="2" t="s">
+        <v>220</v>
       </c>
       <c r="F298" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="299" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="299" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A299" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>632</v>
+        <v>218</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>633</v>
-      </c>
-      <c r="F299" s="20" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="300" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>219</v>
+      </c>
+      <c r="F299" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A300" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>571</v>
+        <v>632</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>573</v>
-      </c>
-      <c r="F300" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="G300" s="2" t="s">
-        <v>574</v>
+        <v>633</v>
+      </c>
+      <c r="F300" s="20" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="301" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -8001,81 +8004,81 @@
         <v>71</v>
       </c>
       <c r="B301" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="C301" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="F301" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G301" s="2" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="302" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A302" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B302" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="C301" s="2" t="s">
+      <c r="C302" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="F301" s="16" t="s">
+      <c r="F302" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G301" s="2" t="s">
+      <c r="G302" s="2" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="302" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A302" s="17" t="s">
+    <row r="303" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A303" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B302" s="17" t="s">
+      <c r="B303" s="17" t="s">
         <v>294</v>
       </c>
-      <c r="C302" s="17" t="s">
+      <c r="C303" s="17" t="s">
         <v>295</v>
       </c>
-      <c r="D302" s="17"/>
-      <c r="E302" s="17"/>
-      <c r="F302" s="20" t="s">
+      <c r="D303" s="17"/>
+      <c r="E303" s="17"/>
+      <c r="F303" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="G302" s="17"/>
-    </row>
-    <row r="303" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A303" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B303" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C303" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D303" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="F303" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G303" s="17"/>
+    </row>
+    <row r="304" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A304" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>216</v>
+        <v>89</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>215</v>
+        <v>90</v>
       </c>
       <c r="D304" s="2" t="s">
-        <v>390</v>
+        <v>303</v>
       </c>
       <c r="F304" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="305" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A305" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>242</v>
+        <v>215</v>
       </c>
       <c r="D305" s="2" t="s">
-        <v>243</v>
+        <v>390</v>
       </c>
       <c r="F305" s="5" t="s">
         <v>99</v>
@@ -8086,27 +8089,30 @@
         <v>88</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>792</v>
+        <v>241</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>793</v>
-      </c>
-      <c r="F306" s="25" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+      <c r="D306" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F306" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="307" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A307" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>338</v>
+        <v>792</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="F307" s="4" t="s">
-        <v>98</v>
+        <v>793</v>
+      </c>
+      <c r="F307" s="25" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="308" spans="1:7" x14ac:dyDescent="0.35">
@@ -8114,36 +8120,50 @@
         <v>88</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>551</v>
+        <v>338</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="D308" s="2" t="s">
-        <v>553</v>
+        <v>339</v>
       </c>
       <c r="F308" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="309" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A309" s="17" t="s">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A309" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B309" s="17" t="s">
+      <c r="B309" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="C309" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="D309" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="F309" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="310" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A310" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B310" s="17" t="s">
         <v>279</v>
       </c>
-      <c r="C309" s="17" t="s">
+      <c r="C310" s="17" t="s">
         <v>280</v>
       </c>
-      <c r="D309" s="17" t="s">
+      <c r="D310" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="E309" s="17"/>
-      <c r="F309" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="G309" s="17"/>
+      <c r="E310" s="17"/>
+      <c r="F310" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="G310" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Integrate 4.0.4: commit #7f7e6df, 2/14/25, Adds 45X for grid batteries; adjusts 45X implementation in transport sector
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AA14AFB-0DA1-476E-B275-10CEAF1CFFF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{606D8603-F01D-4DB3-99F3-85E8BA982B2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29595" yWindow="3060" windowWidth="26655" windowHeight="13965" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="59235" yWindow="3345" windowWidth="21900" windowHeight="12420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1470" uniqueCount="850">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="854">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2582,6 +2582,18 @@
   </si>
   <si>
     <t>Time Adjusted Capacity Factor Multiplier for Plants Built This Year</t>
+  </si>
+  <si>
+    <t>BSfGBP</t>
+  </si>
+  <si>
+    <t>BAU Subsidy for Grid Battery Production</t>
+  </si>
+  <si>
+    <t>FoGBPD</t>
+  </si>
+  <si>
+    <t>Fraction of Grid Batteries Produced Domestically</t>
   </si>
 </sst>
 </file>
@@ -3393,7 +3405,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G310"/>
+  <dimension ref="A1:G312"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
@@ -4734,29 +4746,29 @@
         <v>97</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>671</v>
+        <v>850</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>672</v>
+        <v>851</v>
       </c>
       <c r="F85" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>158</v>
+        <v>671</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>159</v>
+        <v>672</v>
       </c>
       <c r="F86" s="3" t="s">
         <v>97</v>
@@ -4767,120 +4779,120 @@
         <v>43</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>642</v>
+        <v>158</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="F87" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>46</v>
+        <v>642</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>709</v>
+        <v>643</v>
       </c>
       <c r="F88" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="89" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>710</v>
+        <v>46</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>711</v>
+        <v>52</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>709</v>
       </c>
       <c r="F89" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="90" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>498</v>
+        <v>710</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="F90" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G90" s="2" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+        <v>711</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>774</v>
+        <v>498</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>775</v>
-      </c>
-      <c r="F91" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+        <v>499</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>712</v>
+        <v>774</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>746</v>
+        <v>775</v>
       </c>
       <c r="F92" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>632</v>
+        <v>712</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>633</v>
+        <v>713</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>746</v>
       </c>
       <c r="F93" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>297</v>
+        <v>632</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="F94" s="4" t="s">
-        <v>98</v>
+        <v>633</v>
+      </c>
+      <c r="F94" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.35">
@@ -4888,64 +4900,61 @@
         <v>43</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>725</v>
+        <v>297</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>726</v>
+        <v>298</v>
       </c>
       <c r="F95" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>47</v>
+        <v>725</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>687</v>
-      </c>
-      <c r="F96" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+        <v>726</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>276</v>
+        <v>47</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>277</v>
+        <v>169</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="F97" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>687</v>
+      </c>
+      <c r="F97" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>644</v>
+        <v>276</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>645</v>
+        <v>277</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>714</v>
-      </c>
-      <c r="F98" s="5" t="s">
-        <v>99</v>
+        <v>278</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -4953,33 +4962,33 @@
         <v>43</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>167</v>
+        <v>644</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>168</v>
+        <v>645</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="F99" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+        <v>714</v>
+      </c>
+      <c r="F99" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>655</v>
+        <v>167</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>656</v>
+        <v>168</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>657</v>
-      </c>
-      <c r="F100" s="4" t="s">
-        <v>98</v>
+        <v>434</v>
+      </c>
+      <c r="F100" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.35">
@@ -4987,13 +4996,16 @@
         <v>43</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>776</v>
+        <v>655</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>777</v>
-      </c>
-      <c r="F101" s="5" t="s">
-        <v>99</v>
+        <v>656</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.35">
@@ -5001,10 +5013,10 @@
         <v>43</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>715</v>
+        <v>776</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>716</v>
+        <v>777</v>
       </c>
       <c r="F102" s="5" t="s">
         <v>99</v>
@@ -5015,33 +5027,27 @@
         <v>43</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>476</v>
+        <v>852</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>688</v>
+        <v>853</v>
       </c>
       <c r="F103" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>175</v>
+        <v>715</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="F104" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G104" s="2" t="s">
-        <v>309</v>
+        <v>716</v>
+      </c>
+      <c r="F104" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.35">
@@ -5049,52 +5055,58 @@
         <v>43</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>750</v>
+        <v>476</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>752</v>
-      </c>
-      <c r="F105" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+        <v>477</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A106" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="B106" s="2" t="s">
-        <v>751</v>
+        <v>175</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>753</v>
-      </c>
-      <c r="F106" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>174</v>
+      </c>
+      <c r="F106" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G106" s="2" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>697</v>
+        <v>750</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="F107" s="4" t="s">
-        <v>98</v>
+        <v>752</v>
+      </c>
+      <c r="F107" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A108" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="B108" s="2" t="s">
-        <v>717</v>
+        <v>751</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>718</v>
-      </c>
-      <c r="F108" s="4" t="s">
-        <v>98</v>
+        <v>753</v>
+      </c>
+      <c r="F108" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5102,10 +5114,10 @@
         <v>43</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>577</v>
+        <v>697</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>578</v>
+        <v>698</v>
       </c>
       <c r="F109" s="4" t="s">
         <v>98</v>
@@ -5116,27 +5128,27 @@
         <v>43</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>590</v>
+        <v>717</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="F110" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+        <v>718</v>
+      </c>
+      <c r="F110" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>734</v>
+        <v>577</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>735</v>
-      </c>
-      <c r="F111" s="3" t="s">
-        <v>97</v>
+        <v>578</v>
+      </c>
+      <c r="F111" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.35">
@@ -5144,13 +5156,13 @@
         <v>43</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>581</v>
+        <v>590</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>582</v>
-      </c>
-      <c r="F112" s="4" t="s">
-        <v>98</v>
+        <v>591</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.35">
@@ -5158,13 +5170,13 @@
         <v>43</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>646</v>
+        <v>734</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>647</v>
-      </c>
-      <c r="F113" s="4" t="s">
-        <v>98</v>
+        <v>735</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.35">
@@ -5172,13 +5184,13 @@
         <v>43</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>48</v>
+        <v>581</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F114" s="3" t="s">
-        <v>97</v>
+        <v>582</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.35">
@@ -5186,95 +5198,92 @@
         <v>43</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>194</v>
+        <v>646</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>202</v>
+        <v>647</v>
       </c>
       <c r="F115" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F116" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G116" s="2" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>739</v>
+        <v>194</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>740</v>
-      </c>
-      <c r="F117" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G117" s="2" t="s">
-        <v>741</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>202</v>
+      </c>
+      <c r="F117" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>732</v>
+        <v>49</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>733</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>747</v>
-      </c>
-      <c r="F118" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+      <c r="F118" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>653</v>
+        <v>739</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>654</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>719</v>
-      </c>
-      <c r="F119" s="14" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+        <v>740</v>
+      </c>
+      <c r="F119" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>184</v>
+        <v>732</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F120" s="4" t="s">
-        <v>98</v>
+        <v>733</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="F120" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="121" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5282,30 +5291,30 @@
         <v>43</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>564</v>
+        <v>653</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>565</v>
-      </c>
-      <c r="F121" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="122" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>654</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>719</v>
+      </c>
+      <c r="F121" s="14" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F122" s="5" t="s">
-        <v>326</v>
+        <v>185</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5313,86 +5322,89 @@
         <v>43</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>665</v>
+        <v>564</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="D123" s="2" t="s">
-        <v>667</v>
-      </c>
-      <c r="F123" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+        <v>565</v>
+      </c>
+      <c r="F123" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>585</v>
+        <v>199</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>586</v>
+        <v>200</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>589</v>
-      </c>
-      <c r="F124" s="3" t="s">
-        <v>97</v>
+        <v>201</v>
+      </c>
+      <c r="F124" s="5" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A125" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="B125" s="2" t="s">
-        <v>651</v>
+        <v>665</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>652</v>
-      </c>
-      <c r="F125" s="14" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>666</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="F125" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>439</v>
+        <v>585</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>440</v>
+        <v>586</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="F126" s="4" t="s">
-        <v>98</v>
+        <v>589</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A127" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="B127" s="2" t="s">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>664</v>
+        <v>652</v>
       </c>
       <c r="F127" s="14" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>636</v>
+        <v>439</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>637</v>
+        <v>440</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>441</v>
       </c>
       <c r="F128" s="4" t="s">
         <v>98</v>
@@ -5403,13 +5415,13 @@
         <v>43</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>638</v>
+        <v>663</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="F129" s="4" t="s">
-        <v>98</v>
+        <v>664</v>
+      </c>
+      <c r="F129" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5417,75 +5429,72 @@
         <v>43</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>559</v>
+        <v>636</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>560</v>
+        <v>637</v>
       </c>
       <c r="F130" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="F131" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+        <v>639</v>
+      </c>
+      <c r="F131" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>583</v>
+        <v>559</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="E132" s="2" t="s">
-        <v>581</v>
-      </c>
-      <c r="F132" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>560</v>
+      </c>
+      <c r="F132" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>720</v>
+        <v>634</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>721</v>
-      </c>
-      <c r="D133" s="2" t="s">
-        <v>722</v>
+        <v>635</v>
       </c>
       <c r="F133" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>848</v>
+        <v>583</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>849</v>
-      </c>
-      <c r="F134" s="4" t="s">
-        <v>98</v>
+        <v>584</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5493,68 +5502,65 @@
         <v>43</v>
       </c>
       <c r="B135" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>721</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="F135" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A136" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>848</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>849</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A137" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B137" s="2" t="s">
         <v>690</v>
       </c>
-      <c r="C135" s="2" t="s">
+      <c r="C137" s="2" t="s">
         <v>691</v>
       </c>
-      <c r="F135" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A136" s="17" t="s">
+      <c r="F137" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A138" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="B136" s="17" t="s">
+      <c r="B138" s="17" t="s">
         <v>334</v>
       </c>
-      <c r="C136" s="17" t="s">
+      <c r="C138" s="17" t="s">
         <v>335</v>
       </c>
-      <c r="D136" s="17" t="s">
+      <c r="D138" s="17" t="s">
         <v>336</v>
       </c>
-      <c r="E136" s="17"/>
-      <c r="F136" s="21" t="s">
+      <c r="E138" s="17"/>
+      <c r="F138" s="21" t="s">
         <v>291</v>
       </c>
-      <c r="G136" s="17" t="s">
+      <c r="G138" s="17" t="s">
         <v>337</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A137" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="B137" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C137" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="D137" s="2" t="s">
-        <v>689</v>
-      </c>
-      <c r="F137" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A138" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="B138" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C138" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="D138" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="F138" s="4" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.35">
@@ -5562,10 +5568,13 @@
         <v>269</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>689</v>
       </c>
       <c r="F139" s="4" t="s">
         <v>98</v>
@@ -5576,13 +5585,16 @@
         <v>269</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>405</v>
+        <v>267</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="F140" s="5" t="s">
-        <v>99</v>
+        <v>268</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.35">
@@ -5590,97 +5602,97 @@
         <v>269</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>181</v>
+        <v>265</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>180</v>
+        <v>266</v>
       </c>
       <c r="F141" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A142" s="2" t="s">
         <v>269</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>182</v>
+        <v>405</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="F142" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="F142" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A143" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="F143" s="4" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="143" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A143" s="17" t="s">
-        <v>269</v>
-      </c>
-      <c r="B143" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="C143" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="D143" s="17"/>
-      <c r="E143" s="17"/>
-      <c r="F143" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="G143" s="17"/>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
-        <v>55</v>
+        <v>269</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>458</v>
+        <v>182</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>459</v>
-      </c>
-      <c r="F144" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A145" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>778</v>
-      </c>
-      <c r="C145" s="2" t="s">
-        <v>781</v>
-      </c>
-      <c r="F145" s="5" t="s">
-        <v>99</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A145" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="B145" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="C145" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="D145" s="17"/>
+      <c r="E145" s="17"/>
+      <c r="F145" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="G145" s="17"/>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>779</v>
+        <v>458</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>782</v>
-      </c>
-      <c r="F146" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+        <v>459</v>
+      </c>
+      <c r="F146" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A147" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="F147" s="5" t="s">
         <v>99</v>
@@ -5691,16 +5703,13 @@
         <v>55</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>460</v>
+        <v>779</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>461</v>
-      </c>
-      <c r="D148" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="F148" s="3" t="s">
-        <v>97</v>
+        <v>782</v>
+      </c>
+      <c r="F148" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.35">
@@ -5708,27 +5717,27 @@
         <v>55</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>367</v>
+        <v>780</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="F149" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>783</v>
+      </c>
+      <c r="F149" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>56</v>
+        <v>460</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>59</v>
+        <v>461</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>262</v>
+        <v>462</v>
       </c>
       <c r="F150" s="3" t="s">
         <v>97</v>
@@ -5739,13 +5748,13 @@
         <v>55</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>301</v>
+        <v>367</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="F151" s="5" t="s">
-        <v>99</v>
+        <v>368</v>
+      </c>
+      <c r="F151" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="152" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5753,13 +5762,16 @@
         <v>55</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>767</v>
+        <v>56</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>768</v>
-      </c>
-      <c r="F152" s="5" t="s">
-        <v>99</v>
+        <v>59</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F152" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.35">
@@ -5767,27 +5779,24 @@
         <v>55</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>614</v>
+        <v>301</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>615</v>
+        <v>302</v>
       </c>
       <c r="F153" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>511</v>
+        <v>767</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>785</v>
-      </c>
-      <c r="E154" s="2" t="s">
-        <v>512</v>
+        <v>768</v>
       </c>
       <c r="F154" s="5" t="s">
         <v>99</v>
@@ -5798,10 +5807,10 @@
         <v>55</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>784</v>
+        <v>614</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>769</v>
+        <v>615</v>
       </c>
       <c r="F155" s="5" t="s">
         <v>99</v>
@@ -5812,13 +5821,16 @@
         <v>55</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>528</v>
+        <v>511</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>529</v>
-      </c>
-      <c r="F156" s="3" t="s">
-        <v>97</v>
+        <v>785</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="F156" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.35">
@@ -5826,30 +5838,27 @@
         <v>55</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>592</v>
+        <v>784</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="F157" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="158" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>769</v>
+      </c>
+      <c r="F157" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>57</v>
+        <v>528</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F158" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G158" s="2" t="s">
-        <v>325</v>
+        <v>529</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.35">
@@ -5857,13 +5866,13 @@
         <v>55</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>299</v>
+        <v>592</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="F159" s="5" t="s">
-        <v>99</v>
+        <v>593</v>
+      </c>
+      <c r="F159" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5871,33 +5880,30 @@
         <v>55</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>377</v>
+        <v>57</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="F160" s="16" t="s">
-        <v>291</v>
+        <v>60</v>
+      </c>
+      <c r="F160" s="6" t="s">
+        <v>140</v>
       </c>
       <c r="G160" s="2" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="161" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>378</v>
+        <v>299</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="F161" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G161" s="2" t="s">
-        <v>384</v>
+        <v>300</v>
+      </c>
+      <c r="F161" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="162" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5905,143 +5911,149 @@
         <v>55</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="F162" s="16" t="s">
         <v>291</v>
       </c>
       <c r="G162" s="2" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>58</v>
+        <v>378</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D163" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F163" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>381</v>
+      </c>
+      <c r="F163" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G163" s="2" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>363</v>
+        <v>379</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="D164" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="F164" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="165" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+        <v>382</v>
+      </c>
+      <c r="F164" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G164" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>375</v>
+        <v>58</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>376</v>
+        <v>61</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>62</v>
       </c>
       <c r="F165" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="166" spans="1:7" s="17" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A166" s="17" t="s">
+    <row r="166" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A166" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B166" s="17" t="s">
-        <v>428</v>
-      </c>
-      <c r="C166" s="17" t="s">
-        <v>429</v>
-      </c>
-      <c r="F166" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="G166" s="17" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="B166" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
-        <v>391</v>
+        <v>55</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>393</v>
+        <v>375</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="D167" s="2" t="s">
-        <v>395</v>
+        <v>376</v>
       </c>
       <c r="F167" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="168" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="168" spans="1:7" s="17" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A168" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B168" s="17" t="s">
+        <v>428</v>
+      </c>
+      <c r="C168" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F168" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="G168" s="17" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A169" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="F169" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A170" s="17" t="s">
         <v>742</v>
       </c>
-      <c r="B168" s="17" t="s">
+      <c r="B170" s="17" t="s">
         <v>743</v>
       </c>
-      <c r="C168" s="17" t="s">
+      <c r="C170" s="17" t="s">
         <v>744</v>
       </c>
-      <c r="D168" s="17" t="s">
+      <c r="D170" s="17" t="s">
         <v>745</v>
       </c>
-      <c r="F168" s="19" t="s">
+      <c r="F170" s="19" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A169" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="B169" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="C169" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="F169" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A170" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="B170" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="C170" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F170" s="4" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.35">
@@ -6049,109 +6061,106 @@
         <v>344</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="F171" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="172" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>353</v>
+      </c>
+      <c r="F171" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
         <v>344</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="D172" s="2" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="F172" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>344</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="F173" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
         <v>344</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="F174" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G174" s="2" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="175" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A175" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="F174" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A175" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="B175" s="17" t="s">
-        <v>352</v>
-      </c>
-      <c r="C175" s="17" t="s">
-        <v>359</v>
-      </c>
-      <c r="F175" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="G175" s="17" t="s">
-        <v>362</v>
+      <c r="B175" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C175" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F175" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
-        <v>63</v>
+        <v>344</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>810</v>
+        <v>351</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>811</v>
-      </c>
-      <c r="D176" s="2" t="s">
-        <v>812</v>
-      </c>
-      <c r="F176" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A177" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B177" s="2" t="s">
-        <v>815</v>
-      </c>
-      <c r="C177" s="2" t="s">
-        <v>816</v>
-      </c>
-      <c r="F177" s="16" t="s">
-        <v>291</v>
+        <v>358</v>
+      </c>
+      <c r="F176" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G176" s="2" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A177" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="B177" s="17" t="s">
+        <v>352</v>
+      </c>
+      <c r="C177" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="F177" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="G177" s="17" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.35">
@@ -6159,13 +6168,16 @@
         <v>63</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>817</v>
+        <v>810</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>818</v>
-      </c>
-      <c r="F178" s="16" t="s">
-        <v>291</v>
+        <v>811</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>812</v>
+      </c>
+      <c r="F178" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="179" spans="1:7" x14ac:dyDescent="0.35">
@@ -6173,27 +6185,27 @@
         <v>63</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>824</v>
+        <v>815</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="F179" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="180" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>816</v>
+      </c>
+      <c r="F179" s="16" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>827</v>
+        <v>817</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>826</v>
-      </c>
-      <c r="F180" s="3" t="s">
-        <v>97</v>
+        <v>818</v>
+      </c>
+      <c r="F180" s="16" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.35">
@@ -6201,16 +6213,13 @@
         <v>63</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>793</v>
+        <v>824</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>795</v>
-      </c>
-      <c r="D181" s="2" t="s">
-        <v>794</v>
-      </c>
-      <c r="F181" s="12" t="s">
-        <v>244</v>
+        <v>825</v>
+      </c>
+      <c r="F181" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="182" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6218,33 +6227,30 @@
         <v>63</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>504</v>
+        <v>827</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>505</v>
-      </c>
-      <c r="D182" s="2" t="s">
-        <v>506</v>
-      </c>
-      <c r="F182" s="14" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="183" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>826</v>
+      </c>
+      <c r="F182" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>648</v>
+        <v>793</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>649</v>
+        <v>795</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="F183" s="4" t="s">
-        <v>98</v>
+        <v>794</v>
+      </c>
+      <c r="F183" s="12" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="184" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6252,27 +6258,33 @@
         <v>63</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>314</v>
+        <v>504</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="F184" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
+        <v>505</v>
+      </c>
+      <c r="D184" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="F184" s="14" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>484</v>
+        <v>648</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="F185" s="5" t="s">
-        <v>99</v>
+        <v>649</v>
+      </c>
+      <c r="D185" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="F185" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="186" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6280,13 +6292,13 @@
         <v>63</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>799</v>
+        <v>314</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>800</v>
-      </c>
-      <c r="F186" s="4" t="s">
-        <v>98</v>
+        <v>315</v>
+      </c>
+      <c r="F186" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.35">
@@ -6294,44 +6306,44 @@
         <v>63</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>64</v>
+        <v>484</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F187" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G187" s="2" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
+        <v>485</v>
+      </c>
+      <c r="F187" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>802</v>
-      </c>
-      <c r="F188" s="14" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="189" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>800</v>
+      </c>
+      <c r="F188" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>807</v>
+        <v>64</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>808</v>
-      </c>
-      <c r="F189" s="5" t="s">
-        <v>99</v>
+        <v>66</v>
+      </c>
+      <c r="F189" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G189" s="2" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.35">
@@ -6339,47 +6351,41 @@
         <v>63</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="F190" s="14" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>828</v>
+        <v>807</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>829</v>
-      </c>
-      <c r="F191" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="192" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>808</v>
+      </c>
+      <c r="F191" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>796</v>
+        <v>803</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>797</v>
-      </c>
-      <c r="D192" s="2" t="s">
-        <v>809</v>
-      </c>
-      <c r="F192" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="G192" s="2" t="s">
-        <v>798</v>
+        <v>804</v>
+      </c>
+      <c r="F192" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.35">
@@ -6387,27 +6393,33 @@
         <v>63</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>547</v>
+        <v>828</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="F193" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.35">
+        <v>829</v>
+      </c>
+      <c r="F193" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>748</v>
+        <v>796</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>749</v>
+        <v>797</v>
+      </c>
+      <c r="D194" s="2" t="s">
+        <v>809</v>
       </c>
       <c r="F194" s="4" t="s">
         <v>98</v>
+      </c>
+      <c r="G194" s="2" t="s">
+        <v>798</v>
       </c>
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.35">
@@ -6415,61 +6427,58 @@
         <v>63</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>754</v>
+        <v>547</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>755</v>
-      </c>
-      <c r="F195" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="196" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>548</v>
+      </c>
+      <c r="F195" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>501</v>
+        <v>748</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="F196" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G196" s="2" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="197" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>749</v>
+      </c>
+      <c r="F196" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>819</v>
+        <v>754</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>822</v>
-      </c>
-      <c r="D197" s="2" t="s">
-        <v>823</v>
+        <v>755</v>
       </c>
       <c r="F197" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>195</v>
+        <v>501</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="F198" s="4" t="s">
-        <v>98</v>
+        <v>502</v>
+      </c>
+      <c r="F198" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G198" s="2" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="199" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6477,50 +6486,50 @@
         <v>63</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>842</v>
+        <v>819</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>843</v>
+        <v>822</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>844</v>
-      </c>
-      <c r="F199" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G199" s="2" t="s">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="200" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>823</v>
+      </c>
+      <c r="F199" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>65</v>
+        <v>195</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D200" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="F200" s="14" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
+        <v>196</v>
+      </c>
+      <c r="F200" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>188</v>
+        <v>842</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="F201" s="4" t="s">
-        <v>98</v>
+        <v>843</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>844</v>
+      </c>
+      <c r="F201" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G201" s="2" t="s">
+        <v>845</v>
       </c>
     </row>
     <row r="202" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6528,41 +6537,44 @@
         <v>63</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>552</v>
+        <v>65</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>553</v>
-      </c>
-      <c r="F202" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="203" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+      <c r="D202" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="F202" s="14" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>813</v>
+        <v>188</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>814</v>
+        <v>189</v>
       </c>
       <c r="F203" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>464</v>
+        <v>552</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="F204" s="4" t="s">
-        <v>98</v>
+        <v>553</v>
+      </c>
+      <c r="F204" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="205" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6570,27 +6582,27 @@
         <v>63</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>480</v>
+        <v>813</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>481</v>
+        <v>814</v>
       </c>
       <c r="F205" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="206" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>820</v>
+        <v>464</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>821</v>
-      </c>
-      <c r="F206" s="5" t="s">
-        <v>99</v>
+        <v>463</v>
+      </c>
+      <c r="F206" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="207" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6598,89 +6610,86 @@
         <v>63</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F207" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="208" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A208" s="17" t="s">
+    <row r="208" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A208" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B208" s="17" t="s">
+      <c r="B208" s="2" t="s">
+        <v>820</v>
+      </c>
+      <c r="C208" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="F208" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A209" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B209" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C209" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="F209" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A210" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B210" s="17" t="s">
         <v>830</v>
       </c>
-      <c r="C208" s="17" t="s">
+      <c r="C210" s="17" t="s">
         <v>831</v>
       </c>
-      <c r="D208" s="17"/>
-      <c r="E208" s="17"/>
-      <c r="F208" s="19" t="s">
+      <c r="D210" s="17"/>
+      <c r="E210" s="17"/>
+      <c r="F210" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="G208" s="17"/>
-    </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A209" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="B209" s="2" t="s">
-        <v>786</v>
-      </c>
-      <c r="C209" s="2" t="s">
-        <v>787</v>
-      </c>
-      <c r="F209" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="210" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A210" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="B210" s="2" t="s">
-        <v>544</v>
-      </c>
-      <c r="C210" s="2" t="s">
-        <v>545</v>
-      </c>
-      <c r="D210" s="2" t="s">
-        <v>546</v>
-      </c>
-      <c r="F210" s="3" t="s">
-        <v>97</v>
-      </c>
+      <c r="G210" s="17"/>
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>695</v>
+        <v>786</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>696</v>
-      </c>
-      <c r="D211" s="2" t="s">
-        <v>694</v>
+        <v>787</v>
       </c>
       <c r="F211" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>415</v>
+        <v>544</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>416</v>
+        <v>545</v>
+      </c>
+      <c r="D212" s="2" t="s">
+        <v>546</v>
       </c>
       <c r="F212" s="3" t="s">
         <v>97</v>
@@ -6691,10 +6700,13 @@
         <v>407</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>417</v>
+        <v>695</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>418</v>
+        <v>696</v>
+      </c>
+      <c r="D213" s="2" t="s">
+        <v>694</v>
       </c>
       <c r="F213" s="3" t="s">
         <v>97</v>
@@ -6705,10 +6717,10 @@
         <v>407</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>388</v>
+        <v>415</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>389</v>
+        <v>416</v>
       </c>
       <c r="F214" s="3" t="s">
         <v>97</v>
@@ -6719,30 +6731,24 @@
         <v>407</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="F215" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="216" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>598</v>
+        <v>388</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>600</v>
-      </c>
-      <c r="D216" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="E216" s="2" t="s">
-        <v>421</v>
+        <v>389</v>
       </c>
       <c r="F216" s="3" t="s">
         <v>97</v>
@@ -6753,107 +6759,110 @@
         <v>407</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="F217" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>409</v>
+        <v>598</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>411</v>
+        <v>600</v>
+      </c>
+      <c r="D218" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="E218" s="2" t="s">
+        <v>421</v>
       </c>
       <c r="F218" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="219" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>515</v>
+        <v>421</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="F219" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G219" s="2" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="220" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>422</v>
+      </c>
+      <c r="F219" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>467</v>
+        <v>409</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="D220" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="F220" s="3"/>
-    </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.35">
+        <v>411</v>
+      </c>
+      <c r="F220" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="F221" s="6" t="s">
-        <v>140</v>
+        <v>516</v>
+      </c>
+      <c r="F221" s="16" t="s">
+        <v>291</v>
       </c>
       <c r="G221" s="2" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.35">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>488</v>
+        <v>467</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>489</v>
-      </c>
-      <c r="E222" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="F222" s="3" t="s">
-        <v>97</v>
-      </c>
+        <v>468</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="F222" s="3"/>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>486</v>
+        <v>513</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="F223" s="5" t="s">
-        <v>99</v>
+        <v>514</v>
+      </c>
+      <c r="F223" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G223" s="2" t="s">
+        <v>518</v>
       </c>
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.35">
@@ -6861,13 +6870,16 @@
         <v>407</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>454</v>
+        <v>488</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="F224" s="5" t="s">
-        <v>99</v>
+        <v>489</v>
+      </c>
+      <c r="E224" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F224" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.35">
@@ -6875,10 +6887,10 @@
         <v>407</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>410</v>
+        <v>486</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>412</v>
+        <v>487</v>
       </c>
       <c r="F225" s="5" t="s">
         <v>99</v>
@@ -6889,10 +6901,10 @@
         <v>407</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="F226" s="5" t="s">
         <v>99</v>
@@ -6903,151 +6915,151 @@
         <v>407</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>526</v>
+        <v>410</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="F227" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="228" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>412</v>
+      </c>
+      <c r="F227" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>413</v>
+        <v>456</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="F228" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G228" s="2" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="229" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>457</v>
+      </c>
+      <c r="F228" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
         <v>407</v>
       </c>
       <c r="B229" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C229" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="F229" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A230" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B230" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C230" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F230" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G230" s="2" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A231" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B231" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C229" s="2" t="s">
+      <c r="C231" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="F229" s="19" t="s">
+      <c r="F231" s="19" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="230" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A230" s="17" t="s">
+    <row r="232" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A232" s="17" t="s">
         <v>407</v>
       </c>
-      <c r="B230" s="17" t="s">
+      <c r="B232" s="17" t="s">
         <v>478</v>
       </c>
-      <c r="C230" s="17" t="s">
+      <c r="C232" s="17" t="s">
         <v>479</v>
       </c>
-      <c r="D230" s="17"/>
-      <c r="E230" s="17"/>
-      <c r="F230" s="19" t="s">
+      <c r="D232" s="17"/>
+      <c r="E232" s="17"/>
+      <c r="F232" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="G230" s="17"/>
-    </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A231" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B231" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="C231" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="F231" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A232" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B232" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="C232" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="E232" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F232" s="12" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="233" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="G232" s="17"/>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A233" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F233" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="234" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A234" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>207</v>
+        <v>292</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="F234" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G234" s="2" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
+        <v>293</v>
+      </c>
+      <c r="E234" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F234" s="12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A235" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="F235" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A236" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>92</v>
+        <v>207</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F236" s="5" t="s">
-        <v>99</v>
+        <v>208</v>
+      </c>
+      <c r="F236" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G236" s="2" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.35">
@@ -7055,142 +7067,142 @@
         <v>91</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="F237" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="238" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>214</v>
+      </c>
+      <c r="F237" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A238" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>212</v>
+        <v>92</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="F238" s="12" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="239" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A239" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="F238" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A239" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B239" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="C239" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="D239" s="17"/>
-      <c r="E239" s="17"/>
-      <c r="F239" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="G239" s="17"/>
+      <c r="B239" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C239" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F239" s="3" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="240" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A240" s="2" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>69</v>
+        <v>212</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F240" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G240" s="2" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="241" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A241" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B241" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C241" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="F241" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G241" s="2" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
+        <v>213</v>
+      </c>
+      <c r="F240" s="12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A241" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B241" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="C241" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D241" s="17"/>
+      <c r="E241" s="17"/>
+      <c r="F241" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="G241" s="17"/>
+    </row>
+    <row r="242" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A242" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>729</v>
+        <v>69</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>730</v>
+        <v>70</v>
       </c>
       <c r="F242" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G242" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A243" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B243" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C243" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="F243" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="G242" s="2" t="s">
-        <v>731</v>
-      </c>
-    </row>
-    <row r="243" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A243" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="B243" s="17" t="s">
-        <v>191</v>
-      </c>
-      <c r="C243" s="17" t="s">
-        <v>193</v>
-      </c>
-      <c r="D243" s="17"/>
-      <c r="E243" s="17"/>
-      <c r="F243" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="G243" s="17" t="s">
-        <v>324</v>
+      <c r="G243" s="2" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A244" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>617</v>
+        <v>729</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="F244" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A245" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B245" s="2" t="s">
-        <v>535</v>
-      </c>
-      <c r="C245" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="F245" s="5" t="s">
-        <v>99</v>
+        <v>730</v>
+      </c>
+      <c r="F244" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G244" s="2" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="245" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A245" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B245" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="C245" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="D245" s="17"/>
+      <c r="E245" s="17"/>
+      <c r="F245" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="G245" s="17" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="246" spans="1:7" x14ac:dyDescent="0.35">
@@ -7198,10 +7210,10 @@
         <v>71</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>72</v>
+        <v>617</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>80</v>
+        <v>618</v>
       </c>
       <c r="F246" s="4" t="s">
         <v>98</v>
@@ -7212,27 +7224,27 @@
         <v>71</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>73</v>
+        <v>535</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>81</v>
+        <v>536</v>
       </c>
       <c r="F247" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="248" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A248" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>539</v>
+        <v>72</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>540</v>
-      </c>
-      <c r="F248" s="5" t="s">
-        <v>99</v>
+        <v>80</v>
+      </c>
+      <c r="F248" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="249" spans="1:7" x14ac:dyDescent="0.35">
@@ -7240,27 +7252,27 @@
         <v>71</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>398</v>
+        <v>73</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="F249" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+      <c r="F249" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A250" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>661</v>
+        <v>539</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>662</v>
-      </c>
-      <c r="F250" s="4" t="s">
-        <v>98</v>
+        <v>540</v>
+      </c>
+      <c r="F250" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="251" spans="1:7" x14ac:dyDescent="0.35">
@@ -7268,13 +7280,13 @@
         <v>71</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>537</v>
+        <v>398</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>538</v>
-      </c>
-      <c r="F251" s="5" t="s">
-        <v>99</v>
+        <v>399</v>
+      </c>
+      <c r="F251" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.35">
@@ -7282,13 +7294,13 @@
         <v>71</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>271</v>
+        <v>661</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="F252" s="3" t="s">
-        <v>97</v>
+        <v>662</v>
+      </c>
+      <c r="F252" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.35">
@@ -7296,30 +7308,27 @@
         <v>71</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>250</v>
+        <v>537</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="F253" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="254" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>538</v>
+      </c>
+      <c r="F253" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A254" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>230</v>
+        <v>271</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E254" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="F254" s="5" t="s">
-        <v>99</v>
+        <v>272</v>
+      </c>
+      <c r="F254" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.35">
@@ -7327,24 +7336,27 @@
         <v>71</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>788</v>
+        <v>250</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>789</v>
+        <v>251</v>
       </c>
       <c r="F255" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A256" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>603</v>
+        <v>230</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>604</v>
+        <v>231</v>
+      </c>
+      <c r="E256" s="2" t="s">
+        <v>366</v>
       </c>
       <c r="F256" s="5" t="s">
         <v>99</v>
@@ -7355,13 +7367,13 @@
         <v>71</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>605</v>
+        <v>788</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="F257" s="5" t="s">
-        <v>99</v>
+        <v>789</v>
+      </c>
+      <c r="F257" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.35">
@@ -7369,10 +7381,10 @@
         <v>71</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>226</v>
+        <v>603</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>227</v>
+        <v>604</v>
       </c>
       <c r="F258" s="5" t="s">
         <v>99</v>
@@ -7383,10 +7395,10 @@
         <v>71</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>222</v>
+        <v>605</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>223</v>
+        <v>606</v>
       </c>
       <c r="F259" s="5" t="s">
         <v>99</v>
@@ -7397,13 +7409,10 @@
         <v>71</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>619</v>
+        <v>226</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="D260" s="2" t="s">
-        <v>621</v>
+        <v>227</v>
       </c>
       <c r="F260" s="5" t="s">
         <v>99</v>
@@ -7414,10 +7423,10 @@
         <v>71</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>607</v>
+        <v>222</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>608</v>
+        <v>223</v>
       </c>
       <c r="F261" s="5" t="s">
         <v>99</v>
@@ -7428,13 +7437,16 @@
         <v>71</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>846</v>
+        <v>619</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>847</v>
-      </c>
-      <c r="F262" s="3" t="s">
-        <v>97</v>
+        <v>620</v>
+      </c>
+      <c r="D262" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="F262" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.35">
@@ -7442,13 +7454,13 @@
         <v>71</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>692</v>
+        <v>607</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="F263" s="3" t="s">
-        <v>97</v>
+        <v>608</v>
+      </c>
+      <c r="F263" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.35">
@@ -7456,10 +7468,10 @@
         <v>71</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>622</v>
+        <v>846</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>623</v>
+        <v>847</v>
       </c>
       <c r="F264" s="3" t="s">
         <v>97</v>
@@ -7470,10 +7482,10 @@
         <v>71</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>594</v>
+        <v>692</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>595</v>
+        <v>693</v>
       </c>
       <c r="F265" s="3" t="s">
         <v>97</v>
@@ -7484,13 +7496,13 @@
         <v>71</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>574</v>
+        <v>622</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="F266" s="4" t="s">
-        <v>98</v>
+        <v>623</v>
+      </c>
+      <c r="F266" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.35">
@@ -7498,30 +7510,27 @@
         <v>71</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>235</v>
+        <v>594</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="F267" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="268" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>595</v>
+      </c>
+      <c r="F267" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A268" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>273</v>
+        <v>574</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="F268" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="G268" s="2" t="s">
-        <v>322</v>
+        <v>575</v>
+      </c>
+      <c r="F268" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.35">
@@ -7529,27 +7538,30 @@
         <v>71</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>74</v>
+        <v>235</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F269" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.35">
+        <v>236</v>
+      </c>
+      <c r="F269" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A270" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>75</v>
+        <v>273</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F270" s="5" t="s">
-        <v>99</v>
+        <v>274</v>
+      </c>
+      <c r="F270" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G270" s="2" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="271" spans="1:7" x14ac:dyDescent="0.35">
@@ -7557,10 +7569,10 @@
         <v>71</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F271" s="5" t="s">
         <v>99</v>
@@ -7571,13 +7583,13 @@
         <v>71</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F272" s="4" t="s">
-        <v>98</v>
+        <v>83</v>
+      </c>
+      <c r="F272" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.35">
@@ -7585,13 +7597,10 @@
         <v>71</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>609</v>
+        <v>76</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="D273" s="2" t="s">
-        <v>611</v>
+        <v>84</v>
       </c>
       <c r="F273" s="5" t="s">
         <v>99</v>
@@ -7602,10 +7611,10 @@
         <v>71</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>435</v>
+        <v>77</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>436</v>
+        <v>85</v>
       </c>
       <c r="F274" s="4" t="s">
         <v>98</v>
@@ -7616,27 +7625,30 @@
         <v>71</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>465</v>
+        <v>609</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="F275" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="276" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>610</v>
+      </c>
+      <c r="D275" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="F275" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="276" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A276" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>624</v>
+        <v>435</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>625</v>
-      </c>
-      <c r="F276" s="5" t="s">
-        <v>99</v>
+        <v>436</v>
+      </c>
+      <c r="F276" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.35">
@@ -7644,27 +7656,27 @@
         <v>71</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>723</v>
+        <v>465</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>724</v>
-      </c>
-      <c r="F277" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
+        <v>466</v>
+      </c>
+      <c r="F277" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A278" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>78</v>
+        <v>624</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F278" s="3" t="s">
-        <v>97</v>
+        <v>625</v>
+      </c>
+      <c r="F278" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.35">
@@ -7672,47 +7684,41 @@
         <v>71</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>533</v>
+        <v>723</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="F279" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="280" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>724</v>
+      </c>
+      <c r="F279" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="280" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A280" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>281</v>
+        <v>78</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="F280" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G280" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="281" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+      <c r="F280" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A281" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>283</v>
+        <v>533</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="F281" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G281" s="2" t="s">
-        <v>323</v>
+        <v>534</v>
+      </c>
+      <c r="F281" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="282" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -7720,10 +7726,10 @@
         <v>71</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>233</v>
+        <v>281</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>234</v>
+        <v>282</v>
       </c>
       <c r="F282" s="16" t="s">
         <v>291</v>
@@ -7732,80 +7738,83 @@
         <v>323</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A283" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>224</v>
+        <v>283</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E283" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="F283" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="284" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>284</v>
+      </c>
+      <c r="F283" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G283" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A284" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>675</v>
+        <v>233</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>676</v>
-      </c>
-      <c r="F284" s="5" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="285" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+      <c r="F284" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G284" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A285" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>79</v>
+        <v>224</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>87</v>
+        <v>225</v>
+      </c>
+      <c r="E285" s="2" t="s">
+        <v>222</v>
       </c>
       <c r="F285" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A286" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>727</v>
+        <v>675</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>728</v>
-      </c>
-      <c r="F286" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="287" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>676</v>
+      </c>
+      <c r="F286" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A287" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>430</v>
+        <v>79</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="F287" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G287" s="2" t="s">
-        <v>364</v>
+        <v>87</v>
+      </c>
+      <c r="F287" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.35">
@@ -7813,44 +7822,44 @@
         <v>71</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>626</v>
+        <v>727</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="F288" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.35">
+        <v>728</v>
+      </c>
+      <c r="F288" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A289" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>492</v>
+        <v>430</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="F289" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="290" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>431</v>
+      </c>
+      <c r="F289" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G289" s="2" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A290" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>760</v>
+        <v>626</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>761</v>
-      </c>
-      <c r="F290" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G290" s="2" t="s">
-        <v>762</v>
+        <v>627</v>
+      </c>
+      <c r="F290" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.35">
@@ -7858,27 +7867,30 @@
         <v>71</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>239</v>
+        <v>492</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="F291" s="14" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.35">
+        <v>493</v>
+      </c>
+      <c r="F291" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A292" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>286</v>
+        <v>760</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="F292" s="5" t="s">
-        <v>99</v>
+        <v>761</v>
+      </c>
+      <c r="F292" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G292" s="2" t="s">
+        <v>762</v>
       </c>
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.35">
@@ -7886,13 +7898,13 @@
         <v>71</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>628</v>
+        <v>239</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>629</v>
-      </c>
-      <c r="F293" s="4" t="s">
-        <v>98</v>
+        <v>240</v>
+      </c>
+      <c r="F293" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="294" spans="1:7" x14ac:dyDescent="0.35">
@@ -7900,10 +7912,10 @@
         <v>71</v>
       </c>
       <c r="B294" s="2" t="s">
-        <v>228</v>
+        <v>286</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>229</v>
+        <v>285</v>
       </c>
       <c r="F294" s="5" t="s">
         <v>99</v>
@@ -7914,13 +7926,13 @@
         <v>71</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>612</v>
+        <v>628</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="F295" s="5" t="s">
-        <v>99</v>
+        <v>629</v>
+      </c>
+      <c r="F295" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="296" spans="1:7" x14ac:dyDescent="0.35">
@@ -7928,13 +7940,13 @@
         <v>71</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F296" s="12" t="s">
-        <v>244</v>
+        <v>229</v>
+      </c>
+      <c r="F296" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="297" spans="1:7" x14ac:dyDescent="0.35">
@@ -7942,13 +7954,13 @@
         <v>71</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>509</v>
+        <v>612</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>510</v>
-      </c>
-      <c r="F297" s="14" t="s">
-        <v>252</v>
+        <v>613</v>
+      </c>
+      <c r="F297" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="298" spans="1:7" x14ac:dyDescent="0.35">
@@ -7956,16 +7968,13 @@
         <v>71</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>507</v>
+        <v>220</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>508</v>
-      </c>
-      <c r="E298" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="F298" s="5" t="s">
-        <v>99</v>
+        <v>221</v>
+      </c>
+      <c r="F298" s="12" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.35">
@@ -7973,194 +7982,225 @@
         <v>71</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>218</v>
+        <v>509</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F299" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="300" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>510</v>
+      </c>
+      <c r="F299" s="14" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A300" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>630</v>
+        <v>507</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>631</v>
-      </c>
-      <c r="F300" s="20" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="301" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>508</v>
+      </c>
+      <c r="E300" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="F300" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A301" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>569</v>
+        <v>218</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>571</v>
-      </c>
-      <c r="F301" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="G301" s="2" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="302" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>219</v>
+      </c>
+      <c r="F301" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="302" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A302" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B302" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C302" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="F302" s="20" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="303" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A303" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B303" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="C303" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="F303" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G303" s="2" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="304" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A304" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B304" s="2" t="s">
         <v>570</v>
       </c>
-      <c r="C302" s="2" t="s">
+      <c r="C304" s="2" t="s">
         <v>573</v>
       </c>
-      <c r="F302" s="16" t="s">
+      <c r="F304" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G302" s="2" t="s">
+      <c r="G304" s="2" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="303" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A303" s="17" t="s">
+    <row r="305" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A305" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B303" s="17" t="s">
+      <c r="B305" s="17" t="s">
         <v>294</v>
       </c>
-      <c r="C303" s="17" t="s">
+      <c r="C305" s="17" t="s">
         <v>295</v>
       </c>
-      <c r="D303" s="17"/>
-      <c r="E303" s="17"/>
-      <c r="F303" s="20" t="s">
+      <c r="D305" s="17"/>
+      <c r="E305" s="17"/>
+      <c r="F305" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="G303" s="17"/>
-    </row>
-    <row r="304" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A304" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B304" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C304" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D304" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="F304" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A305" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B305" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C305" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="D305" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="F305" s="5" t="s">
-        <v>99</v>
-      </c>
+      <c r="G305" s="17"/>
     </row>
     <row r="306" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A306" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>241</v>
+        <v>89</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>242</v>
+        <v>90</v>
       </c>
       <c r="D306" s="2" t="s">
-        <v>243</v>
+        <v>303</v>
       </c>
       <c r="F306" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="307" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A307" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>790</v>
+        <v>216</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>791</v>
-      </c>
-      <c r="F307" s="25" t="s">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.35">
+        <v>215</v>
+      </c>
+      <c r="D307" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="F307" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="308" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A308" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>338</v>
+        <v>241</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="F308" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+      <c r="D308" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F308" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="309" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A309" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B309" s="2" t="s">
+        <v>790</v>
+      </c>
+      <c r="C309" s="2" t="s">
+        <v>791</v>
+      </c>
+      <c r="F309" s="25" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="310" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A310" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B310" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C310" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F310" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="311" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A311" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B311" s="2" t="s">
         <v>549</v>
       </c>
-      <c r="C309" s="2" t="s">
+      <c r="C311" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="D309" s="2" t="s">
+      <c r="D311" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="F309" s="4" t="s">
+      <c r="F311" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="310" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A310" s="17" t="s">
+    <row r="312" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A312" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="B310" s="17" t="s">
+      <c r="B312" s="17" t="s">
         <v>279</v>
       </c>
-      <c r="C310" s="17" t="s">
+      <c r="C312" s="17" t="s">
         <v>280</v>
       </c>
-      <c r="D310" s="17" t="s">
+      <c r="D312" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="E310" s="17"/>
-      <c r="F310" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="G310" s="17"/>
+      <c r="E312" s="17"/>
+      <c r="F312" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="G312" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Remove Reliability Electricity Source subscript
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6DE3C43-F88F-45B3-93AC-4CC625C8192A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A8D342-CF64-453A-BCA2-30B4659ED6AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1437" uniqueCount="834">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="832">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2399,12 +2399,6 @@
   </si>
   <si>
     <t>Cap Ret per Unit Net Loss</t>
-  </si>
-  <si>
-    <t>ESUfRaLCD</t>
-  </si>
-  <si>
-    <t>Elec Sources Used for Rlbty and Lst Cst Dsptch</t>
   </si>
   <si>
     <t>BFoICbCTBA</t>
@@ -3345,7 +3339,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G302"/>
+  <dimension ref="A1:G301"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
@@ -3588,16 +3582,16 @@
         <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="F15" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -4015,19 +4009,19 @@
         <v>36</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>809</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>810</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>811</v>
       </c>
       <c r="F43" s="21" t="s">
         <v>303</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -4166,16 +4160,16 @@
         <v>413</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -4353,10 +4347,10 @@
         <v>413</v>
       </c>
       <c r="B63" s="17" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="C63" s="17" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="D63" s="17"/>
       <c r="E63" s="17"/>
@@ -4364,7 +4358,7 @@
         <v>303</v>
       </c>
       <c r="G63" s="17" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
@@ -4684,10 +4678,10 @@
         <v>43</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="F84" s="3" t="s">
         <v>99</v>
@@ -4932,13 +4926,13 @@
         <v>43</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>789</v>
+        <v>822</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>790</v>
-      </c>
-      <c r="F100" s="5" t="s">
-        <v>101</v>
+        <v>823</v>
+      </c>
+      <c r="F100" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.35">
@@ -4946,13 +4940,13 @@
         <v>43</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>824</v>
+        <v>731</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="F101" s="3" t="s">
-        <v>99</v>
+        <v>732</v>
+      </c>
+      <c r="F101" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.35">
@@ -4960,114 +4954,114 @@
         <v>43</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>731</v>
+        <v>489</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>732</v>
-      </c>
-      <c r="F102" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+        <v>490</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="F102" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>489</v>
+        <v>177</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>704</v>
-      </c>
-      <c r="F103" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>176</v>
+      </c>
+      <c r="F103" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G103" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>177</v>
+        <v>766</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F104" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G104" s="2" t="s">
-        <v>321</v>
+        <v>768</v>
+      </c>
+      <c r="F104" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A105" s="2" t="s">
+      <c r="B105" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="F105" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A106" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B105" s="2" t="s">
-        <v>766</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>768</v>
-      </c>
-      <c r="F105" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B106" s="2" t="s">
-        <v>767</v>
+        <v>713</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>769</v>
-      </c>
-      <c r="F106" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>714</v>
+      </c>
+      <c r="F106" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>713</v>
+        <v>733</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>714</v>
+        <v>734</v>
       </c>
       <c r="F107" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>733</v>
+        <v>592</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>734</v>
+        <v>593</v>
       </c>
       <c r="F108" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>592</v>
+        <v>605</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="F109" s="4" t="s">
-        <v>100</v>
+        <v>606</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.35">
@@ -5075,10 +5069,10 @@
         <v>43</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>605</v>
+        <v>750</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>606</v>
+        <v>751</v>
       </c>
       <c r="F110" s="3" t="s">
         <v>99</v>
@@ -5089,13 +5083,13 @@
         <v>43</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>750</v>
+        <v>596</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>751</v>
-      </c>
-      <c r="F111" s="3" t="s">
-        <v>99</v>
+        <v>597</v>
+      </c>
+      <c r="F111" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.35">
@@ -5103,10 +5097,10 @@
         <v>43</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>596</v>
+        <v>662</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>597</v>
+        <v>663</v>
       </c>
       <c r="F112" s="4" t="s">
         <v>100</v>
@@ -5117,13 +5111,13 @@
         <v>43</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>662</v>
+        <v>48</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>663</v>
-      </c>
-      <c r="F113" s="4" t="s">
-        <v>100</v>
+        <v>53</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.35">
@@ -5131,27 +5125,30 @@
         <v>43</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>48</v>
+        <v>196</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F114" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+        <v>208</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>196</v>
+        <v>49</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="F115" s="4" t="s">
-        <v>100</v>
+        <v>54</v>
+      </c>
+      <c r="F115" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="116" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -5159,33 +5156,33 @@
         <v>43</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>49</v>
+        <v>755</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>54</v>
+        <v>756</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>102</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>755</v>
+        <v>748</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>756</v>
-      </c>
-      <c r="F117" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G117" s="2" t="s">
-        <v>757</v>
+        <v>749</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="F117" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5193,44 +5190,41 @@
         <v>43</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>748</v>
+        <v>669</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>749</v>
+        <v>670</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>763</v>
-      </c>
-      <c r="F118" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>735</v>
+      </c>
+      <c r="F118" s="14" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>669</v>
+        <v>186</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>735</v>
-      </c>
-      <c r="F119" s="14" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>186</v>
+        <v>579</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>187</v>
+        <v>580</v>
       </c>
       <c r="F120" s="4" t="s">
         <v>100</v>
@@ -5241,13 +5235,16 @@
         <v>43</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>579</v>
+        <v>203</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>580</v>
-      </c>
-      <c r="F121" s="4" t="s">
-        <v>100</v>
+        <v>204</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="F121" s="5" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5255,78 +5252,75 @@
         <v>43</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>203</v>
+        <v>681</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>204</v>
+        <v>682</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>205</v>
+        <v>683</v>
       </c>
       <c r="F122" s="5" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="123" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>681</v>
+        <v>600</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>682</v>
+        <v>601</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>683</v>
-      </c>
-      <c r="F123" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A124" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="F123" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="B124" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="F124" s="14" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A125" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B124" s="2" t="s">
-        <v>600</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="F124" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="125" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B125" s="2" t="s">
-        <v>667</v>
+        <v>452</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>668</v>
-      </c>
-      <c r="F125" s="14" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>453</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="F125" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>452</v>
+        <v>679</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="F126" s="4" t="s">
-        <v>100</v>
+        <v>680</v>
+      </c>
+      <c r="F126" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5334,13 +5328,13 @@
         <v>43</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>679</v>
+        <v>651</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>680</v>
-      </c>
-      <c r="F127" s="14" t="s">
-        <v>258</v>
+        <v>652</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5348,10 +5342,10 @@
         <v>43</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F128" s="4" t="s">
         <v>100</v>
@@ -5362,27 +5356,27 @@
         <v>43</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>653</v>
+        <v>574</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>654</v>
+        <v>575</v>
       </c>
       <c r="F129" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>574</v>
+        <v>649</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="F130" s="4" t="s">
-        <v>100</v>
+        <v>650</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.35">
@@ -5390,27 +5384,30 @@
         <v>43</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>649</v>
+        <v>598</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>650</v>
+        <v>599</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>596</v>
       </c>
       <c r="F131" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>598</v>
+        <v>736</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="E132" s="2" t="s">
-        <v>596</v>
+        <v>737</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>738</v>
       </c>
       <c r="F132" s="3" t="s">
         <v>99</v>
@@ -5421,16 +5418,13 @@
         <v>43</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>736</v>
+        <v>820</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="D133" s="2" t="s">
-        <v>738</v>
-      </c>
-      <c r="F133" s="3" t="s">
-        <v>99</v>
+        <v>821</v>
+      </c>
+      <c r="F133" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5438,110 +5432,110 @@
         <v>43</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>822</v>
+        <v>706</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>823</v>
-      </c>
-      <c r="F134" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="F134" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A135" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B135" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="C135" s="17" t="s">
+        <v>348</v>
+      </c>
+      <c r="D135" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="E135" s="17"/>
+      <c r="F135" s="21" t="s">
+        <v>303</v>
+      </c>
+      <c r="G135" s="17" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A136" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="F136" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A135" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B135" s="2" t="s">
-        <v>706</v>
-      </c>
-      <c r="C135" s="2" t="s">
-        <v>707</v>
-      </c>
-      <c r="F135" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A136" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="B136" s="17" t="s">
-        <v>347</v>
-      </c>
-      <c r="C136" s="17" t="s">
-        <v>348</v>
-      </c>
-      <c r="D136" s="17" t="s">
-        <v>349</v>
-      </c>
-      <c r="E136" s="17"/>
-      <c r="F136" s="21" t="s">
-        <v>303</v>
-      </c>
-      <c r="G136" s="17" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>705</v>
+        <v>631</v>
       </c>
       <c r="F137" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="D138" s="2" t="s">
-        <v>631</v>
+        <v>272</v>
       </c>
       <c r="F138" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>271</v>
+        <v>418</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="F139" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>419</v>
+      </c>
+      <c r="F139" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>418</v>
+        <v>183</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="F140" s="5" t="s">
-        <v>101</v>
+        <v>182</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.35">
@@ -5549,69 +5543,69 @@
         <v>275</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F141" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A142" s="2" t="s">
+    <row r="142" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A142" s="17" t="s">
         <v>275</v>
       </c>
-      <c r="B142" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C142" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="F142" s="4" t="s">
+      <c r="B142" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="C142" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="D142" s="17"/>
+      <c r="E142" s="17"/>
+      <c r="F142" s="20" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="143" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A143" s="17" t="s">
-        <v>275</v>
-      </c>
-      <c r="B143" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="C143" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="D143" s="17"/>
-      <c r="E143" s="17"/>
-      <c r="F143" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="G143" s="17"/>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G142" s="17"/>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A143" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>471</v>
+        <v>789</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="F144" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>792</v>
+      </c>
+      <c r="F144" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="F145" s="5" t="s">
         <v>101</v>
@@ -5622,10 +5616,10 @@
         <v>55</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="F146" s="5" t="s">
         <v>101</v>
@@ -5636,13 +5630,16 @@
         <v>55</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>793</v>
+        <v>473</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>796</v>
-      </c>
-      <c r="F147" s="5" t="s">
-        <v>101</v>
+        <v>474</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.35">
@@ -5650,72 +5647,69 @@
         <v>55</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>473</v>
+        <v>380</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="D148" s="2" t="s">
-        <v>475</v>
+        <v>381</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>380</v>
+        <v>56</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>381</v>
+        <v>59</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>268</v>
       </c>
       <c r="F149" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="150" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>56</v>
+        <v>313</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D150" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="F150" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+        <v>314</v>
+      </c>
+      <c r="F150" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>313</v>
+        <v>780</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>314</v>
+        <v>781</v>
       </c>
       <c r="F151" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="152" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>780</v>
+        <v>629</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>781</v>
+        <v>630</v>
       </c>
       <c r="F152" s="5" t="s">
         <v>101</v>
@@ -5726,10 +5720,13 @@
         <v>55</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>629</v>
+        <v>526</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>630</v>
+        <v>796</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>527</v>
       </c>
       <c r="F153" s="5" t="s">
         <v>101</v>
@@ -5740,13 +5737,10 @@
         <v>55</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>526</v>
+        <v>795</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>798</v>
-      </c>
-      <c r="E154" s="2" t="s">
-        <v>527</v>
+        <v>782</v>
       </c>
       <c r="F154" s="5" t="s">
         <v>101</v>
@@ -5757,13 +5751,13 @@
         <v>55</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>797</v>
+        <v>543</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>782</v>
-      </c>
-      <c r="F155" s="5" t="s">
-        <v>101</v>
+        <v>544</v>
+      </c>
+      <c r="F155" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.35">
@@ -5771,58 +5765,61 @@
         <v>55</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>543</v>
+        <v>607</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>544</v>
-      </c>
-      <c r="F156" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+        <v>608</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>607</v>
+        <v>57</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>608</v>
-      </c>
-      <c r="F157" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="158" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+      <c r="F157" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G157" s="2" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>57</v>
+        <v>311</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F158" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G158" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
+        <v>312</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>311</v>
+        <v>390</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="F159" s="5" t="s">
-        <v>101</v>
+        <v>393</v>
+      </c>
+      <c r="F159" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G159" s="2" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5830,16 +5827,16 @@
         <v>55</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F160" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G160" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="161" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5847,132 +5844,129 @@
         <v>55</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F161" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G161" s="2" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="162" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>392</v>
+        <v>58</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="F162" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G162" s="2" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>58</v>
+        <v>376</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>61</v>
+        <v>340</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F163" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>341</v>
+      </c>
+      <c r="F163" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="D164" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="F164" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="165" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A165" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="F164" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" s="17" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A165" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B165" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="C165" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="F165" s="3" t="s">
+      <c r="B165" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="C165" s="17" t="s">
+        <v>442</v>
+      </c>
+      <c r="F165" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="G165" s="17" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A166" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="F166" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="166" spans="1:7" s="17" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A166" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="B166" s="17" t="s">
-        <v>441</v>
-      </c>
-      <c r="C166" s="17" t="s">
-        <v>442</v>
-      </c>
-      <c r="F166" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="G166" s="17" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A167" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="B167" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="C167" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="D167" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="F167" s="3" t="s">
+    <row r="167" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A167" s="17" t="s">
+        <v>758</v>
+      </c>
+      <c r="B167" s="17" t="s">
+        <v>759</v>
+      </c>
+      <c r="C167" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="D167" s="17" t="s">
+        <v>761</v>
+      </c>
+      <c r="F167" s="19" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="168" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A168" s="17" t="s">
-        <v>758</v>
-      </c>
-      <c r="B168" s="17" t="s">
-        <v>759</v>
-      </c>
-      <c r="C168" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="D168" s="17" t="s">
-        <v>761</v>
-      </c>
-      <c r="F168" s="19" t="s">
-        <v>99</v>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A168" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="F168" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.35">
@@ -5980,13 +5974,13 @@
         <v>357</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="F169" s="5" t="s">
-        <v>101</v>
+        <v>367</v>
+      </c>
+      <c r="F169" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.35">
@@ -5994,24 +5988,27 @@
         <v>357</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F170" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
         <v>357</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>373</v>
       </c>
       <c r="F171" s="4" t="s">
         <v>100</v>
@@ -6022,47 +6019,45 @@
         <v>357</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="D172" s="2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F172" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>357</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="F173" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
+        <v>371</v>
+      </c>
+      <c r="F173" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G173" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
         <v>357</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>364</v>
+        <v>811</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="F174" s="6" t="s">
-        <v>142</v>
-      </c>
+        <v>812</v>
+      </c>
+      <c r="F174" s="6"/>
       <c r="G174" s="2" t="s">
-        <v>374</v>
+        <v>813</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6070,62 +6065,64 @@
         <v>357</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>813</v>
+        <v>365</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>814</v>
-      </c>
-      <c r="F175" s="6"/>
+        <v>372</v>
+      </c>
+      <c r="F175" s="6" t="s">
+        <v>142</v>
+      </c>
       <c r="G175" s="2" t="s">
-        <v>815</v>
-      </c>
-    </row>
-    <row r="176" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A176" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A176" s="17" t="s">
         <v>357</v>
       </c>
-      <c r="B176" s="2" t="s">
-        <v>365</v>
-      </c>
-      <c r="C176" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="F176" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G176" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="177" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A177" s="17" t="s">
-        <v>357</v>
-      </c>
-      <c r="B177" s="17" t="s">
+      <c r="B176" s="17" t="s">
         <v>499</v>
       </c>
-      <c r="C177" s="17" t="s">
+      <c r="C176" s="17" t="s">
         <v>500</v>
       </c>
-      <c r="D177" s="17"/>
-      <c r="E177" s="17"/>
-      <c r="F177" s="20" t="s">
+      <c r="D176" s="17"/>
+      <c r="E176" s="17"/>
+      <c r="F176" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G177" s="17"/>
-    </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G176" s="17"/>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A177" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C177" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F177" s="12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>206</v>
+        <v>519</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F178" s="12" t="s">
-        <v>250</v>
+        <v>520</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="F178" s="14" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6133,16 +6130,16 @@
         <v>63</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>519</v>
+        <v>664</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>520</v>
+        <v>665</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>521</v>
-      </c>
-      <c r="F179" s="14" t="s">
-        <v>400</v>
+        <v>666</v>
+      </c>
+      <c r="F179" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="180" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6150,16 +6147,19 @@
         <v>63</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>664</v>
+        <v>197</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>665</v>
-      </c>
-      <c r="D180" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="F180" s="4" t="s">
-        <v>100</v>
+        <v>198</v>
+      </c>
+      <c r="E180" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F180" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G180" s="2" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="181" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6167,19 +6167,13 @@
         <v>63</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>197</v>
+        <v>326</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="E181" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="F181" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G181" s="2" t="s">
-        <v>339</v>
+        <v>327</v>
+      </c>
+      <c r="F181" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="182" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6187,27 +6181,27 @@
         <v>63</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>326</v>
+        <v>64</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="F182" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="183" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+      <c r="F182" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>64</v>
+        <v>497</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F183" s="4" t="s">
-        <v>100</v>
+        <v>498</v>
+      </c>
+      <c r="F183" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.35">
@@ -6215,13 +6209,16 @@
         <v>63</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>497</v>
+        <v>65</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="F184" s="5" t="s">
-        <v>101</v>
+        <v>68</v>
+      </c>
+      <c r="F184" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G184" s="2" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.35">
@@ -6229,16 +6226,13 @@
         <v>63</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>65</v>
+        <v>562</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F185" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G185" s="2" t="s">
-        <v>345</v>
+        <v>563</v>
+      </c>
+      <c r="F185" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="186" spans="1:7" x14ac:dyDescent="0.35">
@@ -6246,13 +6240,13 @@
         <v>63</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>562</v>
+        <v>764</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="F186" s="5" t="s">
-        <v>101</v>
+        <v>765</v>
+      </c>
+      <c r="F186" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.35">
@@ -6260,58 +6254,64 @@
         <v>63</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="F187" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>770</v>
+        <v>516</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>771</v>
-      </c>
-      <c r="F188" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="189" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>517</v>
+      </c>
+      <c r="F188" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G188" s="2" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>516</v>
+        <v>199</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>517</v>
-      </c>
-      <c r="F189" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G189" s="2" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+      <c r="F189" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>199</v>
+        <v>814</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F190" s="4" t="s">
-        <v>100</v>
+        <v>815</v>
+      </c>
+      <c r="D190" s="2" t="s">
+        <v>816</v>
+      </c>
+      <c r="F190" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G190" s="2" t="s">
+        <v>817</v>
       </c>
     </row>
     <row r="191" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6319,50 +6319,44 @@
         <v>63</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>816</v>
+        <v>66</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>817</v>
+        <v>69</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>818</v>
-      </c>
-      <c r="F191" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G191" s="2" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="192" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>399</v>
+      </c>
+      <c r="F191" s="14" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>66</v>
+        <v>190</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D192" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="F192" s="14" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+      <c r="F192" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>190</v>
+        <v>277</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F193" s="4" t="s">
-        <v>100</v>
+        <v>280</v>
+      </c>
+      <c r="F193" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="194" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6370,10 +6364,10 @@
         <v>63</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F194" s="5" t="s">
         <v>101</v>
@@ -6384,13 +6378,13 @@
         <v>63</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="F195" s="5" t="s">
-        <v>101</v>
+        <v>282</v>
+      </c>
+      <c r="F195" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="196" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6398,100 +6392,103 @@
         <v>63</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>279</v>
+        <v>567</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="F196" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="197" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>568</v>
+      </c>
+      <c r="F196" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>567</v>
+        <v>477</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>568</v>
-      </c>
-      <c r="F197" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
+        <v>476</v>
+      </c>
+      <c r="F197" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>477</v>
+        <v>493</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>476</v>
+        <v>494</v>
       </c>
       <c r="F198" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="199" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A199" s="2" t="s">
+    <row r="199" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A199" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B199" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="C199" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="F199" s="4" t="s">
+      <c r="B199" s="17" t="s">
+        <v>495</v>
+      </c>
+      <c r="C199" s="17" t="s">
+        <v>496</v>
+      </c>
+      <c r="D199" s="17"/>
+      <c r="E199" s="17"/>
+      <c r="F199" s="20" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="200" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A200" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="B200" s="17" t="s">
-        <v>495</v>
-      </c>
-      <c r="C200" s="17" t="s">
-        <v>496</v>
-      </c>
-      <c r="D200" s="17"/>
-      <c r="E200" s="17"/>
-      <c r="F200" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="G200" s="17"/>
-    </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G199" s="17"/>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A200" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="B200" s="2" t="s">
+        <v>797</v>
+      </c>
+      <c r="C200" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="F200" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>799</v>
+        <v>559</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>800</v>
+        <v>560</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>561</v>
       </c>
       <c r="F201" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="202" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>559</v>
+        <v>711</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>560</v>
+        <v>712</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>561</v>
+        <v>710</v>
       </c>
       <c r="F202" s="3" t="s">
         <v>99</v>
@@ -6502,13 +6499,10 @@
         <v>420</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>711</v>
+        <v>428</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>712</v>
-      </c>
-      <c r="D203" s="2" t="s">
-        <v>710</v>
+        <v>429</v>
       </c>
       <c r="F203" s="3" t="s">
         <v>99</v>
@@ -6519,10 +6513,10 @@
         <v>420</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="F204" s="3" t="s">
         <v>99</v>
@@ -6533,10 +6527,10 @@
         <v>420</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>430</v>
+        <v>401</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>431</v>
+        <v>402</v>
       </c>
       <c r="F205" s="3" t="s">
         <v>99</v>
@@ -6547,44 +6541,44 @@
         <v>420</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>401</v>
+        <v>432</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>402</v>
+        <v>433</v>
       </c>
       <c r="F206" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>432</v>
+        <v>613</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>433</v>
+        <v>615</v>
+      </c>
+      <c r="D207" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="E207" s="2" t="s">
+        <v>434</v>
       </c>
       <c r="F207" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="208" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>613</v>
+        <v>434</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>615</v>
-      </c>
-      <c r="D208" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="E208" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F208" s="3" t="s">
         <v>99</v>
@@ -6595,27 +6589,30 @@
         <v>420</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>435</v>
+        <v>424</v>
       </c>
       <c r="F209" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>422</v>
+        <v>530</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="F210" s="3" t="s">
-        <v>99</v>
+        <v>531</v>
+      </c>
+      <c r="F210" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G210" s="2" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="211" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6623,48 +6620,48 @@
         <v>420</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>530</v>
+        <v>480</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="F211" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G211" s="2" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="212" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>481</v>
+      </c>
+      <c r="D211" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="F211" s="3"/>
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>480</v>
+        <v>528</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="D212" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="F212" s="3"/>
+        <v>529</v>
+      </c>
+      <c r="F212" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G212" s="2" t="s">
+        <v>533</v>
+      </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>528</v>
+        <v>503</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>529</v>
-      </c>
-      <c r="F213" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G213" s="2" t="s">
-        <v>533</v>
+        <v>504</v>
+      </c>
+      <c r="E213" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="F213" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.35">
@@ -6672,16 +6669,13 @@
         <v>420</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>504</v>
-      </c>
-      <c r="E214" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="F214" s="3" t="s">
-        <v>99</v>
+        <v>502</v>
+      </c>
+      <c r="F214" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.35">
@@ -6689,10 +6683,10 @@
         <v>420</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>501</v>
+        <v>467</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>502</v>
+        <v>468</v>
       </c>
       <c r="F215" s="5" t="s">
         <v>101</v>
@@ -6703,10 +6697,10 @@
         <v>420</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>467</v>
+        <v>423</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>468</v>
+        <v>425</v>
       </c>
       <c r="F216" s="5" t="s">
         <v>101</v>
@@ -6717,10 +6711,10 @@
         <v>420</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>423</v>
+        <v>469</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>425</v>
+        <v>470</v>
       </c>
       <c r="F217" s="5" t="s">
         <v>101</v>
@@ -6731,106 +6725,106 @@
         <v>420</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>469</v>
+        <v>541</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="F218" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
+        <v>542</v>
+      </c>
+      <c r="F218" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>541</v>
+        <v>426</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>542</v>
-      </c>
-      <c r="F219" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="220" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>427</v>
+      </c>
+      <c r="F219" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G219" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A220" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>426</v>
+        <v>569</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="F220" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G220" s="2" t="s">
-        <v>534</v>
+        <v>570</v>
+      </c>
+      <c r="F220" s="19" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="221" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A221" s="2" t="s">
+      <c r="A221" s="17" t="s">
         <v>420</v>
       </c>
-      <c r="B221" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="C221" s="2" t="s">
-        <v>570</v>
-      </c>
+      <c r="B221" s="17" t="s">
+        <v>491</v>
+      </c>
+      <c r="C221" s="17" t="s">
+        <v>492</v>
+      </c>
+      <c r="D221" s="17"/>
+      <c r="E221" s="17"/>
       <c r="F221" s="19" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="222" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A222" s="17" t="s">
-        <v>420</v>
-      </c>
-      <c r="B222" s="17" t="s">
-        <v>491</v>
-      </c>
-      <c r="C222" s="17" t="s">
-        <v>492</v>
-      </c>
-      <c r="D222" s="17"/>
-      <c r="E222" s="17"/>
-      <c r="F222" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="G222" s="17"/>
+      <c r="G221" s="17"/>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A222" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F222" s="5" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>209</v>
+        <v>304</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="F223" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.35">
+        <v>305</v>
+      </c>
+      <c r="E223" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F223" s="12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>304</v>
+        <v>211</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="E224" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F224" s="12" t="s">
-        <v>250</v>
+        <v>212</v>
+      </c>
+      <c r="F224" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="225" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6838,30 +6832,30 @@
         <v>93</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="F225" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="226" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>214</v>
+      </c>
+      <c r="F225" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G225" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A226" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="F226" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G226" s="2" t="s">
-        <v>346</v>
+        <v>220</v>
+      </c>
+      <c r="F226" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.35">
@@ -6869,10 +6863,10 @@
         <v>93</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>215</v>
+        <v>94</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>220</v>
+        <v>97</v>
       </c>
       <c r="F227" s="5" t="s">
         <v>101</v>
@@ -6883,128 +6877,128 @@
         <v>93</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>94</v>
+        <v>216</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="F228" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
+        <v>217</v>
+      </c>
+      <c r="F228" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="F229" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="230" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A230" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="F229" s="12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A230" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="B230" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="C230" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F230" s="12" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="231" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A231" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="B231" s="17" t="s">
+      <c r="B230" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="C231" s="17" t="s">
+      <c r="C230" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D231" s="17"/>
-      <c r="E231" s="17"/>
-      <c r="F231" s="20" t="s">
+      <c r="D230" s="17"/>
+      <c r="E230" s="17"/>
+      <c r="F230" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G231" s="17"/>
+      <c r="G230" s="17"/>
+    </row>
+    <row r="231" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A231" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B231" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C231" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F231" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G231" s="2" t="s">
+        <v>331</v>
+      </c>
     </row>
     <row r="232" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A232" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>71</v>
+        <v>192</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="F232" s="6" t="s">
-        <v>102</v>
+        <v>142</v>
       </c>
       <c r="G232" s="2" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="233" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A233" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>192</v>
+        <v>745</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>194</v>
+        <v>746</v>
       </c>
       <c r="F233" s="6" t="s">
         <v>142</v>
       </c>
       <c r="G233" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A234" s="2" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A234" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="B234" s="2" t="s">
-        <v>745</v>
-      </c>
-      <c r="C234" s="2" t="s">
-        <v>746</v>
-      </c>
-      <c r="F234" s="6" t="s">
+      <c r="B234" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="C234" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="D234" s="17"/>
+      <c r="E234" s="17"/>
+      <c r="F234" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="G234" s="2" t="s">
-        <v>747</v>
-      </c>
-    </row>
-    <row r="235" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A235" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="B235" s="17" t="s">
-        <v>193</v>
-      </c>
-      <c r="C235" s="17" t="s">
-        <v>195</v>
-      </c>
-      <c r="D235" s="17"/>
-      <c r="E235" s="17"/>
-      <c r="F235" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="G235" s="17" t="s">
+      <c r="G234" s="17" t="s">
         <v>336</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A235" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B235" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="C235" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="F235" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.35">
@@ -7012,13 +7006,13 @@
         <v>73</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>632</v>
+        <v>550</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>633</v>
-      </c>
-      <c r="F236" s="4" t="s">
-        <v>100</v>
+        <v>551</v>
+      </c>
+      <c r="F236" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.35">
@@ -7026,13 +7020,13 @@
         <v>73</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>550</v>
+        <v>74</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>551</v>
-      </c>
-      <c r="F237" s="5" t="s">
-        <v>101</v>
+        <v>82</v>
+      </c>
+      <c r="F237" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.35">
@@ -7040,41 +7034,41 @@
         <v>73</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F238" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
+        <v>83</v>
+      </c>
+      <c r="F238" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A239" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>75</v>
+        <v>554</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>83</v>
+        <v>555</v>
       </c>
       <c r="F239" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="240" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A240" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>554</v>
+        <v>411</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>555</v>
-      </c>
-      <c r="F240" s="5" t="s">
-        <v>101</v>
+        <v>412</v>
+      </c>
+      <c r="F240" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="241" spans="1:6" x14ac:dyDescent="0.35">
@@ -7082,10 +7076,10 @@
         <v>73</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>411</v>
+        <v>677</v>
       </c>
       <c r="C241" s="2" t="s">
-        <v>412</v>
+        <v>678</v>
       </c>
       <c r="F241" s="4" t="s">
         <v>100</v>
@@ -7096,13 +7090,13 @@
         <v>73</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>677</v>
+        <v>552</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="F242" s="4" t="s">
-        <v>100</v>
+        <v>553</v>
+      </c>
+      <c r="F242" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.35">
@@ -7110,13 +7104,13 @@
         <v>73</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>552</v>
+        <v>283</v>
       </c>
       <c r="C243" s="2" t="s">
-        <v>553</v>
-      </c>
-      <c r="F243" s="5" t="s">
-        <v>101</v>
+        <v>284</v>
+      </c>
+      <c r="F243" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.35">
@@ -7124,44 +7118,44 @@
         <v>73</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>284</v>
+        <v>257</v>
       </c>
       <c r="F244" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A245" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="F245" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="246" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>237</v>
+      </c>
+      <c r="E245" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="F245" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="246" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A246" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>236</v>
+        <v>799</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="E246" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="F246" s="5" t="s">
-        <v>101</v>
+        <v>800</v>
+      </c>
+      <c r="F246" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.35">
@@ -7169,13 +7163,13 @@
         <v>73</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>801</v>
+        <v>618</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>802</v>
-      </c>
-      <c r="F247" s="3" t="s">
-        <v>99</v>
+        <v>619</v>
+      </c>
+      <c r="F247" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="248" spans="1:6" x14ac:dyDescent="0.35">
@@ -7183,10 +7177,10 @@
         <v>73</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="F248" s="5" t="s">
         <v>101</v>
@@ -7197,10 +7191,10 @@
         <v>73</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>620</v>
+        <v>232</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>621</v>
+        <v>233</v>
       </c>
       <c r="F249" s="5" t="s">
         <v>101</v>
@@ -7211,10 +7205,10 @@
         <v>73</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="F250" s="5" t="s">
         <v>101</v>
@@ -7225,10 +7219,13 @@
         <v>73</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>228</v>
+        <v>634</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>229</v>
+        <v>635</v>
+      </c>
+      <c r="D251" s="2" t="s">
+        <v>636</v>
       </c>
       <c r="F251" s="5" t="s">
         <v>101</v>
@@ -7239,13 +7236,10 @@
         <v>73</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>634</v>
+        <v>622</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="D252" s="2" t="s">
-        <v>636</v>
+        <v>623</v>
       </c>
       <c r="F252" s="5" t="s">
         <v>101</v>
@@ -7256,13 +7250,13 @@
         <v>73</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>622</v>
+        <v>818</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>623</v>
-      </c>
-      <c r="F253" s="5" t="s">
-        <v>101</v>
+        <v>819</v>
+      </c>
+      <c r="F253" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.35">
@@ -7270,10 +7264,10 @@
         <v>73</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>820</v>
+        <v>708</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>821</v>
+        <v>709</v>
       </c>
       <c r="F254" s="3" t="s">
         <v>99</v>
@@ -7284,10 +7278,10 @@
         <v>73</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>708</v>
+        <v>637</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>709</v>
+        <v>638</v>
       </c>
       <c r="F255" s="3" t="s">
         <v>99</v>
@@ -7298,10 +7292,10 @@
         <v>73</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>637</v>
+        <v>609</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>638</v>
+        <v>610</v>
       </c>
       <c r="F256" s="3" t="s">
         <v>99</v>
@@ -7312,13 +7306,13 @@
         <v>73</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>609</v>
+        <v>589</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="F257" s="3" t="s">
-        <v>99</v>
+        <v>590</v>
+      </c>
+      <c r="F257" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.35">
@@ -7326,44 +7320,44 @@
         <v>73</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>589</v>
+        <v>241</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>590</v>
+        <v>242</v>
       </c>
       <c r="F258" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A259" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>241</v>
+        <v>285</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="F259" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="260" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>286</v>
+      </c>
+      <c r="F259" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="G259" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A260" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>285</v>
+        <v>76</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="F260" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="G260" s="2" t="s">
-        <v>334</v>
+        <v>84</v>
+      </c>
+      <c r="F260" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.35">
@@ -7371,10 +7365,10 @@
         <v>73</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F261" s="5" t="s">
         <v>101</v>
@@ -7385,10 +7379,10 @@
         <v>73</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F262" s="5" t="s">
         <v>101</v>
@@ -7399,13 +7393,13 @@
         <v>73</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F263" s="5" t="s">
-        <v>101</v>
+        <v>87</v>
+      </c>
+      <c r="F263" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.35">
@@ -7413,13 +7407,16 @@
         <v>73</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>79</v>
+        <v>624</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F264" s="4" t="s">
-        <v>100</v>
+        <v>625</v>
+      </c>
+      <c r="D264" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="F264" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.35">
@@ -7427,16 +7424,13 @@
         <v>73</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>624</v>
+        <v>448</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>625</v>
-      </c>
-      <c r="D265" s="2" t="s">
-        <v>626</v>
-      </c>
-      <c r="F265" s="5" t="s">
-        <v>101</v>
+        <v>449</v>
+      </c>
+      <c r="F265" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.35">
@@ -7444,41 +7438,41 @@
         <v>73</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>448</v>
+        <v>478</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>449</v>
+        <v>479</v>
       </c>
       <c r="F266" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A267" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>478</v>
+        <v>639</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="F267" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="268" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>640</v>
+      </c>
+      <c r="F267" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A268" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>639</v>
+        <v>739</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>640</v>
-      </c>
-      <c r="F268" s="5" t="s">
-        <v>101</v>
+        <v>740</v>
+      </c>
+      <c r="F268" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.35">
@@ -7486,10 +7480,10 @@
         <v>73</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>739</v>
+        <v>80</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>740</v>
+        <v>88</v>
       </c>
       <c r="F269" s="3" t="s">
         <v>99</v>
@@ -7500,27 +7494,30 @@
         <v>73</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>80</v>
+        <v>548</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F270" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.35">
+        <v>549</v>
+      </c>
+      <c r="F270" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="271" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A271" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>548</v>
+        <v>293</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>549</v>
-      </c>
-      <c r="F271" s="5" t="s">
-        <v>101</v>
+        <v>294</v>
+      </c>
+      <c r="F271" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G271" s="2" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="272" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -7528,10 +7525,10 @@
         <v>73</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="F272" s="16" t="s">
         <v>303</v>
@@ -7545,10 +7542,10 @@
         <v>73</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>295</v>
+        <v>239</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>296</v>
+        <v>240</v>
       </c>
       <c r="F273" s="16" t="s">
         <v>303</v>
@@ -7557,38 +7554,35 @@
         <v>335</v>
       </c>
     </row>
-    <row r="274" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A274" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="F274" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G274" s="2" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
+        <v>231</v>
+      </c>
+      <c r="E274" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F274" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A275" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>230</v>
+        <v>691</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E275" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="F275" s="4" t="s">
-        <v>100</v>
+        <v>692</v>
+      </c>
+      <c r="F275" s="5" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="276" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7596,58 +7590,58 @@
         <v>73</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>691</v>
+        <v>81</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>692</v>
-      </c>
-      <c r="F276" s="5" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="277" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+      <c r="F276" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="277" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A277" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>81</v>
+        <v>743</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>89</v>
+        <v>744</v>
       </c>
       <c r="F277" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A278" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>743</v>
+        <v>443</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>744</v>
-      </c>
-      <c r="F278" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="279" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>444</v>
+      </c>
+      <c r="F278" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G278" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A279" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>443</v>
+        <v>641</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="F279" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G279" s="2" t="s">
-        <v>377</v>
+        <v>642</v>
+      </c>
+      <c r="F279" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.35">
@@ -7655,44 +7649,44 @@
         <v>73</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>641</v>
+        <v>507</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>642</v>
+        <v>508</v>
       </c>
       <c r="F280" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A281" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>507</v>
+        <v>776</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>508</v>
-      </c>
-      <c r="F281" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="282" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>777</v>
+      </c>
+      <c r="F281" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G281" s="2" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A282" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>776</v>
+        <v>245</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>777</v>
-      </c>
-      <c r="F282" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G282" s="2" t="s">
-        <v>778</v>
+        <v>246</v>
+      </c>
+      <c r="F282" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.35">
@@ -7700,13 +7694,13 @@
         <v>73</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>245</v>
+        <v>298</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="F283" s="14" t="s">
-        <v>258</v>
+        <v>297</v>
+      </c>
+      <c r="F283" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.35">
@@ -7714,13 +7708,13 @@
         <v>73</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>298</v>
+        <v>643</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="F284" s="5" t="s">
-        <v>101</v>
+        <v>644</v>
+      </c>
+      <c r="F284" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.35">
@@ -7728,13 +7722,13 @@
         <v>73</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>643</v>
+        <v>234</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>644</v>
-      </c>
-      <c r="F285" s="4" t="s">
-        <v>100</v>
+        <v>235</v>
+      </c>
+      <c r="F285" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="286" spans="1:7" x14ac:dyDescent="0.35">
@@ -7742,10 +7736,10 @@
         <v>73</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>234</v>
+        <v>627</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>235</v>
+        <v>628</v>
       </c>
       <c r="F286" s="5" t="s">
         <v>101</v>
@@ -7756,13 +7750,13 @@
         <v>73</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>627</v>
+        <v>226</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>628</v>
-      </c>
-      <c r="F287" s="5" t="s">
-        <v>101</v>
+        <v>227</v>
+      </c>
+      <c r="F287" s="12" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.35">
@@ -7770,13 +7764,13 @@
         <v>73</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>226</v>
+        <v>524</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="F288" s="12" t="s">
-        <v>250</v>
+        <v>525</v>
+      </c>
+      <c r="F288" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.35">
@@ -7784,13 +7778,16 @@
         <v>73</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="F289" s="14" t="s">
-        <v>258</v>
+        <v>523</v>
+      </c>
+      <c r="E289" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F289" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.35">
@@ -7798,44 +7795,44 @@
         <v>73</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>522</v>
+        <v>224</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>523</v>
-      </c>
-      <c r="E290" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F290" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A291" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>224</v>
+        <v>645</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="F291" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="292" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>646</v>
+      </c>
+      <c r="F291" s="20" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A292" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>645</v>
+        <v>584</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>646</v>
-      </c>
-      <c r="F292" s="20" t="s">
-        <v>100</v>
+        <v>586</v>
+      </c>
+      <c r="F292" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G292" s="2" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="293" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7843,81 +7840,81 @@
         <v>73</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>586</v>
-      </c>
-      <c r="F293" s="3" t="s">
-        <v>99</v>
+        <v>588</v>
+      </c>
+      <c r="F293" s="16" t="s">
+        <v>303</v>
       </c>
       <c r="G293" s="2" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="294" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A294" s="2" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A294" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B294" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="C294" s="2" t="s">
-        <v>588</v>
-      </c>
-      <c r="F294" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G294" s="2" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="295" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A295" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B295" s="17" t="s">
+      <c r="B294" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="C295" s="17" t="s">
+      <c r="C294" s="17" t="s">
         <v>307</v>
       </c>
-      <c r="D295" s="17"/>
-      <c r="E295" s="17"/>
-      <c r="F295" s="20" t="s">
+      <c r="D294" s="17"/>
+      <c r="E294" s="17"/>
+      <c r="F294" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G295" s="17"/>
-    </row>
-    <row r="296" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="G294" s="17"/>
+    </row>
+    <row r="295" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A295" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B295" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C295" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D295" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F295" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="296" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A296" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>91</v>
+        <v>222</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>92</v>
+        <v>221</v>
       </c>
       <c r="D296" s="2" t="s">
-        <v>315</v>
+        <v>403</v>
       </c>
       <c r="F296" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A297" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>222</v>
+        <v>247</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>221</v>
+        <v>248</v>
       </c>
       <c r="D297" s="2" t="s">
-        <v>403</v>
+        <v>249</v>
       </c>
       <c r="F297" s="5" t="s">
         <v>101</v>
@@ -7928,30 +7925,27 @@
         <v>90</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>247</v>
+        <v>801</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="D298" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="F298" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="299" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>802</v>
+      </c>
+      <c r="F298" s="25" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A299" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>803</v>
+        <v>351</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>804</v>
-      </c>
-      <c r="F299" s="25" t="s">
-        <v>805</v>
+        <v>352</v>
+      </c>
+      <c r="F299" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="300" spans="1:7" x14ac:dyDescent="0.35">
@@ -7959,50 +7953,36 @@
         <v>90</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>351</v>
+        <v>564</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>352</v>
+        <v>565</v>
+      </c>
+      <c r="D300" s="2" t="s">
+        <v>566</v>
       </c>
       <c r="F300" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A301" s="2" t="s">
+    <row r="301" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A301" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B301" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="C301" s="2" t="s">
-        <v>565</v>
-      </c>
-      <c r="D301" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="F301" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="302" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A302" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B302" s="17" t="s">
+      <c r="B301" s="17" t="s">
         <v>291</v>
       </c>
-      <c r="C302" s="17" t="s">
+      <c r="C301" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="D302" s="17" t="s">
+      <c r="D301" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="E302" s="17"/>
-      <c r="F302" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="G302" s="17"/>
+      <c r="E301" s="17"/>
+      <c r="F301" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G301" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Remove remaining unused variables (including unused EIaE-BEEP input data variable), update version to 4.0.5
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A8D342-CF64-453A-BCA2-30B4659ED6AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90689264-523C-45BA-A423-5DBE46709A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1375,9 +1375,6 @@
     <t>Quantization Size for Pollutants</t>
   </si>
   <si>
-    <t>BAU Imported Electricity, BAU Exported Electricity, Imported Electricity Price, BAU Exported Electricity Price</t>
-  </si>
-  <si>
     <t>EVCC</t>
   </si>
   <si>
@@ -2528,6 +2525,9 @@
   </si>
   <si>
     <t>You are using a different model start year than the US EPS (this file should note which vintages are for historical years rather than modeled years)</t>
+  </si>
+  <si>
+    <t>BAU Imported Electricity, BAU Exported Electricity, Imported Electricity Price</t>
   </si>
 </sst>
 </file>
@@ -3380,10 +3380,10 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>538</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>539</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -3391,7 +3391,7 @@
         <v>99</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -3399,16 +3399,16 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>535</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>536</v>
       </c>
       <c r="F3" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -3416,10 +3416,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>461</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>462</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>101</v>
@@ -3430,16 +3430,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>581</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>582</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>142</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -3506,10 +3506,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>715</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>716</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>99</v>
@@ -3537,10 +3537,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>611</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>612</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>99</v>
@@ -3582,16 +3582,16 @@
         <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>804</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>805</v>
       </c>
       <c r="F15" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -3605,7 +3605,7 @@
         <v>168</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>100</v>
@@ -3686,10 +3686,10 @@
         <v>9</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>484</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>101</v>
@@ -3700,10 +3700,10 @@
         <v>9</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>772</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>773</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>101</v>
@@ -3807,10 +3807,10 @@
         <v>9</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>450</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>451</v>
       </c>
       <c r="F30" s="16" t="s">
         <v>303</v>
@@ -3824,10 +3824,10 @@
         <v>9</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>455</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>456</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>100</v>
@@ -3838,10 +3838,10 @@
         <v>9</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>505</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>506</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>101</v>
@@ -3866,10 +3866,10 @@
         <v>9</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>487</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>488</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>100</v>
@@ -3880,10 +3880,10 @@
         <v>9</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>459</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>460</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>11</v>
@@ -3897,10 +3897,10 @@
         <v>9</v>
       </c>
       <c r="B36" s="17" t="s">
+        <v>456</v>
+      </c>
+      <c r="C36" s="17" t="s">
         <v>457</v>
-      </c>
-      <c r="C36" s="17" t="s">
-        <v>458</v>
       </c>
       <c r="D36" s="17"/>
       <c r="E36" s="17" t="s">
@@ -3916,10 +3916,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>616</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>617</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>99</v>
@@ -3930,13 +3930,13 @@
         <v>36</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>694</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>695</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>696</v>
       </c>
       <c r="F38" s="5" t="s">
         <v>101</v>
@@ -3947,10 +3947,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>698</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>699</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>100</v>
@@ -3967,7 +3967,7 @@
         <v>417</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="F40" s="5" t="s">
         <v>101</v>
@@ -3984,7 +3984,7 @@
         <v>410</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="F41" s="5" t="s">
         <v>101</v>
@@ -3995,10 +3995,10 @@
         <v>36</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>687</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>688</v>
       </c>
       <c r="F42" s="5" t="s">
         <v>101</v>
@@ -4009,19 +4009,19 @@
         <v>36</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>806</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>807</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="D43" s="2" t="s">
         <v>808</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>809</v>
       </c>
       <c r="F43" s="21" t="s">
         <v>303</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -4029,10 +4029,10 @@
         <v>36</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>701</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>702</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>100</v>
@@ -4043,10 +4043,10 @@
         <v>36</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="F45" s="20" t="s">
         <v>100</v>
@@ -4087,7 +4087,7 @@
     </row>
     <row r="48" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="17" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B48" s="17" t="s">
         <v>445</v>
@@ -4101,7 +4101,7 @@
         <v>142</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -4126,16 +4126,16 @@
         <v>413</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>556</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>557</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -4160,16 +4160,16 @@
         <v>413</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>826</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>827</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -4211,16 +4211,16 @@
         <v>413</v>
       </c>
       <c r="B55" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>718</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>719</v>
       </c>
       <c r="F55" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -4228,16 +4228,16 @@
         <v>413</v>
       </c>
       <c r="B56" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>509</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>510</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -4254,7 +4254,7 @@
         <v>180</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -4262,16 +4262,16 @@
         <v>413</v>
       </c>
       <c r="B58" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>571</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>572</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -4296,16 +4296,16 @@
         <v>413</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -4327,19 +4327,19 @@
         <v>413</v>
       </c>
       <c r="B62" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="C62" s="2" t="s">
-        <v>465</v>
-      </c>
       <c r="D62" s="2" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="44" thickBot="1" x14ac:dyDescent="0.4">
@@ -4347,10 +4347,10 @@
         <v>413</v>
       </c>
       <c r="B63" s="17" t="s">
+        <v>828</v>
+      </c>
+      <c r="C63" s="17" t="s">
         <v>829</v>
-      </c>
-      <c r="C63" s="17" t="s">
-        <v>830</v>
       </c>
       <c r="D63" s="17"/>
       <c r="E63" s="17"/>
@@ -4358,7 +4358,7 @@
         <v>303</v>
       </c>
       <c r="G63" s="17" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
@@ -4408,10 +4408,10 @@
         <v>38</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>545</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>546</v>
       </c>
       <c r="F67" s="4" t="s">
         <v>100</v>
@@ -4441,10 +4441,10 @@
         <v>43</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>100</v>
@@ -4455,10 +4455,10 @@
         <v>43</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>100</v>
@@ -4469,13 +4469,13 @@
         <v>43</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="C71" s="2" t="s">
         <v>655</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="D71" s="2" t="s">
         <v>656</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>657</v>
       </c>
       <c r="F71" s="5" t="s">
         <v>101</v>
@@ -4489,10 +4489,10 @@
         <v>181</v>
       </c>
       <c r="C72" s="2" t="s">
+        <v>721</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>722</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>723</v>
       </c>
       <c r="F72" s="4" t="s">
         <v>100</v>
@@ -4517,10 +4517,10 @@
         <v>43</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F74" s="5" t="s">
         <v>101</v>
@@ -4531,13 +4531,13 @@
         <v>43</v>
       </c>
       <c r="B75" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="C75" s="2" t="s">
         <v>684</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="D75" s="2" t="s">
         <v>685</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>686</v>
       </c>
       <c r="F75" s="4" t="s">
         <v>100</v>
@@ -4565,13 +4565,13 @@
         <v>43</v>
       </c>
       <c r="B77" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="C77" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="C77" s="2" t="s">
-        <v>595</v>
-      </c>
       <c r="D77" s="2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="F77" s="12" t="s">
         <v>250</v>
@@ -4613,16 +4613,16 @@
         <v>43</v>
       </c>
       <c r="B80" s="2" t="s">
+        <v>751</v>
+      </c>
+      <c r="C80" s="2" t="s">
         <v>752</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>753</v>
       </c>
       <c r="F80" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.35">
@@ -4630,10 +4630,10 @@
         <v>43</v>
       </c>
       <c r="B81" s="2" t="s">
+        <v>773</v>
+      </c>
+      <c r="C81" s="2" t="s">
         <v>774</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>775</v>
       </c>
       <c r="F81" s="5" t="s">
         <v>101</v>
@@ -4644,10 +4644,10 @@
         <v>43</v>
       </c>
       <c r="B82" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>689</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>690</v>
       </c>
       <c r="F82" s="3" t="s">
         <v>99</v>
@@ -4658,13 +4658,13 @@
         <v>43</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>674</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="D83" s="2" t="s">
         <v>675</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>676</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>203</v>
@@ -4678,10 +4678,10 @@
         <v>43</v>
       </c>
       <c r="B84" s="2" t="s">
+        <v>823</v>
+      </c>
+      <c r="C84" s="2" t="s">
         <v>824</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>825</v>
       </c>
       <c r="F84" s="3" t="s">
         <v>99</v>
@@ -4706,10 +4706,10 @@
         <v>43</v>
       </c>
       <c r="B86" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>658</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>659</v>
       </c>
       <c r="F86" s="5" t="s">
         <v>101</v>
@@ -4726,7 +4726,7 @@
         <v>52</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="F87" s="5" t="s">
         <v>101</v>
@@ -4737,10 +4737,10 @@
         <v>43</v>
       </c>
       <c r="B88" s="2" t="s">
+        <v>725</v>
+      </c>
+      <c r="C88" s="2" t="s">
         <v>726</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>727</v>
       </c>
       <c r="F88" s="5" t="s">
         <v>101</v>
@@ -4751,16 +4751,16 @@
         <v>43</v>
       </c>
       <c r="B89" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="C89" s="2" t="s">
         <v>513</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>514</v>
       </c>
       <c r="F89" s="6" t="s">
         <v>102</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.35">
@@ -4768,10 +4768,10 @@
         <v>43</v>
       </c>
       <c r="B90" s="2" t="s">
+        <v>786</v>
+      </c>
+      <c r="C90" s="2" t="s">
         <v>787</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>788</v>
       </c>
       <c r="F90" s="5" t="s">
         <v>101</v>
@@ -4782,13 +4782,13 @@
         <v>43</v>
       </c>
       <c r="B91" s="2" t="s">
+        <v>727</v>
+      </c>
+      <c r="C91" s="2" t="s">
         <v>728</v>
       </c>
-      <c r="C91" s="2" t="s">
-        <v>729</v>
-      </c>
       <c r="D91" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="F91" s="5" t="s">
         <v>101</v>
@@ -4799,10 +4799,10 @@
         <v>43</v>
       </c>
       <c r="B92" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="C92" s="2" t="s">
         <v>647</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>648</v>
       </c>
       <c r="F92" s="5" t="s">
         <v>101</v>
@@ -4827,10 +4827,10 @@
         <v>43</v>
       </c>
       <c r="B94" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="C94" s="2" t="s">
         <v>741</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>742</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>100</v>
@@ -4847,7 +4847,7 @@
         <v>171</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="F95" s="3" t="s">
         <v>99</v>
@@ -4875,19 +4875,19 @@
         <v>43</v>
       </c>
       <c r="B97" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="C97" s="2" t="s">
         <v>660</v>
       </c>
-      <c r="C97" s="2" t="s">
-        <v>661</v>
-      </c>
       <c r="D97" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="F97" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>43</v>
       </c>
@@ -4898,7 +4898,7 @@
         <v>170</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>447</v>
+        <v>831</v>
       </c>
       <c r="F98" s="3" t="s">
         <v>99</v>
@@ -4909,13 +4909,13 @@
         <v>43</v>
       </c>
       <c r="B99" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="C99" s="2" t="s">
         <v>671</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="D99" s="2" t="s">
         <v>672</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>673</v>
       </c>
       <c r="F99" s="4" t="s">
         <v>100</v>
@@ -4926,10 +4926,10 @@
         <v>43</v>
       </c>
       <c r="B100" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="C100" s="2" t="s">
         <v>822</v>
-      </c>
-      <c r="C100" s="2" t="s">
-        <v>823</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>99</v>
@@ -4940,10 +4940,10 @@
         <v>43</v>
       </c>
       <c r="B101" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="C101" s="2" t="s">
         <v>731</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>732</v>
       </c>
       <c r="F101" s="5" t="s">
         <v>101</v>
@@ -4954,13 +4954,13 @@
         <v>43</v>
       </c>
       <c r="B102" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="C102" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="C102" s="2" t="s">
-        <v>490</v>
-      </c>
       <c r="D102" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="F102" s="3" t="s">
         <v>99</v>
@@ -4988,10 +4988,10 @@
         <v>43</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="F104" s="5" t="s">
         <v>101</v>
@@ -4999,10 +4999,10 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B105" s="2" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="F105" s="5" t="s">
         <v>101</v>
@@ -5013,10 +5013,10 @@
         <v>43</v>
       </c>
       <c r="B106" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="C106" s="2" t="s">
         <v>713</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>714</v>
       </c>
       <c r="F106" s="4" t="s">
         <v>100</v>
@@ -5027,10 +5027,10 @@
         <v>43</v>
       </c>
       <c r="B107" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="C107" s="2" t="s">
         <v>733</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>734</v>
       </c>
       <c r="F107" s="4" t="s">
         <v>100</v>
@@ -5041,10 +5041,10 @@
         <v>43</v>
       </c>
       <c r="B108" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="C108" s="2" t="s">
         <v>592</v>
-      </c>
-      <c r="C108" s="2" t="s">
-        <v>593</v>
       </c>
       <c r="F108" s="4" t="s">
         <v>100</v>
@@ -5055,10 +5055,10 @@
         <v>43</v>
       </c>
       <c r="B109" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="C109" s="2" t="s">
         <v>605</v>
-      </c>
-      <c r="C109" s="2" t="s">
-        <v>606</v>
       </c>
       <c r="F109" s="3" t="s">
         <v>99</v>
@@ -5069,10 +5069,10 @@
         <v>43</v>
       </c>
       <c r="B110" s="2" t="s">
+        <v>749</v>
+      </c>
+      <c r="C110" s="2" t="s">
         <v>750</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>751</v>
       </c>
       <c r="F110" s="3" t="s">
         <v>99</v>
@@ -5083,10 +5083,10 @@
         <v>43</v>
       </c>
       <c r="B111" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="C111" s="2" t="s">
         <v>596</v>
-      </c>
-      <c r="C111" s="2" t="s">
-        <v>597</v>
       </c>
       <c r="F111" s="4" t="s">
         <v>100</v>
@@ -5097,10 +5097,10 @@
         <v>43</v>
       </c>
       <c r="B112" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="C112" s="2" t="s">
         <v>662</v>
-      </c>
-      <c r="C112" s="2" t="s">
-        <v>663</v>
       </c>
       <c r="F112" s="4" t="s">
         <v>100</v>
@@ -5156,16 +5156,16 @@
         <v>43</v>
       </c>
       <c r="B116" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="C116" s="2" t="s">
         <v>755</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>756</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>102</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5173,13 +5173,13 @@
         <v>43</v>
       </c>
       <c r="B117" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="C117" s="2" t="s">
         <v>748</v>
       </c>
-      <c r="C117" s="2" t="s">
-        <v>749</v>
-      </c>
       <c r="D117" s="2" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="F117" s="5" t="s">
         <v>101</v>
@@ -5190,13 +5190,13 @@
         <v>43</v>
       </c>
       <c r="B118" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="C118" s="2" t="s">
         <v>669</v>
       </c>
-      <c r="C118" s="2" t="s">
-        <v>670</v>
-      </c>
       <c r="D118" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="F118" s="14" t="s">
         <v>258</v>
@@ -5221,10 +5221,10 @@
         <v>43</v>
       </c>
       <c r="B120" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="C120" s="2" t="s">
         <v>579</v>
-      </c>
-      <c r="C120" s="2" t="s">
-        <v>580</v>
       </c>
       <c r="F120" s="4" t="s">
         <v>100</v>
@@ -5252,13 +5252,13 @@
         <v>43</v>
       </c>
       <c r="B122" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="C122" s="2" t="s">
         <v>681</v>
       </c>
-      <c r="C122" s="2" t="s">
+      <c r="D122" s="2" t="s">
         <v>682</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>683</v>
       </c>
       <c r="F122" s="5" t="s">
         <v>101</v>
@@ -5269,13 +5269,13 @@
         <v>43</v>
       </c>
       <c r="B123" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="C123" s="2" t="s">
         <v>600</v>
       </c>
-      <c r="C123" s="2" t="s">
-        <v>601</v>
-      </c>
       <c r="D123" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F123" s="3" t="s">
         <v>99</v>
@@ -5283,10 +5283,10 @@
     </row>
     <row r="124" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B124" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="C124" s="2" t="s">
         <v>667</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>668</v>
       </c>
       <c r="F124" s="14" t="s">
         <v>258</v>
@@ -5297,13 +5297,13 @@
         <v>43</v>
       </c>
       <c r="B125" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="C125" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="C125" s="2" t="s">
+      <c r="D125" s="2" t="s">
         <v>453</v>
-      </c>
-      <c r="D125" s="2" t="s">
-        <v>454</v>
       </c>
       <c r="F125" s="4" t="s">
         <v>100</v>
@@ -5314,10 +5314,10 @@
         <v>43</v>
       </c>
       <c r="B126" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="C126" s="2" t="s">
         <v>679</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>680</v>
       </c>
       <c r="F126" s="14" t="s">
         <v>258</v>
@@ -5328,10 +5328,10 @@
         <v>43</v>
       </c>
       <c r="B127" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="C127" s="2" t="s">
         <v>651</v>
-      </c>
-      <c r="C127" s="2" t="s">
-        <v>652</v>
       </c>
       <c r="F127" s="4" t="s">
         <v>100</v>
@@ -5342,10 +5342,10 @@
         <v>43</v>
       </c>
       <c r="B128" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="C128" s="2" t="s">
         <v>653</v>
-      </c>
-      <c r="C128" s="2" t="s">
-        <v>654</v>
       </c>
       <c r="F128" s="4" t="s">
         <v>100</v>
@@ -5356,10 +5356,10 @@
         <v>43</v>
       </c>
       <c r="B129" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="C129" s="2" t="s">
         <v>574</v>
-      </c>
-      <c r="C129" s="2" t="s">
-        <v>575</v>
       </c>
       <c r="F129" s="4" t="s">
         <v>100</v>
@@ -5370,10 +5370,10 @@
         <v>43</v>
       </c>
       <c r="B130" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="C130" s="2" t="s">
         <v>649</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>650</v>
       </c>
       <c r="F130" s="3" t="s">
         <v>99</v>
@@ -5384,13 +5384,13 @@
         <v>43</v>
       </c>
       <c r="B131" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="C131" s="2" t="s">
         <v>598</v>
       </c>
-      <c r="C131" s="2" t="s">
-        <v>599</v>
-      </c>
       <c r="E131" s="2" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="F131" s="3" t="s">
         <v>99</v>
@@ -5401,13 +5401,13 @@
         <v>43</v>
       </c>
       <c r="B132" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="C132" s="2" t="s">
         <v>736</v>
       </c>
-      <c r="C132" s="2" t="s">
+      <c r="D132" s="2" t="s">
         <v>737</v>
-      </c>
-      <c r="D132" s="2" t="s">
-        <v>738</v>
       </c>
       <c r="F132" s="3" t="s">
         <v>99</v>
@@ -5418,10 +5418,10 @@
         <v>43</v>
       </c>
       <c r="B133" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="C133" s="2" t="s">
         <v>820</v>
-      </c>
-      <c r="C133" s="2" t="s">
-        <v>821</v>
       </c>
       <c r="F133" s="4" t="s">
         <v>100</v>
@@ -5432,10 +5432,10 @@
         <v>43</v>
       </c>
       <c r="B134" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="C134" s="2" t="s">
         <v>706</v>
-      </c>
-      <c r="C134" s="2" t="s">
-        <v>707</v>
       </c>
       <c r="F134" s="5" t="s">
         <v>101</v>
@@ -5473,7 +5473,7 @@
         <v>270</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="F136" s="4" t="s">
         <v>100</v>
@@ -5490,7 +5490,7 @@
         <v>274</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F137" s="4" t="s">
         <v>100</v>
@@ -5574,10 +5574,10 @@
         <v>55</v>
       </c>
       <c r="B143" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="C143" s="2" t="s">
         <v>471</v>
-      </c>
-      <c r="C143" s="2" t="s">
-        <v>472</v>
       </c>
       <c r="F143" s="3" t="s">
         <v>99</v>
@@ -5588,10 +5588,10 @@
         <v>55</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="F144" s="5" t="s">
         <v>101</v>
@@ -5602,10 +5602,10 @@
         <v>55</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="F145" s="5" t="s">
         <v>101</v>
@@ -5616,10 +5616,10 @@
         <v>55</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="F146" s="5" t="s">
         <v>101</v>
@@ -5630,13 +5630,13 @@
         <v>55</v>
       </c>
       <c r="B147" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="C147" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="C147" s="2" t="s">
+      <c r="D147" s="2" t="s">
         <v>474</v>
-      </c>
-      <c r="D147" s="2" t="s">
-        <v>475</v>
       </c>
       <c r="F147" s="3" t="s">
         <v>99</v>
@@ -5692,10 +5692,10 @@
         <v>55</v>
       </c>
       <c r="B151" s="2" t="s">
+        <v>779</v>
+      </c>
+      <c r="C151" s="2" t="s">
         <v>780</v>
-      </c>
-      <c r="C151" s="2" t="s">
-        <v>781</v>
       </c>
       <c r="F151" s="5" t="s">
         <v>101</v>
@@ -5706,10 +5706,10 @@
         <v>55</v>
       </c>
       <c r="B152" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="C152" s="2" t="s">
         <v>629</v>
-      </c>
-      <c r="C152" s="2" t="s">
-        <v>630</v>
       </c>
       <c r="F152" s="5" t="s">
         <v>101</v>
@@ -5720,13 +5720,13 @@
         <v>55</v>
       </c>
       <c r="B153" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="E153" s="2" t="s">
         <v>526</v>
-      </c>
-      <c r="C153" s="2" t="s">
-        <v>796</v>
-      </c>
-      <c r="E153" s="2" t="s">
-        <v>527</v>
       </c>
       <c r="F153" s="5" t="s">
         <v>101</v>
@@ -5737,10 +5737,10 @@
         <v>55</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="F154" s="5" t="s">
         <v>101</v>
@@ -5751,10 +5751,10 @@
         <v>55</v>
       </c>
       <c r="B155" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="C155" s="2" t="s">
         <v>543</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>544</v>
       </c>
       <c r="F155" s="3" t="s">
         <v>99</v>
@@ -5765,10 +5765,10 @@
         <v>55</v>
       </c>
       <c r="B156" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="C156" s="2" t="s">
         <v>607</v>
-      </c>
-      <c r="C156" s="2" t="s">
-        <v>608</v>
       </c>
       <c r="F156" s="4" t="s">
         <v>100</v>
@@ -5940,16 +5940,16 @@
     </row>
     <row r="167" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A167" s="17" t="s">
+        <v>757</v>
+      </c>
+      <c r="B167" s="17" t="s">
         <v>758</v>
       </c>
-      <c r="B167" s="17" t="s">
+      <c r="C167" s="17" t="s">
         <v>759</v>
       </c>
-      <c r="C167" s="17" t="s">
+      <c r="D167" s="17" t="s">
         <v>760</v>
-      </c>
-      <c r="D167" s="17" t="s">
-        <v>761</v>
       </c>
       <c r="F167" s="19" t="s">
         <v>99</v>
@@ -6050,14 +6050,14 @@
         <v>357</v>
       </c>
       <c r="B174" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="C174" s="2" t="s">
         <v>811</v>
-      </c>
-      <c r="C174" s="2" t="s">
-        <v>812</v>
       </c>
       <c r="F174" s="6"/>
       <c r="G174" s="2" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6082,10 +6082,10 @@
         <v>357</v>
       </c>
       <c r="B176" s="17" t="s">
+        <v>498</v>
+      </c>
+      <c r="C176" s="17" t="s">
         <v>499</v>
-      </c>
-      <c r="C176" s="17" t="s">
-        <v>500</v>
       </c>
       <c r="D176" s="17"/>
       <c r="E176" s="17"/>
@@ -6113,13 +6113,13 @@
         <v>63</v>
       </c>
       <c r="B178" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="C178" s="2" t="s">
         <v>519</v>
       </c>
-      <c r="C178" s="2" t="s">
+      <c r="D178" s="2" t="s">
         <v>520</v>
-      </c>
-      <c r="D178" s="2" t="s">
-        <v>521</v>
       </c>
       <c r="F178" s="14" t="s">
         <v>400</v>
@@ -6130,13 +6130,13 @@
         <v>63</v>
       </c>
       <c r="B179" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="C179" s="2" t="s">
         <v>664</v>
       </c>
-      <c r="C179" s="2" t="s">
+      <c r="D179" s="2" t="s">
         <v>665</v>
-      </c>
-      <c r="D179" s="2" t="s">
-        <v>666</v>
       </c>
       <c r="F179" s="4" t="s">
         <v>100</v>
@@ -6195,10 +6195,10 @@
         <v>63</v>
       </c>
       <c r="B183" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C183" s="2" t="s">
         <v>497</v>
-      </c>
-      <c r="C183" s="2" t="s">
-        <v>498</v>
       </c>
       <c r="F183" s="5" t="s">
         <v>101</v>
@@ -6226,10 +6226,10 @@
         <v>63</v>
       </c>
       <c r="B185" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="C185" s="2" t="s">
         <v>562</v>
-      </c>
-      <c r="C185" s="2" t="s">
-        <v>563</v>
       </c>
       <c r="F185" s="5" t="s">
         <v>101</v>
@@ -6240,10 +6240,10 @@
         <v>63</v>
       </c>
       <c r="B186" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="C186" s="2" t="s">
         <v>764</v>
-      </c>
-      <c r="C186" s="2" t="s">
-        <v>765</v>
       </c>
       <c r="F186" s="4" t="s">
         <v>100</v>
@@ -6254,10 +6254,10 @@
         <v>63</v>
       </c>
       <c r="B187" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="C187" s="2" t="s">
         <v>770</v>
-      </c>
-      <c r="C187" s="2" t="s">
-        <v>771</v>
       </c>
       <c r="F187" s="4" t="s">
         <v>100</v>
@@ -6268,16 +6268,16 @@
         <v>63</v>
       </c>
       <c r="B188" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="C188" s="2" t="s">
         <v>516</v>
-      </c>
-      <c r="C188" s="2" t="s">
-        <v>517</v>
       </c>
       <c r="F188" s="6" t="s">
         <v>102</v>
       </c>
       <c r="G188" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.35">
@@ -6299,19 +6299,19 @@
         <v>63</v>
       </c>
       <c r="B190" s="2" t="s">
+        <v>813</v>
+      </c>
+      <c r="C190" s="2" t="s">
         <v>814</v>
       </c>
-      <c r="C190" s="2" t="s">
+      <c r="D190" s="2" t="s">
         <v>815</v>
-      </c>
-      <c r="D190" s="2" t="s">
-        <v>816</v>
       </c>
       <c r="F190" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G190" s="2" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="191" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6392,10 +6392,10 @@
         <v>63</v>
       </c>
       <c r="B196" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="C196" s="2" t="s">
         <v>567</v>
-      </c>
-      <c r="C196" s="2" t="s">
-        <v>568</v>
       </c>
       <c r="F196" s="5" t="s">
         <v>101</v>
@@ -6406,10 +6406,10 @@
         <v>63</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="F197" s="4" t="s">
         <v>100</v>
@@ -6420,10 +6420,10 @@
         <v>63</v>
       </c>
       <c r="B198" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="C198" s="2" t="s">
         <v>493</v>
-      </c>
-      <c r="C198" s="2" t="s">
-        <v>494</v>
       </c>
       <c r="F198" s="4" t="s">
         <v>100</v>
@@ -6434,10 +6434,10 @@
         <v>63</v>
       </c>
       <c r="B199" s="17" t="s">
+        <v>494</v>
+      </c>
+      <c r="C199" s="17" t="s">
         <v>495</v>
-      </c>
-      <c r="C199" s="17" t="s">
-        <v>496</v>
       </c>
       <c r="D199" s="17"/>
       <c r="E199" s="17"/>
@@ -6451,10 +6451,10 @@
         <v>420</v>
       </c>
       <c r="B200" s="2" t="s">
+        <v>796</v>
+      </c>
+      <c r="C200" s="2" t="s">
         <v>797</v>
-      </c>
-      <c r="C200" s="2" t="s">
-        <v>798</v>
       </c>
       <c r="F200" s="3" t="s">
         <v>99</v>
@@ -6465,13 +6465,13 @@
         <v>420</v>
       </c>
       <c r="B201" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="C201" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="C201" s="2" t="s">
+      <c r="D201" s="2" t="s">
         <v>560</v>
-      </c>
-      <c r="D201" s="2" t="s">
-        <v>561</v>
       </c>
       <c r="F201" s="3" t="s">
         <v>99</v>
@@ -6482,13 +6482,13 @@
         <v>420</v>
       </c>
       <c r="B202" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="C202" s="2" t="s">
         <v>711</v>
       </c>
-      <c r="C202" s="2" t="s">
-        <v>712</v>
-      </c>
       <c r="D202" s="2" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F202" s="3" t="s">
         <v>99</v>
@@ -6555,13 +6555,13 @@
         <v>420</v>
       </c>
       <c r="B207" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="D207" s="2" t="s">
         <v>613</v>
-      </c>
-      <c r="C207" s="2" t="s">
-        <v>615</v>
-      </c>
-      <c r="D207" s="2" t="s">
-        <v>614</v>
       </c>
       <c r="E207" s="2" t="s">
         <v>434</v>
@@ -6603,16 +6603,16 @@
         <v>420</v>
       </c>
       <c r="B210" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="C210" s="2" t="s">
         <v>530</v>
-      </c>
-      <c r="C210" s="2" t="s">
-        <v>531</v>
       </c>
       <c r="F210" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G210" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="211" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6620,13 +6620,13 @@
         <v>420</v>
       </c>
       <c r="B211" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="C211" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="C211" s="2" t="s">
+      <c r="D211" s="2" t="s">
         <v>481</v>
-      </c>
-      <c r="D211" s="2" t="s">
-        <v>482</v>
       </c>
       <c r="F211" s="3"/>
     </row>
@@ -6635,16 +6635,16 @@
         <v>420</v>
       </c>
       <c r="B212" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="C212" s="2" t="s">
         <v>528</v>
-      </c>
-      <c r="C212" s="2" t="s">
-        <v>529</v>
       </c>
       <c r="F212" s="6" t="s">
         <v>142</v>
       </c>
       <c r="G212" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.35">
@@ -6652,10 +6652,10 @@
         <v>420</v>
       </c>
       <c r="B213" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C213" s="2" t="s">
         <v>503</v>
-      </c>
-      <c r="C213" s="2" t="s">
-        <v>504</v>
       </c>
       <c r="E213" s="2" t="s">
         <v>422</v>
@@ -6669,10 +6669,10 @@
         <v>420</v>
       </c>
       <c r="B214" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C214" s="2" t="s">
         <v>501</v>
-      </c>
-      <c r="C214" s="2" t="s">
-        <v>502</v>
       </c>
       <c r="F214" s="5" t="s">
         <v>101</v>
@@ -6683,10 +6683,10 @@
         <v>420</v>
       </c>
       <c r="B215" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="C215" s="2" t="s">
         <v>467</v>
-      </c>
-      <c r="C215" s="2" t="s">
-        <v>468</v>
       </c>
       <c r="F215" s="5" t="s">
         <v>101</v>
@@ -6711,10 +6711,10 @@
         <v>420</v>
       </c>
       <c r="B217" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="C217" s="2" t="s">
         <v>469</v>
-      </c>
-      <c r="C217" s="2" t="s">
-        <v>470</v>
       </c>
       <c r="F217" s="5" t="s">
         <v>101</v>
@@ -6725,10 +6725,10 @@
         <v>420</v>
       </c>
       <c r="B218" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="C218" s="2" t="s">
         <v>541</v>
-      </c>
-      <c r="C218" s="2" t="s">
-        <v>542</v>
       </c>
       <c r="F218" s="3" t="s">
         <v>99</v>
@@ -6748,7 +6748,7 @@
         <v>303</v>
       </c>
       <c r="G219" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="220" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6756,10 +6756,10 @@
         <v>420</v>
       </c>
       <c r="B220" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="C220" s="2" t="s">
         <v>569</v>
-      </c>
-      <c r="C220" s="2" t="s">
-        <v>570</v>
       </c>
       <c r="F220" s="19" t="s">
         <v>99</v>
@@ -6770,10 +6770,10 @@
         <v>420</v>
       </c>
       <c r="B221" s="17" t="s">
+        <v>490</v>
+      </c>
+      <c r="C221" s="17" t="s">
         <v>491</v>
-      </c>
-      <c r="C221" s="17" t="s">
-        <v>492</v>
       </c>
       <c r="D221" s="17"/>
       <c r="E221" s="17"/>
@@ -6948,7 +6948,7 @@
         <v>142</v>
       </c>
       <c r="G232" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.35">
@@ -6956,16 +6956,16 @@
         <v>70</v>
       </c>
       <c r="B233" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="C233" s="2" t="s">
         <v>745</v>
-      </c>
-      <c r="C233" s="2" t="s">
-        <v>746</v>
       </c>
       <c r="F233" s="6" t="s">
         <v>142</v>
       </c>
       <c r="G233" s="2" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="234" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -6992,10 +6992,10 @@
         <v>73</v>
       </c>
       <c r="B235" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="C235" s="2" t="s">
         <v>632</v>
-      </c>
-      <c r="C235" s="2" t="s">
-        <v>633</v>
       </c>
       <c r="F235" s="4" t="s">
         <v>100</v>
@@ -7006,10 +7006,10 @@
         <v>73</v>
       </c>
       <c r="B236" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C236" s="2" t="s">
         <v>550</v>
-      </c>
-      <c r="C236" s="2" t="s">
-        <v>551</v>
       </c>
       <c r="F236" s="5" t="s">
         <v>101</v>
@@ -7048,10 +7048,10 @@
         <v>73</v>
       </c>
       <c r="B239" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="C239" s="2" t="s">
         <v>554</v>
-      </c>
-      <c r="C239" s="2" t="s">
-        <v>555</v>
       </c>
       <c r="F239" s="5" t="s">
         <v>101</v>
@@ -7076,10 +7076,10 @@
         <v>73</v>
       </c>
       <c r="B241" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="C241" s="2" t="s">
         <v>677</v>
-      </c>
-      <c r="C241" s="2" t="s">
-        <v>678</v>
       </c>
       <c r="F241" s="4" t="s">
         <v>100</v>
@@ -7090,10 +7090,10 @@
         <v>73</v>
       </c>
       <c r="B242" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="C242" s="2" t="s">
         <v>552</v>
-      </c>
-      <c r="C242" s="2" t="s">
-        <v>553</v>
       </c>
       <c r="F242" s="5" t="s">
         <v>101</v>
@@ -7149,10 +7149,10 @@
         <v>73</v>
       </c>
       <c r="B246" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="C246" s="2" t="s">
         <v>799</v>
-      </c>
-      <c r="C246" s="2" t="s">
-        <v>800</v>
       </c>
       <c r="F246" s="3" t="s">
         <v>99</v>
@@ -7163,10 +7163,10 @@
         <v>73</v>
       </c>
       <c r="B247" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="C247" s="2" t="s">
         <v>618</v>
-      </c>
-      <c r="C247" s="2" t="s">
-        <v>619</v>
       </c>
       <c r="F247" s="5" t="s">
         <v>101</v>
@@ -7177,10 +7177,10 @@
         <v>73</v>
       </c>
       <c r="B248" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="C248" s="2" t="s">
         <v>620</v>
-      </c>
-      <c r="C248" s="2" t="s">
-        <v>621</v>
       </c>
       <c r="F248" s="5" t="s">
         <v>101</v>
@@ -7219,13 +7219,13 @@
         <v>73</v>
       </c>
       <c r="B251" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="C251" s="2" t="s">
         <v>634</v>
       </c>
-      <c r="C251" s="2" t="s">
+      <c r="D251" s="2" t="s">
         <v>635</v>
-      </c>
-      <c r="D251" s="2" t="s">
-        <v>636</v>
       </c>
       <c r="F251" s="5" t="s">
         <v>101</v>
@@ -7236,10 +7236,10 @@
         <v>73</v>
       </c>
       <c r="B252" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="C252" s="2" t="s">
         <v>622</v>
-      </c>
-      <c r="C252" s="2" t="s">
-        <v>623</v>
       </c>
       <c r="F252" s="5" t="s">
         <v>101</v>
@@ -7250,10 +7250,10 @@
         <v>73</v>
       </c>
       <c r="B253" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="C253" s="2" t="s">
         <v>818</v>
-      </c>
-      <c r="C253" s="2" t="s">
-        <v>819</v>
       </c>
       <c r="F253" s="3" t="s">
         <v>99</v>
@@ -7264,10 +7264,10 @@
         <v>73</v>
       </c>
       <c r="B254" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="C254" s="2" t="s">
         <v>708</v>
-      </c>
-      <c r="C254" s="2" t="s">
-        <v>709</v>
       </c>
       <c r="F254" s="3" t="s">
         <v>99</v>
@@ -7278,10 +7278,10 @@
         <v>73</v>
       </c>
       <c r="B255" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="C255" s="2" t="s">
         <v>637</v>
-      </c>
-      <c r="C255" s="2" t="s">
-        <v>638</v>
       </c>
       <c r="F255" s="3" t="s">
         <v>99</v>
@@ -7292,10 +7292,10 @@
         <v>73</v>
       </c>
       <c r="B256" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="C256" s="2" t="s">
         <v>609</v>
-      </c>
-      <c r="C256" s="2" t="s">
-        <v>610</v>
       </c>
       <c r="F256" s="3" t="s">
         <v>99</v>
@@ -7306,10 +7306,10 @@
         <v>73</v>
       </c>
       <c r="B257" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="C257" s="2" t="s">
         <v>589</v>
-      </c>
-      <c r="C257" s="2" t="s">
-        <v>590</v>
       </c>
       <c r="F257" s="4" t="s">
         <v>100</v>
@@ -7407,13 +7407,13 @@
         <v>73</v>
       </c>
       <c r="B264" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="C264" s="2" t="s">
         <v>624</v>
       </c>
-      <c r="C264" s="2" t="s">
+      <c r="D264" s="2" t="s">
         <v>625</v>
-      </c>
-      <c r="D264" s="2" t="s">
-        <v>626</v>
       </c>
       <c r="F264" s="5" t="s">
         <v>101</v>
@@ -7424,10 +7424,10 @@
         <v>73</v>
       </c>
       <c r="B265" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C265" s="2" t="s">
         <v>448</v>
-      </c>
-      <c r="C265" s="2" t="s">
-        <v>449</v>
       </c>
       <c r="F265" s="4" t="s">
         <v>100</v>
@@ -7438,10 +7438,10 @@
         <v>73</v>
       </c>
       <c r="B266" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="C266" s="2" t="s">
         <v>478</v>
-      </c>
-      <c r="C266" s="2" t="s">
-        <v>479</v>
       </c>
       <c r="F266" s="4" t="s">
         <v>100</v>
@@ -7452,10 +7452,10 @@
         <v>73</v>
       </c>
       <c r="B267" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="C267" s="2" t="s">
         <v>639</v>
-      </c>
-      <c r="C267" s="2" t="s">
-        <v>640</v>
       </c>
       <c r="F267" s="5" t="s">
         <v>101</v>
@@ -7466,10 +7466,10 @@
         <v>73</v>
       </c>
       <c r="B268" s="2" t="s">
+        <v>738</v>
+      </c>
+      <c r="C268" s="2" t="s">
         <v>739</v>
-      </c>
-      <c r="C268" s="2" t="s">
-        <v>740</v>
       </c>
       <c r="F268" s="3" t="s">
         <v>99</v>
@@ -7494,10 +7494,10 @@
         <v>73</v>
       </c>
       <c r="B270" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="C270" s="2" t="s">
         <v>548</v>
-      </c>
-      <c r="C270" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="F270" s="5" t="s">
         <v>101</v>
@@ -7576,10 +7576,10 @@
         <v>73</v>
       </c>
       <c r="B275" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="C275" s="2" t="s">
         <v>691</v>
-      </c>
-      <c r="C275" s="2" t="s">
-        <v>692</v>
       </c>
       <c r="F275" s="5" t="s">
         <v>238</v>
@@ -7604,10 +7604,10 @@
         <v>73</v>
       </c>
       <c r="B277" s="2" t="s">
+        <v>742</v>
+      </c>
+      <c r="C277" s="2" t="s">
         <v>743</v>
-      </c>
-      <c r="C277" s="2" t="s">
-        <v>744</v>
       </c>
       <c r="F277" s="4" t="s">
         <v>100</v>
@@ -7635,10 +7635,10 @@
         <v>73</v>
       </c>
       <c r="B279" s="2" t="s">
+        <v>640</v>
+      </c>
+      <c r="C279" s="2" t="s">
         <v>641</v>
-      </c>
-      <c r="C279" s="2" t="s">
-        <v>642</v>
       </c>
       <c r="F279" s="5" t="s">
         <v>101</v>
@@ -7649,10 +7649,10 @@
         <v>73</v>
       </c>
       <c r="B280" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="C280" s="2" t="s">
         <v>507</v>
-      </c>
-      <c r="C280" s="2" t="s">
-        <v>508</v>
       </c>
       <c r="F280" s="5" t="s">
         <v>101</v>
@@ -7663,16 +7663,16 @@
         <v>73</v>
       </c>
       <c r="B281" s="2" t="s">
+        <v>775</v>
+      </c>
+      <c r="C281" s="2" t="s">
         <v>776</v>
-      </c>
-      <c r="C281" s="2" t="s">
-        <v>777</v>
       </c>
       <c r="F281" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G281" s="2" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.35">
@@ -7708,10 +7708,10 @@
         <v>73</v>
       </c>
       <c r="B284" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="C284" s="2" t="s">
         <v>643</v>
-      </c>
-      <c r="C284" s="2" t="s">
-        <v>644</v>
       </c>
       <c r="F284" s="4" t="s">
         <v>100</v>
@@ -7736,10 +7736,10 @@
         <v>73</v>
       </c>
       <c r="B286" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="C286" s="2" t="s">
         <v>627</v>
-      </c>
-      <c r="C286" s="2" t="s">
-        <v>628</v>
       </c>
       <c r="F286" s="5" t="s">
         <v>101</v>
@@ -7764,10 +7764,10 @@
         <v>73</v>
       </c>
       <c r="B288" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="C288" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="C288" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="F288" s="14" t="s">
         <v>258</v>
@@ -7778,10 +7778,10 @@
         <v>73</v>
       </c>
       <c r="B289" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="C289" s="2" t="s">
         <v>522</v>
-      </c>
-      <c r="C289" s="2" t="s">
-        <v>523</v>
       </c>
       <c r="E289" s="2" t="s">
         <v>226</v>
@@ -7809,10 +7809,10 @@
         <v>73</v>
       </c>
       <c r="B291" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="C291" s="2" t="s">
         <v>645</v>
-      </c>
-      <c r="C291" s="2" t="s">
-        <v>646</v>
       </c>
       <c r="F291" s="20" t="s">
         <v>100</v>
@@ -7823,16 +7823,16 @@
         <v>73</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="F292" s="3" t="s">
         <v>99</v>
       </c>
       <c r="G292" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="293" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7840,16 +7840,16 @@
         <v>73</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="F293" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G293" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="294" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -7925,13 +7925,13 @@
         <v>90</v>
       </c>
       <c r="B298" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="C298" s="2" t="s">
         <v>801</v>
       </c>
-      <c r="C298" s="2" t="s">
+      <c r="F298" s="25" t="s">
         <v>802</v>
-      </c>
-      <c r="F298" s="25" t="s">
-        <v>803</v>
       </c>
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.35">
@@ -7953,13 +7953,13 @@
         <v>90</v>
       </c>
       <c r="B300" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C300" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="C300" s="2" t="s">
+      <c r="D300" s="2" t="s">
         <v>565</v>
-      </c>
-      <c r="D300" s="2" t="s">
-        <v>566</v>
       </c>
       <c r="F300" s="4" t="s">
         <v>100</v>
@@ -8049,10 +8049,10 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>484</v>
+      </c>
+      <c r="B7" t="s">
         <v>485</v>
-      </c>
-      <c r="B7" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Add new input data variable for the markup on battery packs (separate from manufacturing pack price file, which is unique to some cash flows specific to the battery manufacturing sector)
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B9A522-AC81-49EE-88D1-EB8CBF90E990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730C44AC-7D31-4302-9A0A-C633B8634610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1428" uniqueCount="829">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="831">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2519,6 +2519,12 @@
   </si>
   <si>
     <t>BAU Imported Electricity, BAU Exported Electricity, Imported Electricity Price</t>
+  </si>
+  <si>
+    <t>BPM</t>
+  </si>
+  <si>
+    <t>Battery Pack Markup</t>
   </si>
 </sst>
 </file>
@@ -3330,7 +3336,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G300"/>
+  <dimension ref="A1:G301"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
@@ -7193,16 +7199,13 @@
         <v>73</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>633</v>
+        <v>829</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="D250" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="F250" s="5" t="s">
-        <v>101</v>
+        <v>830</v>
+      </c>
+      <c r="F250" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.35">
@@ -7210,10 +7213,13 @@
         <v>73</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>621</v>
+        <v>633</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>622</v>
+        <v>634</v>
+      </c>
+      <c r="D251" s="2" t="s">
+        <v>635</v>
       </c>
       <c r="F251" s="5" t="s">
         <v>101</v>
@@ -7224,13 +7230,13 @@
         <v>73</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>814</v>
+        <v>621</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>815</v>
-      </c>
-      <c r="F252" s="3" t="s">
-        <v>99</v>
+        <v>622</v>
+      </c>
+      <c r="F252" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.35">
@@ -7238,10 +7244,10 @@
         <v>73</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>705</v>
+        <v>814</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>706</v>
+        <v>815</v>
       </c>
       <c r="F253" s="3" t="s">
         <v>99</v>
@@ -7252,10 +7258,10 @@
         <v>73</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>636</v>
+        <v>705</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>637</v>
+        <v>706</v>
       </c>
       <c r="F254" s="3" t="s">
         <v>99</v>
@@ -7266,10 +7272,10 @@
         <v>73</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>608</v>
+        <v>636</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>609</v>
+        <v>637</v>
       </c>
       <c r="F255" s="3" t="s">
         <v>99</v>
@@ -7280,13 +7286,13 @@
         <v>73</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>588</v>
+        <v>608</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>589</v>
-      </c>
-      <c r="F256" s="4" t="s">
-        <v>100</v>
+        <v>609</v>
+      </c>
+      <c r="F256" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.35">
@@ -7294,44 +7300,44 @@
         <v>73</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>241</v>
+        <v>588</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>242</v>
+        <v>589</v>
       </c>
       <c r="F257" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="258" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A258" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>285</v>
+        <v>241</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="F258" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="G258" s="2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+      <c r="F258" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A259" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>76</v>
+        <v>285</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F259" s="5" t="s">
-        <v>101</v>
+        <v>286</v>
+      </c>
+      <c r="F259" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="G259" s="2" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.35">
@@ -7339,10 +7345,10 @@
         <v>73</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F260" s="5" t="s">
         <v>101</v>
@@ -7353,10 +7359,10 @@
         <v>73</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F261" s="5" t="s">
         <v>101</v>
@@ -7367,13 +7373,13 @@
         <v>73</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F262" s="4" t="s">
-        <v>100</v>
+        <v>86</v>
+      </c>
+      <c r="F262" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.35">
@@ -7381,16 +7387,13 @@
         <v>73</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>623</v>
+        <v>79</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="D263" s="2" t="s">
-        <v>625</v>
-      </c>
-      <c r="F263" s="5" t="s">
-        <v>101</v>
+        <v>87</v>
+      </c>
+      <c r="F263" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.35">
@@ -7398,13 +7401,16 @@
         <v>73</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>447</v>
+        <v>623</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="F264" s="4" t="s">
-        <v>100</v>
+        <v>624</v>
+      </c>
+      <c r="D264" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="F264" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.35">
@@ -7412,41 +7418,41 @@
         <v>73</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>477</v>
+        <v>447</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>478</v>
+        <v>448</v>
       </c>
       <c r="F265" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="266" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A266" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>638</v>
+        <v>477</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="F266" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
+        <v>478</v>
+      </c>
+      <c r="F266" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A267" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>735</v>
+        <v>638</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>736</v>
-      </c>
-      <c r="F267" s="3" t="s">
-        <v>99</v>
+        <v>639</v>
+      </c>
+      <c r="F267" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.35">
@@ -7454,10 +7460,10 @@
         <v>73</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>80</v>
+        <v>735</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>88</v>
+        <v>736</v>
       </c>
       <c r="F268" s="3" t="s">
         <v>99</v>
@@ -7468,30 +7474,27 @@
         <v>73</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>547</v>
+        <v>80</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="F269" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="270" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+      <c r="F269" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A270" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>293</v>
+        <v>547</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="F270" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G270" s="2" t="s">
-        <v>335</v>
+        <v>548</v>
+      </c>
+      <c r="F270" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="271" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -7499,10 +7502,10 @@
         <v>73</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="F271" s="16" t="s">
         <v>303</v>
@@ -7516,10 +7519,10 @@
         <v>73</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>239</v>
+        <v>295</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>240</v>
+        <v>296</v>
       </c>
       <c r="F272" s="16" t="s">
         <v>303</v>
@@ -7528,35 +7531,38 @@
         <v>335</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A273" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E273" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="F273" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="274" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>240</v>
+      </c>
+      <c r="F273" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G273" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A274" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>688</v>
+        <v>230</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>689</v>
-      </c>
-      <c r="F274" s="5" t="s">
-        <v>238</v>
+        <v>231</v>
+      </c>
+      <c r="E274" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F274" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="275" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7564,58 +7570,58 @@
         <v>73</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>81</v>
+        <v>688</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F275" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.35">
+        <v>689</v>
+      </c>
+      <c r="F275" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="276" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A276" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>739</v>
+        <v>81</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>740</v>
+        <v>89</v>
       </c>
       <c r="F276" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="277" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A277" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>443</v>
+        <v>739</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="F277" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G277" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
+        <v>740</v>
+      </c>
+      <c r="F277" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A278" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>640</v>
+        <v>443</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="F278" s="5" t="s">
-        <v>101</v>
+        <v>444</v>
+      </c>
+      <c r="F278" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G278" s="2" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.35">
@@ -7623,44 +7629,44 @@
         <v>73</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>506</v>
+        <v>640</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>507</v>
+        <v>641</v>
       </c>
       <c r="F279" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="280" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A280" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>772</v>
+        <v>506</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>773</v>
-      </c>
-      <c r="F280" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G280" s="2" t="s">
-        <v>774</v>
-      </c>
-    </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
+        <v>507</v>
+      </c>
+      <c r="F280" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A281" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>245</v>
+        <v>772</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="F281" s="14" t="s">
-        <v>258</v>
+        <v>773</v>
+      </c>
+      <c r="F281" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G281" s="2" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.35">
@@ -7668,13 +7674,13 @@
         <v>73</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>298</v>
+        <v>245</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="F282" s="5" t="s">
-        <v>101</v>
+        <v>246</v>
+      </c>
+      <c r="F282" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.35">
@@ -7682,13 +7688,13 @@
         <v>73</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>642</v>
+        <v>298</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="F283" s="4" t="s">
-        <v>100</v>
+        <v>297</v>
+      </c>
+      <c r="F283" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.35">
@@ -7696,13 +7702,13 @@
         <v>73</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>234</v>
+        <v>642</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="F284" s="5" t="s">
-        <v>101</v>
+        <v>643</v>
+      </c>
+      <c r="F284" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.35">
@@ -7710,10 +7716,10 @@
         <v>73</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>626</v>
+        <v>234</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>627</v>
+        <v>235</v>
       </c>
       <c r="F285" s="5" t="s">
         <v>101</v>
@@ -7724,13 +7730,13 @@
         <v>73</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>226</v>
+        <v>626</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="F286" s="12" t="s">
-        <v>250</v>
+        <v>627</v>
+      </c>
+      <c r="F286" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.35">
@@ -7738,13 +7744,13 @@
         <v>73</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>523</v>
+        <v>226</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="F287" s="14" t="s">
-        <v>258</v>
+        <v>227</v>
+      </c>
+      <c r="F287" s="12" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.35">
@@ -7752,16 +7758,13 @@
         <v>73</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="E288" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="F288" s="5" t="s">
-        <v>101</v>
+        <v>524</v>
+      </c>
+      <c r="F288" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.35">
@@ -7769,44 +7772,44 @@
         <v>73</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>224</v>
+        <v>521</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>225</v>
+        <v>522</v>
+      </c>
+      <c r="E289" s="2" t="s">
+        <v>226</v>
       </c>
       <c r="F289" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="290" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="290" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A290" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>644</v>
+        <v>224</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>645</v>
-      </c>
-      <c r="F290" s="20" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="291" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>225</v>
+      </c>
+      <c r="F290" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A291" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="F291" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G291" s="2" t="s">
-        <v>586</v>
+        <v>645</v>
+      </c>
+      <c r="F291" s="20" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="292" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7814,81 +7817,81 @@
         <v>73</v>
       </c>
       <c r="B292" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="C292" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="F292" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G292" s="2" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A293" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B293" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="C292" s="2" t="s">
+      <c r="C293" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="F292" s="16" t="s">
+      <c r="F293" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="G292" s="2" t="s">
+      <c r="G293" s="2" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="293" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A293" s="17" t="s">
+    <row r="294" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A294" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B293" s="17" t="s">
+      <c r="B294" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="C293" s="17" t="s">
+      <c r="C294" s="17" t="s">
         <v>307</v>
       </c>
-      <c r="D293" s="17"/>
-      <c r="E293" s="17"/>
-      <c r="F293" s="20" t="s">
+      <c r="D294" s="17"/>
+      <c r="E294" s="17"/>
+      <c r="F294" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G293" s="17"/>
-    </row>
-    <row r="294" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A294" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B294" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C294" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D294" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="F294" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G294" s="17"/>
+    </row>
+    <row r="295" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A295" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>222</v>
+        <v>91</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>221</v>
+        <v>92</v>
       </c>
       <c r="D295" s="2" t="s">
-        <v>403</v>
+        <v>315</v>
       </c>
       <c r="F295" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="296" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A296" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>247</v>
+        <v>222</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>248</v>
+        <v>221</v>
       </c>
       <c r="D296" s="2" t="s">
-        <v>249</v>
+        <v>403</v>
       </c>
       <c r="F296" s="5" t="s">
         <v>101</v>
@@ -7899,27 +7902,30 @@
         <v>90</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>797</v>
+        <v>247</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>798</v>
-      </c>
-      <c r="F297" s="25" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.35">
+        <v>248</v>
+      </c>
+      <c r="D297" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="F297" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A298" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>351</v>
+        <v>797</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="F298" s="4" t="s">
-        <v>100</v>
+        <v>798</v>
+      </c>
+      <c r="F298" s="25" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.35">
@@ -7927,36 +7933,50 @@
         <v>90</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>563</v>
+        <v>351</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="D299" s="2" t="s">
-        <v>565</v>
+        <v>352</v>
       </c>
       <c r="F299" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="300" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A300" s="17" t="s">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A300" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B300" s="17" t="s">
+      <c r="B300" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C300" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="D300" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="F300" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A301" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B301" s="17" t="s">
         <v>291</v>
       </c>
-      <c r="C300" s="17" t="s">
+      <c r="C301" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="D300" s="17" t="s">
+      <c r="D301" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="E300" s="17"/>
-      <c r="F300" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="G300" s="17"/>
+      <c r="E301" s="17"/>
+      <c r="F301" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G301" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Acronym key update for new BPPM file
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730C44AC-7D31-4302-9A0A-C633B8634610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689CA091-282C-434F-9EC8-B18750BFFC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="831">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="833">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2525,6 +2525,12 @@
   </si>
   <si>
     <t>Battery Pack Markup</t>
+  </si>
+  <si>
+    <t>BPPM</t>
+  </si>
+  <si>
+    <t>Battery Pack Price Multiplier</t>
   </si>
 </sst>
 </file>
@@ -3336,7 +3342,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G301"/>
+  <dimension ref="A1:G302"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
@@ -7230,13 +7236,13 @@
         <v>73</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>621</v>
+        <v>831</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="F252" s="5" t="s">
-        <v>101</v>
+        <v>832</v>
+      </c>
+      <c r="F252" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.35">
@@ -7244,13 +7250,13 @@
         <v>73</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>814</v>
+        <v>621</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>815</v>
-      </c>
-      <c r="F253" s="3" t="s">
-        <v>99</v>
+        <v>622</v>
+      </c>
+      <c r="F253" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.35">
@@ -7258,10 +7264,10 @@
         <v>73</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>705</v>
+        <v>814</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>706</v>
+        <v>815</v>
       </c>
       <c r="F254" s="3" t="s">
         <v>99</v>
@@ -7272,10 +7278,10 @@
         <v>73</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>636</v>
+        <v>705</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>637</v>
+        <v>706</v>
       </c>
       <c r="F255" s="3" t="s">
         <v>99</v>
@@ -7286,10 +7292,10 @@
         <v>73</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>608</v>
+        <v>636</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>609</v>
+        <v>637</v>
       </c>
       <c r="F256" s="3" t="s">
         <v>99</v>
@@ -7300,13 +7306,13 @@
         <v>73</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>588</v>
+        <v>608</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>589</v>
-      </c>
-      <c r="F257" s="4" t="s">
-        <v>100</v>
+        <v>609</v>
+      </c>
+      <c r="F257" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.35">
@@ -7314,44 +7320,44 @@
         <v>73</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>241</v>
+        <v>588</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>242</v>
+        <v>589</v>
       </c>
       <c r="F258" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="259" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A259" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>285</v>
+        <v>241</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="F259" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="G259" s="2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+      <c r="F259" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A260" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>76</v>
+        <v>285</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F260" s="5" t="s">
-        <v>101</v>
+        <v>286</v>
+      </c>
+      <c r="F260" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="G260" s="2" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.35">
@@ -7359,10 +7365,10 @@
         <v>73</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F261" s="5" t="s">
         <v>101</v>
@@ -7373,10 +7379,10 @@
         <v>73</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F262" s="5" t="s">
         <v>101</v>
@@ -7387,13 +7393,13 @@
         <v>73</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F263" s="4" t="s">
-        <v>100</v>
+        <v>86</v>
+      </c>
+      <c r="F263" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.35">
@@ -7401,16 +7407,13 @@
         <v>73</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>623</v>
+        <v>79</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="D264" s="2" t="s">
-        <v>625</v>
-      </c>
-      <c r="F264" s="5" t="s">
-        <v>101</v>
+        <v>87</v>
+      </c>
+      <c r="F264" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.35">
@@ -7418,13 +7421,16 @@
         <v>73</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>447</v>
+        <v>623</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="F265" s="4" t="s">
-        <v>100</v>
+        <v>624</v>
+      </c>
+      <c r="D265" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="F265" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.35">
@@ -7432,41 +7438,41 @@
         <v>73</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>477</v>
+        <v>447</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>478</v>
+        <v>448</v>
       </c>
       <c r="F266" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="267" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A267" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>638</v>
+        <v>477</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="F267" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
+        <v>478</v>
+      </c>
+      <c r="F267" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A268" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>735</v>
+        <v>638</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>736</v>
-      </c>
-      <c r="F268" s="3" t="s">
-        <v>99</v>
+        <v>639</v>
+      </c>
+      <c r="F268" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.35">
@@ -7474,10 +7480,10 @@
         <v>73</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>80</v>
+        <v>735</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>88</v>
+        <v>736</v>
       </c>
       <c r="F269" s="3" t="s">
         <v>99</v>
@@ -7488,30 +7494,27 @@
         <v>73</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>547</v>
+        <v>80</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="F270" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="271" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+      <c r="F270" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="271" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A271" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>293</v>
+        <v>547</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="F271" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G271" s="2" t="s">
-        <v>335</v>
+        <v>548</v>
+      </c>
+      <c r="F271" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="272" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -7519,10 +7522,10 @@
         <v>73</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="F272" s="16" t="s">
         <v>303</v>
@@ -7536,10 +7539,10 @@
         <v>73</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>239</v>
+        <v>295</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>240</v>
+        <v>296</v>
       </c>
       <c r="F273" s="16" t="s">
         <v>303</v>
@@ -7548,35 +7551,38 @@
         <v>335</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A274" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E274" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="F274" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="275" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>240</v>
+      </c>
+      <c r="F274" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G274" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A275" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>688</v>
+        <v>230</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>689</v>
-      </c>
-      <c r="F275" s="5" t="s">
-        <v>238</v>
+        <v>231</v>
+      </c>
+      <c r="E275" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F275" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="276" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7584,58 +7590,58 @@
         <v>73</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>81</v>
+        <v>688</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F276" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.35">
+        <v>689</v>
+      </c>
+      <c r="F276" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="277" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A277" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>739</v>
+        <v>81</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>740</v>
+        <v>89</v>
       </c>
       <c r="F277" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="278" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A278" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>443</v>
+        <v>739</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="F278" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G278" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
+        <v>740</v>
+      </c>
+      <c r="F278" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A279" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>640</v>
+        <v>443</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="F279" s="5" t="s">
-        <v>101</v>
+        <v>444</v>
+      </c>
+      <c r="F279" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G279" s="2" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.35">
@@ -7643,44 +7649,44 @@
         <v>73</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>506</v>
+        <v>640</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>507</v>
+        <v>641</v>
       </c>
       <c r="F280" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="281" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A281" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>772</v>
+        <v>506</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>773</v>
-      </c>
-      <c r="F281" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G281" s="2" t="s">
-        <v>774</v>
-      </c>
-    </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
+        <v>507</v>
+      </c>
+      <c r="F281" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A282" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>245</v>
+        <v>772</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="F282" s="14" t="s">
-        <v>258</v>
+        <v>773</v>
+      </c>
+      <c r="F282" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G282" s="2" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.35">
@@ -7688,13 +7694,13 @@
         <v>73</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>298</v>
+        <v>245</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="F283" s="5" t="s">
-        <v>101</v>
+        <v>246</v>
+      </c>
+      <c r="F283" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.35">
@@ -7702,13 +7708,13 @@
         <v>73</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>642</v>
+        <v>298</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="F284" s="4" t="s">
-        <v>100</v>
+        <v>297</v>
+      </c>
+      <c r="F284" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.35">
@@ -7716,13 +7722,13 @@
         <v>73</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>234</v>
+        <v>642</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="F285" s="5" t="s">
-        <v>101</v>
+        <v>643</v>
+      </c>
+      <c r="F285" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="286" spans="1:7" x14ac:dyDescent="0.35">
@@ -7730,10 +7736,10 @@
         <v>73</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>626</v>
+        <v>234</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>627</v>
+        <v>235</v>
       </c>
       <c r="F286" s="5" t="s">
         <v>101</v>
@@ -7744,13 +7750,13 @@
         <v>73</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>226</v>
+        <v>626</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="F287" s="12" t="s">
-        <v>250</v>
+        <v>627</v>
+      </c>
+      <c r="F287" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.35">
@@ -7758,13 +7764,13 @@
         <v>73</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>523</v>
+        <v>226</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="F288" s="14" t="s">
-        <v>258</v>
+        <v>227</v>
+      </c>
+      <c r="F288" s="12" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.35">
@@ -7772,16 +7778,13 @@
         <v>73</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="E289" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="F289" s="5" t="s">
-        <v>101</v>
+        <v>524</v>
+      </c>
+      <c r="F289" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.35">
@@ -7789,44 +7792,44 @@
         <v>73</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>224</v>
+        <v>521</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>225</v>
+        <v>522</v>
+      </c>
+      <c r="E290" s="2" t="s">
+        <v>226</v>
       </c>
       <c r="F290" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="291" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A291" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>644</v>
+        <v>224</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>645</v>
-      </c>
-      <c r="F291" s="20" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="292" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>225</v>
+      </c>
+      <c r="F291" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A292" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="F292" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G292" s="2" t="s">
-        <v>586</v>
+        <v>645</v>
+      </c>
+      <c r="F292" s="20" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="293" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7834,81 +7837,81 @@
         <v>73</v>
       </c>
       <c r="B293" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="C293" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="F293" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G293" s="2" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A294" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B294" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="C293" s="2" t="s">
+      <c r="C294" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="F293" s="16" t="s">
+      <c r="F294" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="G293" s="2" t="s">
+      <c r="G294" s="2" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="294" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A294" s="17" t="s">
+    <row r="295" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A295" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B294" s="17" t="s">
+      <c r="B295" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="C294" s="17" t="s">
+      <c r="C295" s="17" t="s">
         <v>307</v>
       </c>
-      <c r="D294" s="17"/>
-      <c r="E294" s="17"/>
-      <c r="F294" s="20" t="s">
+      <c r="D295" s="17"/>
+      <c r="E295" s="17"/>
+      <c r="F295" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G294" s="17"/>
-    </row>
-    <row r="295" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A295" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B295" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C295" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D295" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="F295" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G295" s="17"/>
+    </row>
+    <row r="296" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A296" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>222</v>
+        <v>91</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>221</v>
+        <v>92</v>
       </c>
       <c r="D296" s="2" t="s">
-        <v>403</v>
+        <v>315</v>
       </c>
       <c r="F296" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="297" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A297" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>247</v>
+        <v>222</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>248</v>
+        <v>221</v>
       </c>
       <c r="D297" s="2" t="s">
-        <v>249</v>
+        <v>403</v>
       </c>
       <c r="F297" s="5" t="s">
         <v>101</v>
@@ -7919,27 +7922,30 @@
         <v>90</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>797</v>
+        <v>247</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>798</v>
-      </c>
-      <c r="F298" s="25" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.35">
+        <v>248</v>
+      </c>
+      <c r="D298" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="F298" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A299" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>351</v>
+        <v>797</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="F299" s="4" t="s">
-        <v>100</v>
+        <v>798</v>
+      </c>
+      <c r="F299" s="25" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="300" spans="1:7" x14ac:dyDescent="0.35">
@@ -7947,36 +7953,50 @@
         <v>90</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>563</v>
+        <v>351</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="D300" s="2" t="s">
-        <v>565</v>
+        <v>352</v>
       </c>
       <c r="F300" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="301" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A301" s="17" t="s">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A301" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B301" s="17" t="s">
+      <c r="B301" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C301" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="D301" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="F301" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="302" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A302" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B302" s="17" t="s">
         <v>291</v>
       </c>
-      <c r="C301" s="17" t="s">
+      <c r="C302" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="D301" s="17" t="s">
+      <c r="D302" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="E301" s="17"/>
-      <c r="F301" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="G301" s="17"/>
+      <c r="E302" s="17"/>
+      <c r="F302" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G302" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add a new input data file that applies a discount factor to the amount of load shifting capacity from grid battery storage to account for usage factors < one cycle per day
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689CA091-282C-434F-9EC8-B18750BFFC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F5458D-FD54-4D41-8C5F-134816A8CA9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="833">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="835">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2531,6 +2531,12 @@
   </si>
   <si>
     <t>Battery Pack Price Multiplier</t>
+  </si>
+  <si>
+    <t>UFDfGBS</t>
+  </si>
+  <si>
+    <t>Usage Factor Discount for Grid Battery Storage</t>
   </si>
 </sst>
 </file>
@@ -3342,7 +3348,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G302"/>
+  <dimension ref="A1:G303"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
@@ -5427,101 +5433,101 @@
         <v>101</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A134" s="17" t="s">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A134" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B134" s="17" t="s">
+      <c r="B134" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="F134" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A135" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B135" s="17" t="s">
         <v>347</v>
       </c>
-      <c r="C134" s="17" t="s">
+      <c r="C135" s="17" t="s">
         <v>348</v>
       </c>
-      <c r="D134" s="17" t="s">
+      <c r="D135" s="17" t="s">
         <v>349</v>
       </c>
-      <c r="E134" s="17"/>
-      <c r="F134" s="21" t="s">
+      <c r="E135" s="17"/>
+      <c r="F135" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="G134" s="17" t="s">
+      <c r="G135" s="17" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A135" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="B135" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="C135" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="D135" s="2" t="s">
-        <v>702</v>
-      </c>
-      <c r="F135" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>630</v>
+        <v>702</v>
       </c>
       <c r="F136" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>630</v>
       </c>
       <c r="F137" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>418</v>
+        <v>271</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="F138" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+        <v>272</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
         <v>275</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>183</v>
+        <v>418</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="F139" s="4" t="s">
-        <v>100</v>
+        <v>419</v>
+      </c>
+      <c r="F139" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.35">
@@ -5529,69 +5535,69 @@
         <v>275</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="F140" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A141" s="17" t="s">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A141" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B141" s="17" t="s">
+      <c r="B141" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F141" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A142" s="17" t="s">
+        <v>275</v>
+      </c>
+      <c r="B142" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="C141" s="17" t="s">
+      <c r="C142" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="D141" s="17"/>
-      <c r="E141" s="17"/>
-      <c r="F141" s="20" t="s">
+      <c r="D142" s="17"/>
+      <c r="E142" s="17"/>
+      <c r="F142" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G141" s="17"/>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A142" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B142" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="C142" s="2" t="s">
-        <v>471</v>
-      </c>
-      <c r="F142" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="G142" s="17"/>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>785</v>
+        <v>470</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>788</v>
-      </c>
-      <c r="F143" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+        <v>471</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="F144" s="5" t="s">
         <v>101</v>
@@ -5602,10 +5608,10 @@
         <v>55</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="F145" s="5" t="s">
         <v>101</v>
@@ -5616,16 +5622,13 @@
         <v>55</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>472</v>
+        <v>787</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="D146" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="F146" s="3" t="s">
-        <v>99</v>
+        <v>790</v>
+      </c>
+      <c r="F146" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.35">
@@ -5633,69 +5636,72 @@
         <v>55</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>380</v>
+        <v>472</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>381</v>
+        <v>473</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>474</v>
       </c>
       <c r="F147" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="148" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>56</v>
+        <v>380</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D148" s="2" t="s">
-        <v>268</v>
+        <v>381</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>313</v>
+        <v>56</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="F149" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="F149" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>776</v>
+        <v>313</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>777</v>
+        <v>314</v>
       </c>
       <c r="F150" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>628</v>
+        <v>776</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>629</v>
+        <v>777</v>
       </c>
       <c r="F151" s="5" t="s">
         <v>101</v>
@@ -5706,13 +5712,10 @@
         <v>55</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>525</v>
+        <v>628</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>792</v>
-      </c>
-      <c r="E152" s="2" t="s">
-        <v>526</v>
+        <v>629</v>
       </c>
       <c r="F152" s="5" t="s">
         <v>101</v>
@@ -5723,10 +5726,13 @@
         <v>55</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>791</v>
+        <v>525</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>778</v>
+        <v>792</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>526</v>
       </c>
       <c r="F153" s="5" t="s">
         <v>101</v>
@@ -5737,13 +5743,13 @@
         <v>55</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>542</v>
+        <v>791</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="F154" s="3" t="s">
-        <v>99</v>
+        <v>778</v>
+      </c>
+      <c r="F154" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.35">
@@ -5751,61 +5757,58 @@
         <v>55</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>606</v>
+        <v>542</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>607</v>
-      </c>
-      <c r="F155" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="156" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>543</v>
+      </c>
+      <c r="F155" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>57</v>
+        <v>606</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F156" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G156" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+        <v>607</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>311</v>
+        <v>57</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="F157" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="158" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+      <c r="F157" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G157" s="2" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>390</v>
+        <v>311</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="F158" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G158" s="2" t="s">
-        <v>396</v>
+        <v>312</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="159" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5813,16 +5816,16 @@
         <v>55</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F159" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G159" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5830,129 +5833,132 @@
         <v>55</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F160" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G160" s="2" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="161" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>58</v>
+        <v>392</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D161" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F161" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="162" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+      <c r="F161" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G161" s="2" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>376</v>
+        <v>58</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>340</v>
+        <v>61</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="F162" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B163" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F163" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A164" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B164" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="C163" s="2" t="s">
+      <c r="C164" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="F163" s="3" t="s">
+      <c r="F164" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="164" spans="1:7" s="17" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A164" s="17" t="s">
+    <row r="165" spans="1:7" s="17" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A165" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B164" s="17" t="s">
+      <c r="B165" s="17" t="s">
         <v>441</v>
       </c>
-      <c r="C164" s="17" t="s">
+      <c r="C165" s="17" t="s">
         <v>442</v>
       </c>
-      <c r="F164" s="22" t="s">
+      <c r="F165" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="G164" s="17" t="s">
+      <c r="G165" s="17" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A165" s="2" t="s">
+    <row r="166" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A166" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="B165" s="2" t="s">
+      <c r="B166" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="C165" s="2" t="s">
+      <c r="C166" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="D165" s="2" t="s">
+      <c r="D166" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="F165" s="3" t="s">
+      <c r="F166" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="166" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A166" s="17" t="s">
+    <row r="167" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A167" s="17" t="s">
         <v>754</v>
       </c>
-      <c r="B166" s="17" t="s">
+      <c r="B167" s="17" t="s">
         <v>755</v>
       </c>
-      <c r="C166" s="17" t="s">
+      <c r="C167" s="17" t="s">
         <v>756</v>
       </c>
-      <c r="D166" s="17" t="s">
+      <c r="D167" s="17" t="s">
         <v>757</v>
       </c>
-      <c r="F166" s="19" t="s">
+      <c r="F167" s="19" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A167" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="B167" s="2" t="s">
-        <v>359</v>
-      </c>
-      <c r="C167" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="F167" s="5" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.35">
@@ -5960,13 +5966,13 @@
         <v>357</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="F168" s="4" t="s">
-        <v>100</v>
+        <v>366</v>
+      </c>
+      <c r="F168" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.35">
@@ -5974,27 +5980,24 @@
         <v>357</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F169" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
         <v>357</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="D170" s="2" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="F170" s="4" t="s">
         <v>100</v>
@@ -6005,45 +6008,47 @@
         <v>357</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>373</v>
       </c>
       <c r="F171" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
         <v>357</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="F172" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G172" s="2" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="173" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>370</v>
+      </c>
+      <c r="F172" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>357</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>807</v>
+        <v>364</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>808</v>
-      </c>
-      <c r="F173" s="6"/>
+        <v>371</v>
+      </c>
+      <c r="F173" s="6" t="s">
+        <v>142</v>
+      </c>
       <c r="G173" s="2" t="s">
-        <v>809</v>
+        <v>374</v>
       </c>
     </row>
     <row r="174" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6051,64 +6056,62 @@
         <v>357</v>
       </c>
       <c r="B174" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="F174" s="6"/>
+      <c r="G174" s="2" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A175" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="B175" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="C174" s="2" t="s">
+      <c r="C175" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="F174" s="6" t="s">
+      <c r="F175" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="G174" s="2" t="s">
+      <c r="G175" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="175" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A175" s="17" t="s">
+    <row r="176" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A176" s="17" t="s">
         <v>357</v>
       </c>
-      <c r="B175" s="17" t="s">
+      <c r="B176" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="C175" s="17" t="s">
+      <c r="C176" s="17" t="s">
         <v>499</v>
       </c>
-      <c r="D175" s="17"/>
-      <c r="E175" s="17"/>
-      <c r="F175" s="20" t="s">
+      <c r="D176" s="17"/>
+      <c r="E176" s="17"/>
+      <c r="F176" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G175" s="17"/>
-    </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A176" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B176" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C176" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F176" s="12" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="177" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="G176" s="17"/>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>518</v>
+        <v>206</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="D177" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="F177" s="14" t="s">
-        <v>400</v>
+        <v>207</v>
+      </c>
+      <c r="F177" s="12" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="178" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6116,16 +6119,16 @@
         <v>63</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>661</v>
+        <v>518</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>662</v>
+        <v>519</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>663</v>
-      </c>
-      <c r="F178" s="4" t="s">
-        <v>100</v>
+        <v>520</v>
+      </c>
+      <c r="F178" s="14" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6133,19 +6136,16 @@
         <v>63</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>197</v>
+        <v>661</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="E179" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="F179" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G179" s="2" t="s">
-        <v>339</v>
+        <v>662</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="F179" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="180" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6153,13 +6153,19 @@
         <v>63</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>326</v>
+        <v>197</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="F180" s="5" t="s">
-        <v>101</v>
+        <v>198</v>
+      </c>
+      <c r="E180" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F180" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G180" s="2" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="181" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6167,27 +6173,27 @@
         <v>63</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>64</v>
+        <v>326</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F181" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
+        <v>327</v>
+      </c>
+      <c r="F181" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>496</v>
+        <v>64</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="F182" s="5" t="s">
-        <v>101</v>
+        <v>67</v>
+      </c>
+      <c r="F182" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.35">
@@ -6195,16 +6201,13 @@
         <v>63</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>65</v>
+        <v>496</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F183" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G183" s="2" t="s">
-        <v>345</v>
+        <v>497</v>
+      </c>
+      <c r="F183" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.35">
@@ -6212,13 +6215,16 @@
         <v>63</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>561</v>
+        <v>65</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="F184" s="5" t="s">
-        <v>101</v>
+        <v>68</v>
+      </c>
+      <c r="F184" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G184" s="2" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.35">
@@ -6226,13 +6232,13 @@
         <v>63</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>760</v>
+        <v>561</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>761</v>
-      </c>
-      <c r="F185" s="4" t="s">
-        <v>100</v>
+        <v>562</v>
+      </c>
+      <c r="F185" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="186" spans="1:7" x14ac:dyDescent="0.35">
@@ -6240,64 +6246,58 @@
         <v>63</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>766</v>
+        <v>760</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>767</v>
+        <v>761</v>
       </c>
       <c r="F186" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="187" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>515</v>
+        <v>766</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="F187" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G187" s="2" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
+        <v>767</v>
+      </c>
+      <c r="F187" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>199</v>
+        <v>515</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F188" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="189" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>516</v>
+      </c>
+      <c r="F188" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G188" s="2" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>810</v>
+        <v>199</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>811</v>
-      </c>
-      <c r="D189" s="2" t="s">
-        <v>812</v>
-      </c>
-      <c r="F189" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G189" s="2" t="s">
-        <v>813</v>
+        <v>200</v>
+      </c>
+      <c r="F189" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="190" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6305,44 +6305,50 @@
         <v>63</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>66</v>
+        <v>810</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>69</v>
+        <v>811</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="F190" s="14" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
+        <v>812</v>
+      </c>
+      <c r="F190" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G190" s="2" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>190</v>
+        <v>66</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F191" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="192" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+      <c r="D191" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="F191" s="14" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>277</v>
+        <v>190</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="F192" s="5" t="s">
-        <v>101</v>
+        <v>191</v>
+      </c>
+      <c r="F192" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="193" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6350,10 +6356,10 @@
         <v>63</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F193" s="5" t="s">
         <v>101</v>
@@ -6364,13 +6370,13 @@
         <v>63</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="F194" s="4" t="s">
-        <v>100</v>
+        <v>281</v>
+      </c>
+      <c r="F194" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="195" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6378,103 +6384,100 @@
         <v>63</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>566</v>
+        <v>279</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>567</v>
-      </c>
-      <c r="F195" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.35">
+        <v>282</v>
+      </c>
+      <c r="F195" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>476</v>
+        <v>566</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="F196" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="197" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>567</v>
+      </c>
+      <c r="F196" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>492</v>
+        <v>476</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>493</v>
+        <v>475</v>
       </c>
       <c r="F197" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="198" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A198" s="17" t="s">
+    <row r="198" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A198" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B198" s="17" t="s">
+      <c r="B198" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="C198" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="F198" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A199" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B199" s="17" t="s">
         <v>494</v>
       </c>
-      <c r="C198" s="17" t="s">
+      <c r="C199" s="17" t="s">
         <v>495</v>
       </c>
-      <c r="D198" s="17"/>
-      <c r="E198" s="17"/>
-      <c r="F198" s="20" t="s">
+      <c r="D199" s="17"/>
+      <c r="E199" s="17"/>
+      <c r="F199" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G198" s="17"/>
-    </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A199" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="B199" s="2" t="s">
-        <v>793</v>
-      </c>
-      <c r="C199" s="2" t="s">
-        <v>794</v>
-      </c>
-      <c r="F199" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="200" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="G199" s="17"/>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>558</v>
+        <v>793</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>559</v>
-      </c>
-      <c r="D200" s="2" t="s">
-        <v>560</v>
+        <v>794</v>
       </c>
       <c r="F200" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>708</v>
+        <v>558</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>709</v>
+        <v>559</v>
       </c>
       <c r="D201" s="2" t="s">
-        <v>707</v>
+        <v>560</v>
       </c>
       <c r="F201" s="3" t="s">
         <v>99</v>
@@ -6485,10 +6488,13 @@
         <v>420</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>428</v>
+        <v>708</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>429</v>
+        <v>709</v>
+      </c>
+      <c r="D202" s="2" t="s">
+        <v>707</v>
       </c>
       <c r="F202" s="3" t="s">
         <v>99</v>
@@ -6499,10 +6505,10 @@
         <v>420</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F203" s="3" t="s">
         <v>99</v>
@@ -6513,10 +6519,10 @@
         <v>420</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>401</v>
+        <v>430</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>402</v>
+        <v>431</v>
       </c>
       <c r="F204" s="3" t="s">
         <v>99</v>
@@ -6527,44 +6533,44 @@
         <v>420</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>432</v>
+        <v>401</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>433</v>
+        <v>402</v>
       </c>
       <c r="F205" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="206" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>612</v>
+        <v>432</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="D206" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="E206" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="F206" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B207" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="D207" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="E207" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="C207" s="2" t="s">
-        <v>435</v>
       </c>
       <c r="F207" s="3" t="s">
         <v>99</v>
@@ -6575,30 +6581,27 @@
         <v>420</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>422</v>
+        <v>434</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>424</v>
+        <v>435</v>
       </c>
       <c r="F208" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="209" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>529</v>
+        <v>422</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>530</v>
-      </c>
-      <c r="F209" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G209" s="2" t="s">
-        <v>531</v>
+        <v>424</v>
+      </c>
+      <c r="F209" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="210" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6606,48 +6609,48 @@
         <v>420</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>479</v>
+        <v>529</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>480</v>
-      </c>
-      <c r="D210" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="F210" s="3"/>
-    </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
+        <v>530</v>
+      </c>
+      <c r="F210" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G210" s="2" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>527</v>
+        <v>479</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="F211" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G211" s="2" t="s">
-        <v>532</v>
-      </c>
+        <v>480</v>
+      </c>
+      <c r="D211" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="F211" s="3"/>
     </row>
     <row r="212" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>502</v>
+        <v>527</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="E212" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="F212" s="3" t="s">
-        <v>99</v>
+        <v>528</v>
+      </c>
+      <c r="F212" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G212" s="2" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.35">
@@ -6655,13 +6658,16 @@
         <v>420</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>501</v>
-      </c>
-      <c r="F213" s="5" t="s">
-        <v>101</v>
+        <v>503</v>
+      </c>
+      <c r="E213" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="F213" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.35">
@@ -6669,10 +6675,10 @@
         <v>420</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>466</v>
+        <v>500</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>467</v>
+        <v>501</v>
       </c>
       <c r="F214" s="5" t="s">
         <v>101</v>
@@ -6683,10 +6689,10 @@
         <v>420</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>423</v>
+        <v>466</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>425</v>
+        <v>467</v>
       </c>
       <c r="F215" s="5" t="s">
         <v>101</v>
@@ -6697,10 +6703,10 @@
         <v>420</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>468</v>
+        <v>423</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>469</v>
+        <v>425</v>
       </c>
       <c r="F216" s="5" t="s">
         <v>101</v>
@@ -6711,106 +6717,106 @@
         <v>420</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>540</v>
+        <v>468</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>541</v>
-      </c>
-      <c r="F217" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="218" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>469</v>
+      </c>
+      <c r="F217" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>426</v>
+        <v>540</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="F218" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G218" s="2" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="219" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>541</v>
+      </c>
+      <c r="F218" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B219" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F219" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G219" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A220" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="B220" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="C219" s="2" t="s">
+      <c r="C220" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="F219" s="19" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="220" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A220" s="17" t="s">
-        <v>420</v>
-      </c>
-      <c r="B220" s="17" t="s">
-        <v>490</v>
-      </c>
-      <c r="C220" s="17" t="s">
-        <v>491</v>
-      </c>
-      <c r="D220" s="17"/>
-      <c r="E220" s="17"/>
       <c r="F220" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="G220" s="17"/>
-    </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A221" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B221" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="C221" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="F221" s="5" t="s">
-        <v>101</v>
-      </c>
+    </row>
+    <row r="221" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A221" s="17" t="s">
+        <v>420</v>
+      </c>
+      <c r="B221" s="17" t="s">
+        <v>490</v>
+      </c>
+      <c r="C221" s="17" t="s">
+        <v>491</v>
+      </c>
+      <c r="D221" s="17"/>
+      <c r="E221" s="17"/>
+      <c r="F221" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="G221" s="17"/>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>304</v>
+        <v>209</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="E222" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F222" s="12" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="223" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>210</v>
+      </c>
+      <c r="F222" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>211</v>
+        <v>304</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="F223" s="5" t="s">
-        <v>101</v>
+        <v>305</v>
+      </c>
+      <c r="E223" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F223" s="12" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="224" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6818,30 +6824,30 @@
         <v>93</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="F224" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G224" s="2" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
+        <v>212</v>
+      </c>
+      <c r="F224" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A225" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="F225" s="5" t="s">
-        <v>101</v>
+        <v>214</v>
+      </c>
+      <c r="F225" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G225" s="2" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.35">
@@ -6849,10 +6855,10 @@
         <v>93</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>94</v>
+        <v>215</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>97</v>
+        <v>220</v>
       </c>
       <c r="F226" s="5" t="s">
         <v>101</v>
@@ -6863,128 +6869,128 @@
         <v>93</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>216</v>
+        <v>94</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="F227" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="228" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>97</v>
+      </c>
+      <c r="F227" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B228" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="F228" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A229" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B229" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="C228" s="2" t="s">
+      <c r="C229" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="F228" s="12" t="s">
+      <c r="F229" s="12" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="229" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A229" s="17" t="s">
+    <row r="230" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A230" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="B229" s="17" t="s">
+      <c r="B230" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="C229" s="17" t="s">
+      <c r="C230" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D229" s="17"/>
-      <c r="E229" s="17"/>
-      <c r="F229" s="20" t="s">
+      <c r="D230" s="17"/>
+      <c r="E230" s="17"/>
+      <c r="F230" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G229" s="17"/>
-    </row>
-    <row r="230" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A230" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B230" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C230" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F230" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G230" s="2" t="s">
-        <v>331</v>
-      </c>
+      <c r="G230" s="17"/>
     </row>
     <row r="231" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A231" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>192</v>
+        <v>71</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="F231" s="6" t="s">
-        <v>142</v>
+        <v>102</v>
       </c>
       <c r="G231" s="2" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A232" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>741</v>
+        <v>192</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>742</v>
+        <v>194</v>
       </c>
       <c r="F232" s="6" t="s">
         <v>142</v>
       </c>
       <c r="G232" s="2" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A233" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B233" s="2" t="s">
+        <v>741</v>
+      </c>
+      <c r="C233" s="2" t="s">
+        <v>742</v>
+      </c>
+      <c r="F233" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G233" s="2" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="233" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A233" s="17" t="s">
+    <row r="234" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A234" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="B233" s="17" t="s">
+      <c r="B234" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="C233" s="17" t="s">
+      <c r="C234" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="D233" s="17"/>
-      <c r="E233" s="17"/>
-      <c r="F233" s="22" t="s">
+      <c r="D234" s="17"/>
+      <c r="E234" s="17"/>
+      <c r="F234" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="G233" s="17" t="s">
+      <c r="G234" s="17" t="s">
         <v>336</v>
-      </c>
-    </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A234" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B234" s="2" t="s">
-        <v>631</v>
-      </c>
-      <c r="C234" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="F234" s="4" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.35">
@@ -6992,13 +6998,13 @@
         <v>73</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>549</v>
+        <v>631</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>550</v>
-      </c>
-      <c r="F235" s="5" t="s">
-        <v>101</v>
+        <v>632</v>
+      </c>
+      <c r="F235" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.35">
@@ -7006,13 +7012,13 @@
         <v>73</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>74</v>
+        <v>549</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F236" s="4" t="s">
-        <v>100</v>
+        <v>550</v>
+      </c>
+      <c r="F236" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.35">
@@ -7020,41 +7026,41 @@
         <v>73</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F237" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="238" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="F237" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A238" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>553</v>
+        <v>75</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>554</v>
+        <v>83</v>
       </c>
       <c r="F238" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A239" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>411</v>
+        <v>553</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="F239" s="4" t="s">
-        <v>100</v>
+        <v>554</v>
+      </c>
+      <c r="F239" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.35">
@@ -7062,10 +7068,10 @@
         <v>73</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>674</v>
+        <v>411</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>675</v>
+        <v>412</v>
       </c>
       <c r="F240" s="4" t="s">
         <v>100</v>
@@ -7076,13 +7082,13 @@
         <v>73</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>551</v>
+        <v>674</v>
       </c>
       <c r="C241" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="F241" s="5" t="s">
-        <v>101</v>
+        <v>675</v>
+      </c>
+      <c r="F241" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.35">
@@ -7090,13 +7096,13 @@
         <v>73</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>283</v>
+        <v>551</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="F242" s="3" t="s">
-        <v>99</v>
+        <v>552</v>
+      </c>
+      <c r="F242" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.35">
@@ -7104,44 +7110,44 @@
         <v>73</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>256</v>
+        <v>283</v>
       </c>
       <c r="C243" s="2" t="s">
-        <v>257</v>
+        <v>284</v>
       </c>
       <c r="F243" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="244" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A244" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="E244" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="F244" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
+        <v>257</v>
+      </c>
+      <c r="F244" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="245" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A245" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>795</v>
+        <v>236</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>796</v>
-      </c>
-      <c r="F245" s="3" t="s">
-        <v>99</v>
+        <v>237</v>
+      </c>
+      <c r="E245" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="F245" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="246" spans="1:6" x14ac:dyDescent="0.35">
@@ -7149,13 +7155,13 @@
         <v>73</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>617</v>
+        <v>795</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="F246" s="5" t="s">
-        <v>101</v>
+        <v>796</v>
+      </c>
+      <c r="F246" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.35">
@@ -7163,10 +7169,10 @@
         <v>73</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="F247" s="5" t="s">
         <v>101</v>
@@ -7177,10 +7183,10 @@
         <v>73</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>232</v>
+        <v>619</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>233</v>
+        <v>620</v>
       </c>
       <c r="F248" s="5" t="s">
         <v>101</v>
@@ -7191,10 +7197,10 @@
         <v>73</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="F249" s="5" t="s">
         <v>101</v>
@@ -7205,13 +7211,13 @@
         <v>73</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>829</v>
+        <v>228</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>830</v>
-      </c>
-      <c r="F250" s="4" t="s">
-        <v>100</v>
+        <v>229</v>
+      </c>
+      <c r="F250" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.35">
@@ -7219,16 +7225,13 @@
         <v>73</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>633</v>
+        <v>829</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="D251" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="F251" s="5" t="s">
-        <v>101</v>
+        <v>830</v>
+      </c>
+      <c r="F251" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.35">
@@ -7236,13 +7239,16 @@
         <v>73</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>831</v>
+        <v>633</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>832</v>
-      </c>
-      <c r="F252" s="4" t="s">
-        <v>100</v>
+        <v>634</v>
+      </c>
+      <c r="D252" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="F252" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.35">
@@ -7250,13 +7256,13 @@
         <v>73</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>621</v>
+        <v>831</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="F253" s="5" t="s">
-        <v>101</v>
+        <v>832</v>
+      </c>
+      <c r="F253" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.35">
@@ -7264,13 +7270,13 @@
         <v>73</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>814</v>
+        <v>621</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>815</v>
-      </c>
-      <c r="F254" s="3" t="s">
-        <v>99</v>
+        <v>622</v>
+      </c>
+      <c r="F254" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.35">
@@ -7278,10 +7284,10 @@
         <v>73</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>705</v>
+        <v>814</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>706</v>
+        <v>815</v>
       </c>
       <c r="F255" s="3" t="s">
         <v>99</v>
@@ -7292,10 +7298,10 @@
         <v>73</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>636</v>
+        <v>705</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>637</v>
+        <v>706</v>
       </c>
       <c r="F256" s="3" t="s">
         <v>99</v>
@@ -7306,10 +7312,10 @@
         <v>73</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>608</v>
+        <v>636</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>609</v>
+        <v>637</v>
       </c>
       <c r="F257" s="3" t="s">
         <v>99</v>
@@ -7320,13 +7326,13 @@
         <v>73</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>588</v>
+        <v>608</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>589</v>
-      </c>
-      <c r="F258" s="4" t="s">
-        <v>100</v>
+        <v>609</v>
+      </c>
+      <c r="F258" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.35">
@@ -7334,44 +7340,44 @@
         <v>73</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>241</v>
+        <v>588</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>242</v>
+        <v>589</v>
       </c>
       <c r="F259" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="260" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A260" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>285</v>
+        <v>241</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="F260" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="G260" s="2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+      <c r="F260" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A261" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>76</v>
+        <v>285</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F261" s="5" t="s">
-        <v>101</v>
+        <v>286</v>
+      </c>
+      <c r="F261" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="G261" s="2" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.35">
@@ -7379,10 +7385,10 @@
         <v>73</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F262" s="5" t="s">
         <v>101</v>
@@ -7393,10 +7399,10 @@
         <v>73</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F263" s="5" t="s">
         <v>101</v>
@@ -7407,13 +7413,13 @@
         <v>73</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F264" s="4" t="s">
-        <v>100</v>
+        <v>86</v>
+      </c>
+      <c r="F264" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.35">
@@ -7421,16 +7427,13 @@
         <v>73</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>623</v>
+        <v>79</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="D265" s="2" t="s">
-        <v>625</v>
-      </c>
-      <c r="F265" s="5" t="s">
-        <v>101</v>
+        <v>87</v>
+      </c>
+      <c r="F265" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.35">
@@ -7438,13 +7441,16 @@
         <v>73</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>447</v>
+        <v>623</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="F266" s="4" t="s">
-        <v>100</v>
+        <v>624</v>
+      </c>
+      <c r="D266" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="F266" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.35">
@@ -7452,41 +7458,41 @@
         <v>73</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>477</v>
+        <v>447</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>478</v>
+        <v>448</v>
       </c>
       <c r="F267" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="268" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A268" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>638</v>
+        <v>477</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="F268" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.35">
+        <v>478</v>
+      </c>
+      <c r="F268" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="269" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A269" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>735</v>
+        <v>638</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>736</v>
-      </c>
-      <c r="F269" s="3" t="s">
-        <v>99</v>
+        <v>639</v>
+      </c>
+      <c r="F269" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="270" spans="1:7" x14ac:dyDescent="0.35">
@@ -7494,10 +7500,10 @@
         <v>73</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>80</v>
+        <v>735</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>88</v>
+        <v>736</v>
       </c>
       <c r="F270" s="3" t="s">
         <v>99</v>
@@ -7508,30 +7514,27 @@
         <v>73</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>547</v>
+        <v>80</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="F271" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="272" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+      <c r="F271" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="272" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A272" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>293</v>
+        <v>547</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="F272" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G272" s="2" t="s">
-        <v>335</v>
+        <v>548</v>
+      </c>
+      <c r="F272" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="273" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -7539,10 +7542,10 @@
         <v>73</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="F273" s="16" t="s">
         <v>303</v>
@@ -7556,10 +7559,10 @@
         <v>73</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>239</v>
+        <v>295</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>240</v>
+        <v>296</v>
       </c>
       <c r="F274" s="16" t="s">
         <v>303</v>
@@ -7568,35 +7571,38 @@
         <v>335</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A275" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E275" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="F275" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="276" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>240</v>
+      </c>
+      <c r="F275" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G275" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="276" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A276" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>688</v>
+        <v>230</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>689</v>
-      </c>
-      <c r="F276" s="5" t="s">
-        <v>238</v>
+        <v>231</v>
+      </c>
+      <c r="E276" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F276" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="277" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7604,58 +7610,58 @@
         <v>73</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>81</v>
+        <v>688</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F277" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
+        <v>689</v>
+      </c>
+      <c r="F277" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A278" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>739</v>
+        <v>81</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>740</v>
+        <v>89</v>
       </c>
       <c r="F278" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="279" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A279" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>443</v>
+        <v>739</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="F279" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G279" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.35">
+        <v>740</v>
+      </c>
+      <c r="F279" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="280" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A280" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>640</v>
+        <v>443</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="F280" s="5" t="s">
-        <v>101</v>
+        <v>444</v>
+      </c>
+      <c r="F280" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G280" s="2" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.35">
@@ -7663,44 +7669,44 @@
         <v>73</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>506</v>
+        <v>640</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>507</v>
+        <v>641</v>
       </c>
       <c r="F281" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="282" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A282" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>772</v>
+        <v>506</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>773</v>
-      </c>
-      <c r="F282" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G282" s="2" t="s">
-        <v>774</v>
-      </c>
-    </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.35">
+        <v>507</v>
+      </c>
+      <c r="F282" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A283" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>245</v>
+        <v>772</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="F283" s="14" t="s">
-        <v>258</v>
+        <v>773</v>
+      </c>
+      <c r="F283" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G283" s="2" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.35">
@@ -7708,13 +7714,13 @@
         <v>73</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>298</v>
+        <v>245</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="F284" s="5" t="s">
-        <v>101</v>
+        <v>246</v>
+      </c>
+      <c r="F284" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.35">
@@ -7722,13 +7728,13 @@
         <v>73</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>642</v>
+        <v>298</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="F285" s="4" t="s">
-        <v>100</v>
+        <v>297</v>
+      </c>
+      <c r="F285" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="286" spans="1:7" x14ac:dyDescent="0.35">
@@ -7736,13 +7742,13 @@
         <v>73</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>234</v>
+        <v>642</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="F286" s="5" t="s">
-        <v>101</v>
+        <v>643</v>
+      </c>
+      <c r="F286" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.35">
@@ -7750,10 +7756,10 @@
         <v>73</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>626</v>
+        <v>234</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>627</v>
+        <v>235</v>
       </c>
       <c r="F287" s="5" t="s">
         <v>101</v>
@@ -7764,13 +7770,13 @@
         <v>73</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>226</v>
+        <v>626</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="F288" s="12" t="s">
-        <v>250</v>
+        <v>627</v>
+      </c>
+      <c r="F288" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.35">
@@ -7778,13 +7784,13 @@
         <v>73</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>523</v>
+        <v>226</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="F289" s="14" t="s">
-        <v>258</v>
+        <v>227</v>
+      </c>
+      <c r="F289" s="12" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.35">
@@ -7792,16 +7798,13 @@
         <v>73</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="E290" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="F290" s="5" t="s">
-        <v>101</v>
+        <v>524</v>
+      </c>
+      <c r="F290" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.35">
@@ -7809,44 +7812,44 @@
         <v>73</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>224</v>
+        <v>521</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>225</v>
+        <v>522</v>
+      </c>
+      <c r="E291" s="2" t="s">
+        <v>226</v>
       </c>
       <c r="F291" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="292" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A292" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>644</v>
+        <v>224</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>645</v>
-      </c>
-      <c r="F292" s="20" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="293" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>225</v>
+      </c>
+      <c r="F292" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A293" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="F293" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G293" s="2" t="s">
-        <v>586</v>
+        <v>645</v>
+      </c>
+      <c r="F293" s="20" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="294" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7854,81 +7857,81 @@
         <v>73</v>
       </c>
       <c r="B294" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="C294" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="F294" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G294" s="2" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="295" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A295" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B295" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="C294" s="2" t="s">
+      <c r="C295" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="F294" s="16" t="s">
+      <c r="F295" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="G294" s="2" t="s">
+      <c r="G295" s="2" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="295" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A295" s="17" t="s">
+    <row r="296" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A296" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B295" s="17" t="s">
+      <c r="B296" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="C295" s="17" t="s">
+      <c r="C296" s="17" t="s">
         <v>307</v>
       </c>
-      <c r="D295" s="17"/>
-      <c r="E295" s="17"/>
-      <c r="F295" s="20" t="s">
+      <c r="D296" s="17"/>
+      <c r="E296" s="17"/>
+      <c r="F296" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G295" s="17"/>
-    </row>
-    <row r="296" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A296" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B296" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C296" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D296" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="F296" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G296" s="17"/>
+    </row>
+    <row r="297" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A297" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>222</v>
+        <v>91</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>221</v>
+        <v>92</v>
       </c>
       <c r="D297" s="2" t="s">
-        <v>403</v>
+        <v>315</v>
       </c>
       <c r="F297" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="298" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A298" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>247</v>
+        <v>222</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>248</v>
+        <v>221</v>
       </c>
       <c r="D298" s="2" t="s">
-        <v>249</v>
+        <v>403</v>
       </c>
       <c r="F298" s="5" t="s">
         <v>101</v>
@@ -7939,27 +7942,30 @@
         <v>90</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>797</v>
+        <v>247</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>798</v>
-      </c>
-      <c r="F299" s="25" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
+        <v>248</v>
+      </c>
+      <c r="D299" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="F299" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A300" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>351</v>
+        <v>797</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="F300" s="4" t="s">
-        <v>100</v>
+        <v>798</v>
+      </c>
+      <c r="F300" s="25" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="301" spans="1:7" x14ac:dyDescent="0.35">
@@ -7967,36 +7973,50 @@
         <v>90</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>563</v>
+        <v>351</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="D301" s="2" t="s">
-        <v>565</v>
+        <v>352</v>
       </c>
       <c r="F301" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="302" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A302" s="17" t="s">
+    <row r="302" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A302" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B302" s="17" t="s">
+      <c r="B302" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C302" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="D302" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="F302" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="303" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A303" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B303" s="17" t="s">
         <v>291</v>
       </c>
-      <c r="C302" s="17" t="s">
+      <c r="C303" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="D302" s="17" t="s">
+      <c r="D303" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="E302" s="17"/>
-      <c r="F302" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="G302" s="17"/>
+      <c r="E303" s="17"/>
+      <c r="F303" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G303" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Change the binding hour in the reliability mechanism to be based off hourly demand before load shifting, with an adjustment for the MW load shifting capacity available
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FCE50AF-4C8E-4775-9637-E8E8FCB2BF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05E678C4-344F-464B-B0C7-135154764FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1448" uniqueCount="839">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1452" uniqueCount="841">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2549,6 +2549,12 @@
   </si>
   <si>
     <t>Bool Use Cap Life for Retirements</t>
+  </si>
+  <si>
+    <t>AVCC</t>
+  </si>
+  <si>
+    <t>Avg Vehicle Charger Capacity</t>
   </si>
 </sst>
 </file>
@@ -3360,7 +3366,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G305"/>
+  <dimension ref="A1:G306"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
@@ -7052,13 +7058,13 @@
         <v>73</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>549</v>
+        <v>839</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>550</v>
-      </c>
-      <c r="F238" s="5" t="s">
-        <v>101</v>
+        <v>840</v>
+      </c>
+      <c r="F238" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.35">
@@ -7066,13 +7072,13 @@
         <v>73</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>74</v>
+        <v>549</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F239" s="4" t="s">
-        <v>100</v>
+        <v>550</v>
+      </c>
+      <c r="F239" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.35">
@@ -7080,41 +7086,41 @@
         <v>73</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F240" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="241" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="F240" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="241" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A241" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>553</v>
+        <v>75</v>
       </c>
       <c r="C241" s="2" t="s">
-        <v>554</v>
+        <v>83</v>
       </c>
       <c r="F241" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A242" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>411</v>
+        <v>553</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="F242" s="4" t="s">
-        <v>100</v>
+        <v>554</v>
+      </c>
+      <c r="F242" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.35">
@@ -7122,10 +7128,10 @@
         <v>73</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>674</v>
+        <v>411</v>
       </c>
       <c r="C243" s="2" t="s">
-        <v>675</v>
+        <v>412</v>
       </c>
       <c r="F243" s="4" t="s">
         <v>100</v>
@@ -7136,13 +7142,13 @@
         <v>73</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>551</v>
+        <v>674</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="F244" s="5" t="s">
-        <v>101</v>
+        <v>675</v>
+      </c>
+      <c r="F244" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="245" spans="1:6" x14ac:dyDescent="0.35">
@@ -7150,13 +7156,13 @@
         <v>73</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>283</v>
+        <v>551</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="F245" s="3" t="s">
-        <v>99</v>
+        <v>552</v>
+      </c>
+      <c r="F245" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="246" spans="1:6" x14ac:dyDescent="0.35">
@@ -7164,44 +7170,44 @@
         <v>73</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>256</v>
+        <v>283</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>257</v>
+        <v>284</v>
       </c>
       <c r="F246" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="247" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A247" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="E247" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="F247" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.35">
+        <v>257</v>
+      </c>
+      <c r="F247" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="248" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A248" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>795</v>
+        <v>236</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>796</v>
-      </c>
-      <c r="F248" s="3" t="s">
-        <v>99</v>
+        <v>237</v>
+      </c>
+      <c r="E248" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="F248" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="249" spans="1:6" x14ac:dyDescent="0.35">
@@ -7209,13 +7215,13 @@
         <v>73</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>617</v>
+        <v>795</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="F249" s="5" t="s">
-        <v>101</v>
+        <v>796</v>
+      </c>
+      <c r="F249" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.35">
@@ -7223,10 +7229,10 @@
         <v>73</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="F250" s="5" t="s">
         <v>101</v>
@@ -7237,10 +7243,10 @@
         <v>73</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>232</v>
+        <v>619</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>233</v>
+        <v>620</v>
       </c>
       <c r="F251" s="5" t="s">
         <v>101</v>
@@ -7251,10 +7257,10 @@
         <v>73</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="F252" s="5" t="s">
         <v>101</v>
@@ -7265,13 +7271,13 @@
         <v>73</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>829</v>
+        <v>228</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>830</v>
-      </c>
-      <c r="F253" s="4" t="s">
-        <v>100</v>
+        <v>229</v>
+      </c>
+      <c r="F253" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.35">
@@ -7279,16 +7285,13 @@
         <v>73</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>633</v>
+        <v>829</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="D254" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="F254" s="5" t="s">
-        <v>101</v>
+        <v>830</v>
+      </c>
+      <c r="F254" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.35">
@@ -7296,13 +7299,16 @@
         <v>73</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>831</v>
+        <v>633</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>832</v>
-      </c>
-      <c r="F255" s="4" t="s">
-        <v>100</v>
+        <v>634</v>
+      </c>
+      <c r="D255" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="F255" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.35">
@@ -7310,13 +7316,13 @@
         <v>73</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>621</v>
+        <v>831</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="F256" s="5" t="s">
-        <v>101</v>
+        <v>832</v>
+      </c>
+      <c r="F256" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.35">
@@ -7324,13 +7330,13 @@
         <v>73</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>814</v>
+        <v>621</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>815</v>
-      </c>
-      <c r="F257" s="3" t="s">
-        <v>99</v>
+        <v>622</v>
+      </c>
+      <c r="F257" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.35">
@@ -7338,10 +7344,10 @@
         <v>73</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>705</v>
+        <v>814</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>706</v>
+        <v>815</v>
       </c>
       <c r="F258" s="3" t="s">
         <v>99</v>
@@ -7352,10 +7358,10 @@
         <v>73</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>636</v>
+        <v>705</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>637</v>
+        <v>706</v>
       </c>
       <c r="F259" s="3" t="s">
         <v>99</v>
@@ -7366,10 +7372,10 @@
         <v>73</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>608</v>
+        <v>636</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>609</v>
+        <v>637</v>
       </c>
       <c r="F260" s="3" t="s">
         <v>99</v>
@@ -7380,13 +7386,13 @@
         <v>73</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>588</v>
+        <v>608</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>589</v>
-      </c>
-      <c r="F261" s="4" t="s">
-        <v>100</v>
+        <v>609</v>
+      </c>
+      <c r="F261" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.35">
@@ -7394,44 +7400,44 @@
         <v>73</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>241</v>
+        <v>588</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>242</v>
+        <v>589</v>
       </c>
       <c r="F262" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="263" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A263" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>285</v>
+        <v>241</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="F263" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="G263" s="2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+      <c r="F263" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="264" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A264" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>76</v>
+        <v>285</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F264" s="5" t="s">
-        <v>101</v>
+        <v>286</v>
+      </c>
+      <c r="F264" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="G264" s="2" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.35">
@@ -7439,10 +7445,10 @@
         <v>73</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F265" s="5" t="s">
         <v>101</v>
@@ -7453,10 +7459,10 @@
         <v>73</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F266" s="5" t="s">
         <v>101</v>
@@ -7467,13 +7473,13 @@
         <v>73</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F267" s="4" t="s">
-        <v>100</v>
+        <v>86</v>
+      </c>
+      <c r="F267" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.35">
@@ -7481,16 +7487,13 @@
         <v>73</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>623</v>
+        <v>79</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="D268" s="2" t="s">
-        <v>625</v>
-      </c>
-      <c r="F268" s="5" t="s">
-        <v>101</v>
+        <v>87</v>
+      </c>
+      <c r="F268" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.35">
@@ -7498,13 +7501,16 @@
         <v>73</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>447</v>
+        <v>623</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="F269" s="4" t="s">
-        <v>100</v>
+        <v>624</v>
+      </c>
+      <c r="D269" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="F269" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="270" spans="1:7" x14ac:dyDescent="0.35">
@@ -7512,41 +7518,41 @@
         <v>73</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>477</v>
+        <v>447</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>478</v>
+        <v>448</v>
       </c>
       <c r="F270" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="271" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A271" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>638</v>
+        <v>477</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="F271" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.35">
+        <v>478</v>
+      </c>
+      <c r="F271" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="272" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A272" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>735</v>
+        <v>638</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>736</v>
-      </c>
-      <c r="F272" s="3" t="s">
-        <v>99</v>
+        <v>639</v>
+      </c>
+      <c r="F272" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.35">
@@ -7554,10 +7560,10 @@
         <v>73</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>80</v>
+        <v>735</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>88</v>
+        <v>736</v>
       </c>
       <c r="F273" s="3" t="s">
         <v>99</v>
@@ -7568,30 +7574,27 @@
         <v>73</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>547</v>
+        <v>80</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="F274" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="275" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+      <c r="F274" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A275" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>293</v>
+        <v>547</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="F275" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G275" s="2" t="s">
-        <v>335</v>
+        <v>548</v>
+      </c>
+      <c r="F275" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="276" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -7599,10 +7602,10 @@
         <v>73</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="F276" s="16" t="s">
         <v>303</v>
@@ -7616,10 +7619,10 @@
         <v>73</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>239</v>
+        <v>295</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>240</v>
+        <v>296</v>
       </c>
       <c r="F277" s="16" t="s">
         <v>303</v>
@@ -7628,35 +7631,38 @@
         <v>335</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A278" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E278" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="F278" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="279" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>240</v>
+      </c>
+      <c r="F278" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G278" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A279" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>688</v>
+        <v>230</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>689</v>
-      </c>
-      <c r="F279" s="5" t="s">
-        <v>238</v>
+        <v>231</v>
+      </c>
+      <c r="E279" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F279" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="280" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7664,58 +7670,58 @@
         <v>73</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>81</v>
+        <v>688</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F280" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
+        <v>689</v>
+      </c>
+      <c r="F280" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A281" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>739</v>
+        <v>81</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>740</v>
+        <v>89</v>
       </c>
       <c r="F281" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="282" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A282" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>443</v>
+        <v>739</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="F282" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G282" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.35">
+        <v>740</v>
+      </c>
+      <c r="F282" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A283" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>640</v>
+        <v>443</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="F283" s="5" t="s">
-        <v>101</v>
+        <v>444</v>
+      </c>
+      <c r="F283" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G283" s="2" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.35">
@@ -7723,44 +7729,44 @@
         <v>73</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>506</v>
+        <v>640</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>507</v>
+        <v>641</v>
       </c>
       <c r="F284" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="285" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A285" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>772</v>
+        <v>506</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>773</v>
-      </c>
-      <c r="F285" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="G285" s="2" t="s">
-        <v>774</v>
-      </c>
-    </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.35">
+        <v>507</v>
+      </c>
+      <c r="F285" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A286" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>245</v>
+        <v>772</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="F286" s="14" t="s">
-        <v>258</v>
+        <v>773</v>
+      </c>
+      <c r="F286" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="G286" s="2" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.35">
@@ -7768,13 +7774,13 @@
         <v>73</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>298</v>
+        <v>245</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="F287" s="5" t="s">
-        <v>101</v>
+        <v>246</v>
+      </c>
+      <c r="F287" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.35">
@@ -7782,13 +7788,13 @@
         <v>73</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>642</v>
+        <v>298</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="F288" s="4" t="s">
-        <v>100</v>
+        <v>297</v>
+      </c>
+      <c r="F288" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.35">
@@ -7796,13 +7802,13 @@
         <v>73</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>234</v>
+        <v>642</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="F289" s="5" t="s">
-        <v>101</v>
+        <v>643</v>
+      </c>
+      <c r="F289" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.35">
@@ -7810,10 +7816,10 @@
         <v>73</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>626</v>
+        <v>234</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>627</v>
+        <v>235</v>
       </c>
       <c r="F290" s="5" t="s">
         <v>101</v>
@@ -7824,13 +7830,13 @@
         <v>73</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>226</v>
+        <v>626</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="F291" s="12" t="s">
-        <v>250</v>
+        <v>627</v>
+      </c>
+      <c r="F291" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.35">
@@ -7838,13 +7844,13 @@
         <v>73</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>523</v>
+        <v>226</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="F292" s="14" t="s">
-        <v>258</v>
+        <v>227</v>
+      </c>
+      <c r="F292" s="12" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.35">
@@ -7852,16 +7858,13 @@
         <v>73</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="E293" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="F293" s="5" t="s">
-        <v>101</v>
+        <v>524</v>
+      </c>
+      <c r="F293" s="14" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="294" spans="1:7" x14ac:dyDescent="0.35">
@@ -7869,44 +7872,44 @@
         <v>73</v>
       </c>
       <c r="B294" s="2" t="s">
-        <v>224</v>
+        <v>521</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>225</v>
+        <v>522</v>
+      </c>
+      <c r="E294" s="2" t="s">
+        <v>226</v>
       </c>
       <c r="F294" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="295" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A295" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>644</v>
+        <v>224</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>645</v>
-      </c>
-      <c r="F295" s="20" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="296" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>225</v>
+      </c>
+      <c r="F295" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="296" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A296" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="F296" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G296" s="2" t="s">
-        <v>586</v>
+        <v>645</v>
+      </c>
+      <c r="F296" s="20" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="297" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7914,81 +7917,81 @@
         <v>73</v>
       </c>
       <c r="B297" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="C297" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="F297" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G297" s="2" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A298" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B298" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="C297" s="2" t="s">
+      <c r="C298" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="F297" s="16" t="s">
+      <c r="F298" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="G297" s="2" t="s">
+      <c r="G298" s="2" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="298" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A298" s="17" t="s">
+    <row r="299" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A299" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B298" s="17" t="s">
+      <c r="B299" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="C298" s="17" t="s">
+      <c r="C299" s="17" t="s">
         <v>307</v>
       </c>
-      <c r="D298" s="17"/>
-      <c r="E298" s="17"/>
-      <c r="F298" s="20" t="s">
+      <c r="D299" s="17"/>
+      <c r="E299" s="17"/>
+      <c r="F299" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G298" s="17"/>
-    </row>
-    <row r="299" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A299" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B299" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C299" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D299" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="F299" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G299" s="17"/>
+    </row>
+    <row r="300" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A300" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>222</v>
+        <v>91</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>221</v>
+        <v>92</v>
       </c>
       <c r="D300" s="2" t="s">
-        <v>403</v>
+        <v>315</v>
       </c>
       <c r="F300" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="301" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A301" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>247</v>
+        <v>222</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>248</v>
+        <v>221</v>
       </c>
       <c r="D301" s="2" t="s">
-        <v>249</v>
+        <v>403</v>
       </c>
       <c r="F301" s="5" t="s">
         <v>101</v>
@@ -7999,27 +8002,30 @@
         <v>90</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>797</v>
+        <v>247</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>798</v>
-      </c>
-      <c r="F302" s="25" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.35">
+        <v>248</v>
+      </c>
+      <c r="D302" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="F302" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="303" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A303" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>351</v>
+        <v>797</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="F303" s="4" t="s">
-        <v>100</v>
+        <v>798</v>
+      </c>
+      <c r="F303" s="25" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="304" spans="1:7" x14ac:dyDescent="0.35">
@@ -8027,36 +8033,50 @@
         <v>90</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>563</v>
+        <v>351</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="D304" s="2" t="s">
-        <v>565</v>
+        <v>352</v>
       </c>
       <c r="F304" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="305" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A305" s="17" t="s">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A305" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B305" s="17" t="s">
+      <c r="B305" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C305" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="D305" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="F305" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="306" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A306" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B306" s="17" t="s">
         <v>291</v>
       </c>
-      <c r="C305" s="17" t="s">
+      <c r="C306" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="D305" s="17" t="s">
+      <c r="D306" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="E305" s="17"/>
-      <c r="F305" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="G305" s="17"/>
+      <c r="E306" s="17"/>
+      <c r="F306" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G306" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Adds AVCC to key
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269C63F9-B54A-4174-91B3-9FBC835E562E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F6A0BF-6443-4E4C-917E-19DAE8485170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="1260" windowWidth="21120" windowHeight="14655" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5070" yWindow="1125" windowWidth="21600" windowHeight="11235" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1627" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1631" uniqueCount="933">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2825,6 +2825,12 @@
   </si>
   <si>
     <t>Battery Pack Price Multiplier</t>
+  </si>
+  <si>
+    <t>AVCC</t>
+  </si>
+  <si>
+    <t>Avg Vehicle Charger Capacity</t>
   </si>
 </sst>
 </file>
@@ -2933,7 +2939,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2994,52 +3000,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3682,7 +3642,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G348"/>
+  <dimension ref="A1:G349"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" style="2" customWidth="1"/>
@@ -4235,7 +4195,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>9</v>
       </c>
@@ -4249,7 +4209,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>9</v>
       </c>
@@ -4759,69 +4719,66 @@
       <c r="C68" s="2" t="s">
         <v>803</v>
       </c>
-      <c r="F68" s="27" t="s">
+      <c r="F68" s="6" t="s">
         <v>178</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="69" spans="1:7" s="26" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A69" s="26" t="s">
+    <row r="69" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="B69" s="26" t="s">
+      <c r="B69" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="C69" s="26" t="s">
+      <c r="C69" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="D69" s="26" t="s">
+      <c r="D69" s="2" t="s">
         <v>682</v>
       </c>
-      <c r="F69" s="27" t="s">
+      <c r="F69" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="G69" s="26" t="s">
+      <c r="G69" s="2" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="70" spans="1:7" s="26" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A70" s="26" t="s">
+    <row r="70" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="B70" s="26" t="s">
+      <c r="B70" s="2" t="s">
         <v>856</v>
       </c>
-      <c r="C70" s="26" t="s">
+      <c r="C70" s="2" t="s">
         <v>857</v>
       </c>
-      <c r="E70" s="26" t="s">
+      <c r="E70" s="2" t="s">
         <v>859</v>
       </c>
-      <c r="F70" s="28" t="s">
+      <c r="F70" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G70" s="26" t="s">
+      <c r="G70" s="2" t="s">
         <v>858</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="26" t="s">
+      <c r="A71" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="B71" s="26" t="s">
+      <c r="B71" s="2" t="s">
         <v>861</v>
       </c>
-      <c r="C71" s="26" t="s">
+      <c r="C71" s="2" t="s">
         <v>863</v>
       </c>
-      <c r="D71" s="26"/>
-      <c r="E71" s="26"/>
       <c r="F71" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="G71" s="26"/>
     </row>
     <row r="72" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="17" t="s">
@@ -5983,21 +5940,21 @@
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A148" s="31" t="s">
+      <c r="A148" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B148" s="31" t="s">
+      <c r="B148" s="2" t="s">
         <v>869</v>
       </c>
-      <c r="C148" s="31" t="s">
+      <c r="C148" s="2" t="s">
         <v>870</v>
       </c>
-      <c r="D148" s="30"/>
-      <c r="E148" s="30"/>
-      <c r="F148" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="G148" s="30"/>
+      <c r="D148"/>
+      <c r="E148"/>
+      <c r="F148" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="G148"/>
     </row>
     <row r="149" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A149" s="17" t="s">
@@ -6096,7 +6053,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="155" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>269</v>
       </c>
@@ -6214,17 +6171,17 @@
         <v>97</v>
       </c>
     </row>
-    <row r="163" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A163" s="31" t="s">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B163" s="31" t="s">
+      <c r="B163" s="2" t="s">
         <v>871</v>
       </c>
-      <c r="C163" s="31" t="s">
+      <c r="C163" s="2" t="s">
         <v>872</v>
       </c>
-      <c r="F163" s="33" t="s">
+      <c r="F163" s="4" t="s">
         <v>98</v>
       </c>
     </row>
@@ -6476,20 +6433,20 @@
         <v>97</v>
       </c>
     </row>
-    <row r="180" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A180" s="31" t="s">
+    <row r="180" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A180" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B180" s="31" t="s">
+      <c r="B180" s="2" t="s">
         <v>873</v>
       </c>
-      <c r="C180" s="31" t="s">
+      <c r="C180" s="2" t="s">
         <v>874</v>
       </c>
-      <c r="F180" s="37" t="s">
+      <c r="F180" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G180" s="31" t="s">
+      <c r="G180" s="2" t="s">
         <v>875</v>
       </c>
     </row>
@@ -6558,17 +6515,17 @@
         <v>99</v>
       </c>
     </row>
-    <row r="185" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A185" s="31" t="s">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A185" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B185" s="31" t="s">
+      <c r="B185" s="2" t="s">
         <v>878</v>
       </c>
-      <c r="C185" s="31" t="s">
+      <c r="C185" s="2" t="s">
         <v>879</v>
       </c>
-      <c r="F185" s="29" t="s">
+      <c r="F185" s="3" t="s">
         <v>97</v>
       </c>
     </row>
@@ -6600,17 +6557,17 @@
         <v>98</v>
       </c>
     </row>
-    <row r="188" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A188" s="31" t="s">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B188" s="31" t="s">
+      <c r="B188" s="2" t="s">
         <v>880</v>
       </c>
-      <c r="C188" s="31" t="s">
+      <c r="C188" s="2" t="s">
         <v>881</v>
       </c>
-      <c r="F188" s="34" t="s">
+      <c r="F188" s="5" t="s">
         <v>99</v>
       </c>
     </row>
@@ -6631,17 +6588,17 @@
         <v>98</v>
       </c>
     </row>
-    <row r="190" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="31" t="s">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A190" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B190" s="31" t="s">
+      <c r="B190" s="2" t="s">
         <v>882</v>
       </c>
-      <c r="C190" s="31" t="s">
+      <c r="C190" s="2" t="s">
         <v>883</v>
       </c>
-      <c r="F190" s="34" t="s">
+      <c r="F190" s="5" t="s">
         <v>99</v>
       </c>
     </row>
@@ -6659,17 +6616,17 @@
         <v>98</v>
       </c>
     </row>
-    <row r="192" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A192" s="31" t="s">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A192" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B192" s="31" t="s">
+      <c r="B192" s="2" t="s">
         <v>884</v>
       </c>
-      <c r="C192" s="31" t="s">
+      <c r="C192" s="2" t="s">
         <v>885</v>
       </c>
-      <c r="F192" s="36" t="s">
+      <c r="F192" s="14" t="s">
         <v>252</v>
       </c>
     </row>
@@ -6683,80 +6640,80 @@
       <c r="C193" s="2" t="s">
         <v>887</v>
       </c>
-      <c r="F193" s="37" t="s">
+      <c r="F193" s="16" t="s">
         <v>291</v>
       </c>
       <c r="G193" s="2" t="s">
         <v>888</v>
       </c>
     </row>
-    <row r="194" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A194" s="31" t="s">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A194" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B194" s="31" t="s">
+      <c r="B194" s="2" t="s">
         <v>889</v>
       </c>
-      <c r="C194" s="31" t="s">
+      <c r="C194" s="2" t="s">
         <v>890</v>
       </c>
-      <c r="F194" s="34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="195" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A195" s="31" t="s">
+      <c r="F194" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A195" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B195" s="31" t="s">
+      <c r="B195" s="2" t="s">
         <v>891</v>
       </c>
-      <c r="C195" s="31" t="s">
+      <c r="C195" s="2" t="s">
         <v>892</v>
       </c>
-      <c r="F195" s="34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="196" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A196" s="31" t="s">
+      <c r="F195" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A196" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B196" s="31" t="s">
+      <c r="B196" s="2" t="s">
         <v>895</v>
       </c>
-      <c r="C196" s="31" t="s">
+      <c r="C196" s="2" t="s">
         <v>896</v>
       </c>
-      <c r="F196" s="34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="197" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A197" s="31" t="s">
+      <c r="F196" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A197" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B197" s="31" t="s">
+      <c r="B197" s="2" t="s">
         <v>897</v>
       </c>
-      <c r="C197" s="31" t="s">
+      <c r="C197" s="2" t="s">
         <v>898</v>
       </c>
-      <c r="F197" s="33" t="s">
+      <c r="F197" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="198" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A198" s="31" t="s">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A198" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B198" s="31" t="s">
+      <c r="B198" s="2" t="s">
         <v>893</v>
       </c>
-      <c r="C198" s="31" t="s">
+      <c r="C198" s="2" t="s">
         <v>894</v>
       </c>
-      <c r="F198" s="35" t="s">
+      <c r="F198" s="12" t="s">
         <v>244</v>
       </c>
     </row>
@@ -6770,7 +6727,7 @@
       <c r="C199" s="17" t="s">
         <v>900</v>
       </c>
-      <c r="F199" s="39" t="s">
+      <c r="F199" s="20" t="s">
         <v>98</v>
       </c>
     </row>
@@ -6822,20 +6779,20 @@
         <v>851</v>
       </c>
     </row>
-    <row r="203" spans="1:7" s="31" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A203" s="31" t="s">
+    <row r="203" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A203" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B203" s="31" t="s">
+      <c r="B203" s="2" t="s">
         <v>901</v>
       </c>
-      <c r="C203" s="31" t="s">
+      <c r="C203" s="2" t="s">
         <v>902</v>
       </c>
-      <c r="F203" s="37" t="s">
+      <c r="F203" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G203" s="31" t="s">
+      <c r="G203" s="2" t="s">
         <v>903</v>
       </c>
     </row>
@@ -6884,17 +6841,17 @@
         <v>244</v>
       </c>
     </row>
-    <row r="207" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A207" s="31" t="s">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A207" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B207" s="31" t="s">
+      <c r="B207" s="2" t="s">
         <v>904</v>
       </c>
-      <c r="C207" s="31" t="s">
+      <c r="C207" s="2" t="s">
         <v>905</v>
       </c>
-      <c r="F207" s="32" t="s">
+      <c r="F207" s="3" t="s">
         <v>97</v>
       </c>
     </row>
@@ -6974,17 +6931,17 @@
         <v>98</v>
       </c>
     </row>
-    <row r="213" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A213" s="31" t="s">
+    <row r="213" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A213" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B213" s="31" t="s">
+      <c r="B213" s="2" t="s">
         <v>906</v>
       </c>
-      <c r="C213" s="31" t="s">
+      <c r="C213" s="2" t="s">
         <v>907</v>
       </c>
-      <c r="F213" s="34" t="s">
+      <c r="F213" s="5" t="s">
         <v>99</v>
       </c>
     </row>
@@ -7033,17 +6990,17 @@
         <v>252</v>
       </c>
     </row>
-    <row r="217" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A217" s="31" t="s">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A217" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B217" s="31" t="s">
+      <c r="B217" s="2" t="s">
         <v>908</v>
       </c>
-      <c r="C217" s="31" t="s">
+      <c r="C217" s="2" t="s">
         <v>909</v>
       </c>
-      <c r="F217" s="36" t="s">
+      <c r="F217" s="14" t="s">
         <v>252</v>
       </c>
     </row>
@@ -7140,17 +7097,17 @@
         <v>485</v>
       </c>
     </row>
-    <row r="224" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A224" s="31" t="s">
+    <row r="224" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A224" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B224" s="31" t="s">
+      <c r="B224" s="2" t="s">
         <v>910</v>
       </c>
-      <c r="C224" s="31" t="s">
+      <c r="C224" s="2" t="s">
         <v>911</v>
       </c>
-      <c r="F224" s="33" t="s">
+      <c r="F224" s="4" t="s">
         <v>98</v>
       </c>
     </row>
@@ -7185,20 +7142,20 @@
         <v>98</v>
       </c>
     </row>
-    <row r="227" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A227" s="31" t="s">
+    <row r="227" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A227" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B227" s="31" t="s">
+      <c r="B227" s="2" t="s">
         <v>912</v>
       </c>
-      <c r="C227" s="31" t="s">
+      <c r="C227" s="2" t="s">
         <v>913</v>
       </c>
-      <c r="F227" s="37" t="s">
+      <c r="F227" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G227" s="31" t="s">
+      <c r="G227" s="2" t="s">
         <v>914</v>
       </c>
     </row>
@@ -7253,17 +7210,17 @@
         <v>98</v>
       </c>
     </row>
-    <row r="231" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A231" s="31" t="s">
+    <row r="231" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A231" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B231" s="31" t="s">
+      <c r="B231" s="2" t="s">
         <v>915</v>
       </c>
-      <c r="C231" s="31" t="s">
+      <c r="C231" s="2" t="s">
         <v>916</v>
       </c>
-      <c r="F231" s="33" t="s">
+      <c r="F231" s="4" t="s">
         <v>98</v>
       </c>
     </row>
@@ -7291,7 +7248,7 @@
       <c r="C233" s="2" t="s">
         <v>786</v>
       </c>
-      <c r="F233" s="34" t="s">
+      <c r="F233" s="5" t="s">
         <v>99</v>
       </c>
     </row>
@@ -7337,17 +7294,17 @@
         <v>99</v>
       </c>
     </row>
-    <row r="237" spans="1:7" s="31" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A237" s="31" t="s">
+    <row r="237" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A237" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B237" s="31" t="s">
+      <c r="B237" s="2" t="s">
         <v>917</v>
       </c>
-      <c r="C237" s="31" t="s">
+      <c r="C237" s="2" t="s">
         <v>918</v>
       </c>
-      <c r="F237" s="34" t="s">
+      <c r="F237" s="5" t="s">
         <v>99</v>
       </c>
     </row>
@@ -7365,31 +7322,31 @@
         <v>98</v>
       </c>
     </row>
-    <row r="239" spans="1:7" s="26" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A239" s="26" t="s">
+    <row r="239" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A239" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B239" s="26" t="s">
+      <c r="B239" s="2" t="s">
         <v>800</v>
       </c>
-      <c r="C239" s="26" t="s">
+      <c r="C239" s="2" t="s">
         <v>801</v>
       </c>
-      <c r="F239" s="29" t="s">
+      <c r="F239" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="240" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A240" s="26" t="s">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A240" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B240" s="26" t="s">
+      <c r="B240" s="2" t="s">
         <v>919</v>
       </c>
-      <c r="C240" s="26" t="s">
+      <c r="C240" s="2" t="s">
         <v>922</v>
       </c>
-      <c r="F240" s="40" t="s">
+      <c r="F240" s="5" t="s">
         <v>99</v>
       </c>
     </row>
@@ -7405,7 +7362,7 @@
       </c>
       <c r="D241" s="17"/>
       <c r="E241" s="17"/>
-      <c r="F241" s="38" t="s">
+      <c r="F241" s="18" t="s">
         <v>99</v>
       </c>
       <c r="G241" s="17"/>
@@ -7932,20 +7889,20 @@
         <v>707</v>
       </c>
     </row>
-    <row r="276" spans="1:7" s="26" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A276" s="26" t="s">
+    <row r="276" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A276" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B276" s="26" t="s">
+      <c r="B276" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="C276" s="26" t="s">
+      <c r="C276" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="F276" s="27" t="s">
+      <c r="F276" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="G276" s="26" t="s">
+      <c r="G276" s="2" t="s">
         <v>322</v>
       </c>
     </row>
@@ -7980,17 +7937,17 @@
         <v>98</v>
       </c>
     </row>
-    <row r="279" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A279" s="31" t="s">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A279" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B279" s="31" t="s">
+      <c r="B279" s="2" t="s">
         <v>925</v>
       </c>
-      <c r="C279" s="31" t="s">
+      <c r="C279" s="2" t="s">
         <v>926</v>
       </c>
-      <c r="F279" s="36" t="s">
+      <c r="F279" s="14" t="s">
         <v>252</v>
       </c>
     </row>
@@ -7999,13 +7956,13 @@
         <v>71</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>515</v>
+        <v>931</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="F280" s="5" t="s">
-        <v>99</v>
+        <v>932</v>
+      </c>
+      <c r="F280" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.25">
@@ -8013,13 +7970,13 @@
         <v>71</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>72</v>
+        <v>515</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F281" s="4" t="s">
-        <v>98</v>
+        <v>516</v>
+      </c>
+      <c r="F281" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.25">
@@ -8027,41 +7984,41 @@
         <v>71</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="F282" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="283" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="F282" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A283" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>519</v>
+        <v>73</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>520</v>
+        <v>81</v>
       </c>
       <c r="F283" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A284" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>383</v>
+        <v>519</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="F284" s="4" t="s">
-        <v>98</v>
+        <v>520</v>
+      </c>
+      <c r="F284" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.25">
@@ -8069,10 +8026,10 @@
         <v>71</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>639</v>
+        <v>383</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>640</v>
+        <v>384</v>
       </c>
       <c r="F285" s="4" t="s">
         <v>98</v>
@@ -8083,13 +8040,13 @@
         <v>71</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>517</v>
+        <v>639</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="F286" s="5" t="s">
-        <v>99</v>
+        <v>640</v>
+      </c>
+      <c r="F286" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.25">
@@ -8097,13 +8054,13 @@
         <v>71</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>271</v>
+        <v>517</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="F287" s="3" t="s">
-        <v>97</v>
+        <v>518</v>
+      </c>
+      <c r="F287" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.25">
@@ -8111,44 +8068,44 @@
         <v>71</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>250</v>
+        <v>271</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="F288" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="289" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A289" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E289" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="F289" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
+        <v>251</v>
+      </c>
+      <c r="F289" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>763</v>
+        <v>230</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>764</v>
-      </c>
-      <c r="F290" s="3" t="s">
-        <v>97</v>
+        <v>231</v>
+      </c>
+      <c r="E290" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="F290" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="291" spans="1:6" x14ac:dyDescent="0.25">
@@ -8156,13 +8113,13 @@
         <v>71</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>583</v>
+        <v>763</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="F291" s="5" t="s">
-        <v>99</v>
+        <v>764</v>
+      </c>
+      <c r="F291" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="292" spans="1:6" x14ac:dyDescent="0.25">
@@ -8170,10 +8127,10 @@
         <v>71</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="F292" s="5" t="s">
         <v>99</v>
@@ -8184,26 +8141,26 @@
         <v>71</v>
       </c>
       <c r="B293" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="C293" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="F293" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A294" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B294" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="C293" s="2" t="s">
+      <c r="C294" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="F293" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="294" spans="1:6" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A294" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="B294" s="31" t="s">
-        <v>927</v>
-      </c>
-      <c r="C294" s="31" t="s">
-        <v>928</v>
-      </c>
-      <c r="F294" s="34" t="s">
+      <c r="F294" s="5" t="s">
         <v>99</v>
       </c>
     </row>
@@ -8212,10 +8169,10 @@
         <v>71</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>222</v>
+        <v>927</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>223</v>
+        <v>928</v>
       </c>
       <c r="F295" s="5" t="s">
         <v>99</v>
@@ -8226,29 +8183,29 @@
         <v>71</v>
       </c>
       <c r="B296" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C296" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F296" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A297" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B297" s="2" t="s">
         <v>599</v>
       </c>
-      <c r="C296" s="2" t="s">
+      <c r="C297" s="2" t="s">
         <v>600</v>
       </c>
-      <c r="D296" s="2" t="s">
+      <c r="D297" s="2" t="s">
         <v>601</v>
       </c>
-      <c r="F296" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="297" spans="1:6" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A297" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="B297" s="31" t="s">
-        <v>929</v>
-      </c>
-      <c r="C297" s="31" t="s">
-        <v>930</v>
-      </c>
-      <c r="F297" s="34" t="s">
+      <c r="F297" s="5" t="s">
         <v>99</v>
       </c>
     </row>
@@ -8257,10 +8214,10 @@
         <v>71</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>587</v>
+        <v>929</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>588</v>
+        <v>930</v>
       </c>
       <c r="F298" s="5" t="s">
         <v>99</v>
@@ -8271,13 +8228,13 @@
         <v>71</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>816</v>
+        <v>587</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>817</v>
-      </c>
-      <c r="F299" s="3" t="s">
-        <v>97</v>
+        <v>588</v>
+      </c>
+      <c r="F299" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.25">
@@ -8285,10 +8242,10 @@
         <v>71</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>669</v>
+        <v>816</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>670</v>
+        <v>817</v>
       </c>
       <c r="F300" s="3" t="s">
         <v>97</v>
@@ -8299,10 +8256,10 @@
         <v>71</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>602</v>
+        <v>669</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>603</v>
+        <v>670</v>
       </c>
       <c r="F301" s="3" t="s">
         <v>97</v>
@@ -8313,10 +8270,10 @@
         <v>71</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>574</v>
+        <v>602</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>575</v>
+        <v>603</v>
       </c>
       <c r="F302" s="3" t="s">
         <v>97</v>
@@ -8327,13 +8284,13 @@
         <v>71</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>554</v>
+        <v>574</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>555</v>
-      </c>
-      <c r="F303" s="4" t="s">
-        <v>98</v>
+        <v>575</v>
+      </c>
+      <c r="F303" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="304" spans="1:6" x14ac:dyDescent="0.25">
@@ -8341,44 +8298,44 @@
         <v>71</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>235</v>
+        <v>554</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>236</v>
+        <v>555</v>
       </c>
       <c r="F304" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="305" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A305" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>273</v>
+        <v>235</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="F305" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="G305" s="2" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="F305" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="306" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A306" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>74</v>
+        <v>273</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F306" s="5" t="s">
-        <v>99</v>
+        <v>274</v>
+      </c>
+      <c r="F306" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G306" s="2" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="307" spans="1:7" x14ac:dyDescent="0.25">
@@ -8386,10 +8343,10 @@
         <v>71</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F307" s="5" t="s">
         <v>99</v>
@@ -8400,10 +8357,10 @@
         <v>71</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F308" s="5" t="s">
         <v>99</v>
@@ -8414,44 +8371,44 @@
         <v>71</v>
       </c>
       <c r="B309" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F309" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="310" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+      <c r="F309" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="310" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A310" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B310" s="2" t="s">
-        <v>589</v>
+        <v>77</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>590</v>
-      </c>
-      <c r="D310" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="F310" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="311" spans="1:7" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="F310" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="311" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A311" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B311" s="2" t="s">
-        <v>420</v>
+        <v>589</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="F311" s="4" t="s">
-        <v>98</v>
+        <v>590</v>
+      </c>
+      <c r="D311" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="F311" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="312" spans="1:7" x14ac:dyDescent="0.25">
@@ -8459,41 +8416,41 @@
         <v>71</v>
       </c>
       <c r="B312" s="2" t="s">
-        <v>449</v>
+        <v>420</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>450</v>
+        <v>421</v>
       </c>
       <c r="F312" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="313" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A313" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B313" s="2" t="s">
-        <v>604</v>
+        <v>449</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>605</v>
-      </c>
-      <c r="F313" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="314" spans="1:7" x14ac:dyDescent="0.25">
+        <v>450</v>
+      </c>
+      <c r="F313" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="314" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A314" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B314" s="2" t="s">
-        <v>699</v>
+        <v>604</v>
       </c>
       <c r="C314" s="2" t="s">
-        <v>700</v>
-      </c>
-      <c r="F314" s="3" t="s">
-        <v>97</v>
+        <v>605</v>
+      </c>
+      <c r="F314" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="315" spans="1:7" x14ac:dyDescent="0.25">
@@ -8501,10 +8458,10 @@
         <v>71</v>
       </c>
       <c r="B315" s="2" t="s">
-        <v>78</v>
+        <v>699</v>
       </c>
       <c r="C315" s="2" t="s">
-        <v>86</v>
+        <v>700</v>
       </c>
       <c r="F315" s="3" t="s">
         <v>97</v>
@@ -8515,30 +8472,27 @@
         <v>71</v>
       </c>
       <c r="B316" s="2" t="s">
-        <v>513</v>
+        <v>78</v>
       </c>
       <c r="C316" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="F316" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="317" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+      <c r="F316" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="317" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A317" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B317" s="2" t="s">
-        <v>281</v>
+        <v>513</v>
       </c>
       <c r="C317" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="F317" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G317" s="2" t="s">
-        <v>321</v>
+        <v>514</v>
+      </c>
+      <c r="F317" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="318" spans="1:7" ht="60" x14ac:dyDescent="0.25">
@@ -8546,10 +8500,10 @@
         <v>71</v>
       </c>
       <c r="B318" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C318" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="F318" s="16" t="s">
         <v>291</v>
@@ -8563,10 +8517,10 @@
         <v>71</v>
       </c>
       <c r="B319" s="2" t="s">
-        <v>233</v>
+        <v>283</v>
       </c>
       <c r="C319" s="2" t="s">
-        <v>234</v>
+        <v>284</v>
       </c>
       <c r="F319" s="16" t="s">
         <v>291</v>
@@ -8575,35 +8529,38 @@
         <v>321</v>
       </c>
     </row>
-    <row r="320" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A320" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C320" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E320" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="F320" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="321" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+      <c r="F320" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G320" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="321" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A321" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>653</v>
+        <v>224</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>654</v>
-      </c>
-      <c r="F321" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
+      </c>
+      <c r="E321" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F321" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="322" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -8611,58 +8568,58 @@
         <v>71</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>79</v>
+        <v>653</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F322" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="323" spans="1:7" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+      <c r="F322" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="323" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A323" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B323" s="2" t="s">
-        <v>703</v>
+        <v>79</v>
       </c>
       <c r="C323" s="2" t="s">
-        <v>704</v>
+        <v>87</v>
       </c>
       <c r="F323" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="324" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A324" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B324" s="2" t="s">
-        <v>415</v>
+        <v>703</v>
       </c>
       <c r="C324" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="F324" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G324" s="2" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="325" spans="1:7" x14ac:dyDescent="0.25">
+        <v>704</v>
+      </c>
+      <c r="F324" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="325" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A325" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B325" s="2" t="s">
-        <v>606</v>
+        <v>415</v>
       </c>
       <c r="C325" s="2" t="s">
-        <v>607</v>
-      </c>
-      <c r="F325" s="5" t="s">
-        <v>99</v>
+        <v>416</v>
+      </c>
+      <c r="F325" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G325" s="2" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="326" spans="1:7" x14ac:dyDescent="0.25">
@@ -8670,44 +8627,44 @@
         <v>71</v>
       </c>
       <c r="B326" s="2" t="s">
-        <v>476</v>
+        <v>606</v>
       </c>
       <c r="C326" s="2" t="s">
-        <v>477</v>
+        <v>607</v>
       </c>
       <c r="F326" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="327" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A327" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B327" s="2" t="s">
-        <v>736</v>
+        <v>476</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="F327" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="G327" s="2" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="328" spans="1:7" x14ac:dyDescent="0.25">
+        <v>477</v>
+      </c>
+      <c r="F327" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="328" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A328" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B328" s="2" t="s">
-        <v>239</v>
+        <v>736</v>
       </c>
       <c r="C328" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="F328" s="14" t="s">
-        <v>252</v>
+        <v>737</v>
+      </c>
+      <c r="F328" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="G328" s="2" t="s">
+        <v>738</v>
       </c>
     </row>
     <row r="329" spans="1:7" x14ac:dyDescent="0.25">
@@ -8715,13 +8672,13 @@
         <v>71</v>
       </c>
       <c r="B329" s="2" t="s">
-        <v>286</v>
+        <v>239</v>
       </c>
       <c r="C329" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="F329" s="5" t="s">
-        <v>99</v>
+        <v>240</v>
+      </c>
+      <c r="F329" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="330" spans="1:7" x14ac:dyDescent="0.25">
@@ -8729,13 +8686,13 @@
         <v>71</v>
       </c>
       <c r="B330" s="2" t="s">
-        <v>608</v>
+        <v>286</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>609</v>
-      </c>
-      <c r="F330" s="4" t="s">
-        <v>98</v>
+        <v>285</v>
+      </c>
+      <c r="F330" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="331" spans="1:7" x14ac:dyDescent="0.25">
@@ -8743,13 +8700,13 @@
         <v>71</v>
       </c>
       <c r="B331" s="2" t="s">
-        <v>228</v>
+        <v>608</v>
       </c>
       <c r="C331" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="F331" s="5" t="s">
-        <v>99</v>
+        <v>609</v>
+      </c>
+      <c r="F331" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="332" spans="1:7" x14ac:dyDescent="0.25">
@@ -8757,10 +8714,10 @@
         <v>71</v>
       </c>
       <c r="B332" s="2" t="s">
-        <v>592</v>
+        <v>228</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>593</v>
+        <v>229</v>
       </c>
       <c r="F332" s="5" t="s">
         <v>99</v>
@@ -8771,47 +8728,44 @@
         <v>71</v>
       </c>
       <c r="B333" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="C333" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="F333" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="334" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A334" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B334" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="C333" s="2" t="s">
+      <c r="C334" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="F333" s="12" t="s">
+      <c r="F334" s="12" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="334" spans="1:7" s="31" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="F334" s="35"/>
-    </row>
     <row r="335" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A335" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B335" s="2" t="s">
-        <v>491</v>
-      </c>
-      <c r="C335" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="F335" s="14" t="s">
-        <v>252</v>
-      </c>
+      <c r="F335" s="12"/>
     </row>
     <row r="336" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A336" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B336" s="2" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="E336" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="F336" s="5" t="s">
-        <v>99</v>
+        <v>492</v>
+      </c>
+      <c r="F336" s="14" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="337" spans="1:7" x14ac:dyDescent="0.25">
@@ -8819,10 +8773,13 @@
         <v>71</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>218</v>
+        <v>489</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>219</v>
+        <v>490</v>
+      </c>
+      <c r="E337" s="2" t="s">
+        <v>220</v>
       </c>
       <c r="F337" s="5" t="s">
         <v>99</v>
@@ -8833,30 +8790,27 @@
         <v>71</v>
       </c>
       <c r="B338" s="2" t="s">
-        <v>610</v>
+        <v>218</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>611</v>
-      </c>
-      <c r="F338" s="41" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="339" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+      <c r="F338" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="339" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A339" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B339" s="2" t="s">
-        <v>549</v>
+        <v>610</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>551</v>
-      </c>
-      <c r="F339" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="G339" s="2" t="s">
-        <v>552</v>
+        <v>611</v>
+      </c>
+      <c r="F339" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="340" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -8864,81 +8818,81 @@
         <v>71</v>
       </c>
       <c r="B340" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C340" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="F340" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G340" s="2" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="341" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A341" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B341" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="C340" s="2" t="s">
+      <c r="C341" s="2" t="s">
         <v>553</v>
       </c>
-      <c r="F340" s="16" t="s">
+      <c r="F341" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G340" s="2" t="s">
+      <c r="G341" s="2" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="341" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A341" s="17" t="s">
+    <row r="342" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A342" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B341" s="17" t="s">
+      <c r="B342" s="17" t="s">
         <v>294</v>
       </c>
-      <c r="C341" s="17" t="s">
+      <c r="C342" s="17" t="s">
         <v>295</v>
       </c>
-      <c r="D341" s="17"/>
-      <c r="E341" s="17"/>
-      <c r="F341" s="20" t="s">
+      <c r="D342" s="17"/>
+      <c r="E342" s="17"/>
+      <c r="F342" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="G341" s="17"/>
-    </row>
-    <row r="342" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A342" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B342" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C342" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D342" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="F342" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="343" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G342" s="17"/>
+    </row>
+    <row r="343" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A343" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B343" s="2" t="s">
-        <v>216</v>
+        <v>89</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>215</v>
+        <v>90</v>
       </c>
       <c r="D343" s="2" t="s">
-        <v>375</v>
+        <v>303</v>
       </c>
       <c r="F343" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="344" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B344" s="2" t="s">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>242</v>
+        <v>215</v>
       </c>
       <c r="D344" s="2" t="s">
-        <v>243</v>
+        <v>375</v>
       </c>
       <c r="F344" s="5" t="s">
         <v>99</v>
@@ -8949,27 +8903,30 @@
         <v>88</v>
       </c>
       <c r="B345" s="2" t="s">
-        <v>765</v>
+        <v>241</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>766</v>
-      </c>
-      <c r="F345" s="25" t="s">
-        <v>767</v>
-      </c>
-    </row>
-    <row r="346" spans="1:7" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+      <c r="D345" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F345" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="346" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B346" s="2" t="s">
-        <v>333</v>
+        <v>765</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="F346" s="4" t="s">
-        <v>98</v>
+        <v>766</v>
+      </c>
+      <c r="F346" s="25" t="s">
+        <v>767</v>
       </c>
     </row>
     <row r="347" spans="1:7" x14ac:dyDescent="0.25">
@@ -8977,36 +8934,50 @@
         <v>88</v>
       </c>
       <c r="B347" s="2" t="s">
-        <v>529</v>
+        <v>333</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>530</v>
-      </c>
-      <c r="D347" s="2" t="s">
-        <v>531</v>
+        <v>334</v>
       </c>
       <c r="F347" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="348" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A348" s="17" t="s">
+    <row r="348" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A348" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B348" s="17" t="s">
+      <c r="B348" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="C348" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="D348" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="F348" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="349" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A349" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B349" s="17" t="s">
         <v>279</v>
       </c>
-      <c r="C348" s="17" t="s">
+      <c r="C349" s="17" t="s">
         <v>280</v>
       </c>
-      <c r="D348" s="17" t="s">
+      <c r="D349" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="E348" s="17"/>
-      <c r="F348" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="G348" s="17"/>
+      <c r="E349" s="17"/>
+      <c r="F349" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="G349" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
correct "goeeng" typo in acronym key
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MinshuDeng\Desktop\SyncFreeZone\EPS\GitHubRepos\US\eps-us\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05E678C4-344F-464B-B0C7-135154764FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690A2C50-7980-4403-B9BF-C7CF5998A0B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1452" uniqueCount="841">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1452" uniqueCount="840">
   <si>
     <t>Top Level Folder</t>
   </si>
@@ -2294,9 +2294,6 @@
   </si>
   <si>
     <t>You are modeling a region where power plant CCUS retrofit decisions are based on government mandates rather than being market-driven, and you are setting this policy lever to alter the BAU mandates</t>
-  </si>
-  <si>
-    <t>goeeng</t>
   </si>
   <si>
     <t>ERWD</t>
@@ -3036,82 +3033,82 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C70"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.81640625" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>99</v>
       </c>
@@ -3119,32 +3116,32 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26" s="13" t="s">
         <v>250</v>
       </c>
@@ -3152,17 +3149,17 @@
         <v>253</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>101</v>
       </c>
@@ -3170,42 +3167,42 @@
         <v>126</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
         <v>100</v>
       </c>
@@ -3213,84 +3210,84 @@
         <v>134</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
         <v>258</v>
       </c>
       <c r="B48" s="15"/>
       <c r="C48" s="15"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>142</v>
       </c>
@@ -3298,62 +3295,62 @@
         <v>143</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>152</v>
       </c>
@@ -3367,19 +3364,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G306"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="49.1796875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="49.140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="67" style="2" customWidth="1"/>
-    <col min="5" max="5" width="18.81640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="37.54296875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="37.5703125" style="2" customWidth="1"/>
     <col min="7" max="7" width="54" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.81640625" style="2"/>
+    <col min="8" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -3402,7 +3399,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -3421,7 +3418,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -3438,7 +3435,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -3452,7 +3449,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -3469,7 +3466,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -3483,7 +3480,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
         <v>4</v>
       </c>
@@ -3500,7 +3497,7 @@
       </c>
       <c r="G7" s="17"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
@@ -3514,7 +3511,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -3528,7 +3525,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -3542,7 +3539,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -3559,7 +3556,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
@@ -3573,7 +3570,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -3590,7 +3587,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
@@ -3604,24 +3601,24 @@
         <v>101</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>800</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>801</v>
       </c>
       <c r="F15" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -3638,7 +3635,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>9</v>
       </c>
@@ -3652,7 +3649,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>9</v>
       </c>
@@ -3666,7 +3663,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
@@ -3680,7 +3677,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
@@ -3694,7 +3691,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>9</v>
       </c>
@@ -3708,7 +3705,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>9</v>
       </c>
@@ -3722,21 +3719,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>768</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>769</v>
-      </c>
       <c r="F23" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>9</v>
       </c>
@@ -3753,7 +3750,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>9</v>
       </c>
@@ -3767,7 +3764,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>9</v>
       </c>
@@ -3784,7 +3781,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>9</v>
       </c>
@@ -3798,7 +3795,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
@@ -3812,7 +3809,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>9</v>
       </c>
@@ -3829,7 +3826,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>9</v>
       </c>
@@ -3846,7 +3843,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>9</v>
       </c>
@@ -3860,7 +3857,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>9</v>
       </c>
@@ -3874,7 +3871,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>9</v>
       </c>
@@ -3888,7 +3885,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>9</v>
       </c>
@@ -3902,7 +3899,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>9</v>
       </c>
@@ -3919,7 +3916,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="17" t="s">
         <v>9</v>
       </c>
@@ -3938,7 +3935,7 @@
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
@@ -3952,7 +3949,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -3969,7 +3966,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>36</v>
       </c>
@@ -3983,7 +3980,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>36</v>
       </c>
@@ -4000,7 +3997,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>36</v>
       </c>
@@ -4017,7 +4014,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>36</v>
       </c>
@@ -4031,27 +4028,27 @@
         <v>101</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>802</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>803</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="D43" s="2" t="s">
         <v>804</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>805</v>
       </c>
       <c r="F43" s="21" t="s">
         <v>303</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>806</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>36</v>
       </c>
@@ -4065,12 +4062,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="17" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7" s="17" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="17" t="s">
         <v>36</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="C45" s="17" t="s">
         <v>697</v>
@@ -4079,7 +4076,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>172</v>
       </c>
@@ -4093,7 +4090,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="17" t="s">
         <v>172</v>
       </c>
@@ -4112,7 +4109,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="17" t="s">
         <v>484</v>
       </c>
@@ -4131,7 +4128,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>413</v>
       </c>
@@ -4148,7 +4145,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>413</v>
       </c>
@@ -4165,7 +4162,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>413</v>
       </c>
@@ -4182,24 +4179,24 @@
         <v>438</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>413</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>822</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>823</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>180</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>413</v>
       </c>
@@ -4216,7 +4213,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>413</v>
       </c>
@@ -4233,7 +4230,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>413</v>
       </c>
@@ -4250,7 +4247,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>413</v>
       </c>
@@ -4267,7 +4264,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>413</v>
       </c>
@@ -4284,7 +4281,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>413</v>
       </c>
@@ -4301,21 +4298,21 @@
         <v>572</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>413</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>836</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>837</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>838</v>
       </c>
       <c r="F59" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>413</v>
       </c>
@@ -4332,7 +4329,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>413</v>
       </c>
@@ -4349,7 +4346,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>413</v>
       </c>
@@ -4363,7 +4360,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>413</v>
       </c>
@@ -4383,15 +4380,15 @@
         <v>465</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="17" t="s">
         <v>413</v>
       </c>
       <c r="B64" s="17" t="s">
+        <v>824</v>
+      </c>
+      <c r="C64" s="17" t="s">
         <v>825</v>
-      </c>
-      <c r="C64" s="17" t="s">
-        <v>826</v>
       </c>
       <c r="D64" s="17"/>
       <c r="E64" s="17"/>
@@ -4399,10 +4396,10 @@
         <v>303</v>
       </c>
       <c r="G64" s="17" t="s">
-        <v>827</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>38</v>
       </c>
@@ -4416,7 +4413,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>38</v>
       </c>
@@ -4430,7 +4427,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>38</v>
       </c>
@@ -4444,7 +4441,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>38</v>
       </c>
@@ -4458,7 +4455,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="17" t="s">
         <v>38</v>
       </c>
@@ -4477,35 +4474,35 @@
         <v>387</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>43</v>
       </c>
@@ -4522,7 +4519,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="73" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>43</v>
       </c>
@@ -4539,7 +4536,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>43</v>
       </c>
@@ -4553,7 +4550,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>43</v>
       </c>
@@ -4567,7 +4564,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>43</v>
       </c>
@@ -4584,21 +4581,21 @@
         <v>100</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B77" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="C77" s="2" t="s">
         <v>835</v>
       </c>
-      <c r="C77" s="2" t="s">
-        <v>836</v>
-      </c>
       <c r="F77" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="78" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>43</v>
       </c>
@@ -4615,7 +4612,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>43</v>
       </c>
@@ -4632,7 +4629,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>43</v>
       </c>
@@ -4646,7 +4643,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>43</v>
       </c>
@@ -4663,7 +4660,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="82" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>43</v>
       </c>
@@ -4680,21 +4677,21 @@
         <v>750</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>770</v>
       </c>
-      <c r="C83" s="2" t="s">
-        <v>771</v>
-      </c>
       <c r="F83" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="84" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>43</v>
       </c>
@@ -4708,7 +4705,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>43</v>
       </c>
@@ -4728,21 +4725,21 @@
         <v>99</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B86" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>820</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>821</v>
       </c>
       <c r="F86" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>43</v>
       </c>
@@ -4756,7 +4753,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>43</v>
       </c>
@@ -4770,7 +4767,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="89" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>43</v>
       </c>
@@ -4787,7 +4784,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="90" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>43</v>
       </c>
@@ -4801,7 +4798,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="91" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>43</v>
       </c>
@@ -4818,21 +4815,21 @@
         <v>514</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B92" s="2" t="s">
+        <v>782</v>
+      </c>
+      <c r="C92" s="2" t="s">
         <v>783</v>
       </c>
-      <c r="C92" s="2" t="s">
-        <v>784</v>
-      </c>
       <c r="F92" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>43</v>
       </c>
@@ -4843,13 +4840,13 @@
         <v>726</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="F93" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>43</v>
       </c>
@@ -4863,7 +4860,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>43</v>
       </c>
@@ -4877,7 +4874,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>43</v>
       </c>
@@ -4891,7 +4888,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>43</v>
       </c>
@@ -4908,7 +4905,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>43</v>
       </c>
@@ -4925,7 +4922,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>43</v>
       </c>
@@ -4936,13 +4933,13 @@
         <v>170</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="F99" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>43</v>
       </c>
@@ -4959,21 +4956,21 @@
         <v>100</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B101" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="C101" s="2" t="s">
         <v>818</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>819</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>43</v>
       </c>
@@ -4987,7 +4984,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>43</v>
       </c>
@@ -5004,7 +5001,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>43</v>
       </c>
@@ -5021,32 +5018,32 @@
         <v>321</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B105" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="F105" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B106" s="2" t="s">
         <v>762</v>
       </c>
-      <c r="C105" s="2" t="s">
+      <c r="C106" s="2" t="s">
         <v>764</v>
       </c>
-      <c r="F105" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B106" s="2" t="s">
-        <v>763</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>765</v>
-      </c>
       <c r="F106" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>43</v>
       </c>
@@ -5060,7 +5057,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>43</v>
       </c>
@@ -5074,7 +5071,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>43</v>
       </c>
@@ -5088,7 +5085,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>43</v>
       </c>
@@ -5102,7 +5099,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>43</v>
       </c>
@@ -5116,7 +5113,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>43</v>
       </c>
@@ -5130,7 +5127,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>43</v>
       </c>
@@ -5144,7 +5141,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>43</v>
       </c>
@@ -5158,7 +5155,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>43</v>
       </c>
@@ -5172,7 +5169,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>43</v>
       </c>
@@ -5189,7 +5186,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>43</v>
       </c>
@@ -5206,7 +5203,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>43</v>
       </c>
@@ -5217,13 +5214,13 @@
         <v>745</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="F118" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>43</v>
       </c>
@@ -5240,7 +5237,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>43</v>
       </c>
@@ -5254,7 +5251,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>43</v>
       </c>
@@ -5268,7 +5265,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>43</v>
       </c>
@@ -5285,7 +5282,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="123" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>43</v>
       </c>
@@ -5302,7 +5299,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>43</v>
       </c>
@@ -5319,7 +5316,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="125" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
         <v>664</v>
       </c>
@@ -5330,7 +5327,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="126" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>43</v>
       </c>
@@ -5347,7 +5344,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>43</v>
       </c>
@@ -5361,7 +5358,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>43</v>
       </c>
@@ -5375,7 +5372,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>43</v>
       </c>
@@ -5389,7 +5386,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>43</v>
       </c>
@@ -5403,7 +5400,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>43</v>
       </c>
@@ -5417,7 +5414,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>43</v>
       </c>
@@ -5434,7 +5431,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>43</v>
       </c>
@@ -5451,21 +5448,21 @@
         <v>99</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B134" s="2" t="s">
+        <v>815</v>
+      </c>
+      <c r="C134" s="2" t="s">
         <v>816</v>
-      </c>
-      <c r="C134" s="2" t="s">
-        <v>817</v>
       </c>
       <c r="F134" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>43</v>
       </c>
@@ -5479,21 +5476,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B136" s="2" t="s">
+        <v>832</v>
+      </c>
+      <c r="C136" s="2" t="s">
         <v>833</v>
       </c>
-      <c r="C136" s="2" t="s">
-        <v>834</v>
-      </c>
       <c r="F136" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="17" t="s">
         <v>43</v>
       </c>
@@ -5514,7 +5511,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>275</v>
       </c>
@@ -5531,7 +5528,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>275</v>
       </c>
@@ -5548,7 +5545,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>275</v>
       </c>
@@ -5562,7 +5559,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>275</v>
       </c>
@@ -5576,7 +5573,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>275</v>
       </c>
@@ -5590,7 +5587,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>275</v>
       </c>
@@ -5604,7 +5601,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="17" t="s">
         <v>275</v>
       </c>
@@ -5621,7 +5618,7 @@
       </c>
       <c r="G144" s="17"/>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>55</v>
       </c>
@@ -5635,49 +5632,49 @@
         <v>99</v>
       </c>
     </row>
-    <row r="146" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="F146" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="F147" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="F148" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>55</v>
       </c>
@@ -5694,7 +5691,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>55</v>
       </c>
@@ -5708,7 +5705,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="151" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>55</v>
       </c>
@@ -5725,7 +5722,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>55</v>
       </c>
@@ -5739,21 +5736,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B153" s="2" t="s">
+        <v>775</v>
+      </c>
+      <c r="C153" s="2" t="s">
         <v>776</v>
       </c>
-      <c r="C153" s="2" t="s">
-        <v>777</v>
-      </c>
       <c r="F153" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>55</v>
       </c>
@@ -5767,7 +5764,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>55</v>
       </c>
@@ -5775,7 +5772,7 @@
         <v>525</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="E155" s="2" t="s">
         <v>526</v>
@@ -5784,21 +5781,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="F156" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>55</v>
       </c>
@@ -5812,7 +5809,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>55</v>
       </c>
@@ -5826,7 +5823,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>55</v>
       </c>
@@ -5843,7 +5840,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>55</v>
       </c>
@@ -5857,7 +5854,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>55</v>
       </c>
@@ -5874,7 +5871,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="162" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>55</v>
       </c>
@@ -5891,7 +5888,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>55</v>
       </c>
@@ -5908,7 +5905,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>55</v>
       </c>
@@ -5925,7 +5922,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>55</v>
       </c>
@@ -5942,7 +5939,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>55</v>
       </c>
@@ -5956,7 +5953,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="167" spans="1:7" s="17" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:7" s="17" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A167" s="17" t="s">
         <v>55</v>
       </c>
@@ -5973,7 +5970,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="168" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>404</v>
       </c>
@@ -5990,24 +5987,24 @@
         <v>99</v>
       </c>
     </row>
-    <row r="169" spans="1:7" s="17" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="169" spans="1:7" s="17" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A169" s="17" t="s">
+        <v>404</v>
+      </c>
+      <c r="B169" s="17" t="s">
         <v>754</v>
       </c>
-      <c r="B169" s="17" t="s">
+      <c r="C169" s="17" t="s">
         <v>755</v>
       </c>
-      <c r="C169" s="17" t="s">
+      <c r="D169" s="17" t="s">
         <v>756</v>
-      </c>
-      <c r="D169" s="17" t="s">
-        <v>757</v>
       </c>
       <c r="F169" s="19" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>357</v>
       </c>
@@ -6021,7 +6018,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>357</v>
       </c>
@@ -6035,7 +6032,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>357</v>
       </c>
@@ -6049,7 +6046,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>357</v>
       </c>
@@ -6066,7 +6063,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="174" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>357</v>
       </c>
@@ -6080,7 +6077,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>357</v>
       </c>
@@ -6097,22 +6094,22 @@
         <v>374</v>
       </c>
     </row>
-    <row r="176" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>357</v>
       </c>
       <c r="B176" s="2" t="s">
+        <v>806</v>
+      </c>
+      <c r="C176" s="2" t="s">
         <v>807</v>
-      </c>
-      <c r="C176" s="2" t="s">
-        <v>808</v>
       </c>
       <c r="F176" s="6"/>
       <c r="G176" s="2" t="s">
-        <v>809</v>
-      </c>
-    </row>
-    <row r="177" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>357</v>
       </c>
@@ -6129,7 +6126,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="178" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="178" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A178" s="17" t="s">
         <v>357</v>
       </c>
@@ -6146,7 +6143,7 @@
       </c>
       <c r="G178" s="17"/>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>63</v>
       </c>
@@ -6160,7 +6157,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>63</v>
       </c>
@@ -6177,7 +6174,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="181" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>63</v>
       </c>
@@ -6194,7 +6191,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="182" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>63</v>
       </c>
@@ -6214,7 +6211,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="183" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>63</v>
       </c>
@@ -6228,7 +6225,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="184" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>63</v>
       </c>
@@ -6242,7 +6239,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>63</v>
       </c>
@@ -6256,7 +6253,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>63</v>
       </c>
@@ -6273,7 +6270,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>63</v>
       </c>
@@ -6287,35 +6284,35 @@
         <v>101</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B188" s="2" t="s">
+        <v>759</v>
+      </c>
+      <c r="C188" s="2" t="s">
         <v>760</v>
-      </c>
-      <c r="C188" s="2" t="s">
-        <v>761</v>
       </c>
       <c r="F188" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B189" s="2" t="s">
+        <v>765</v>
+      </c>
+      <c r="C189" s="2" t="s">
         <v>766</v>
-      </c>
-      <c r="C189" s="2" t="s">
-        <v>767</v>
       </c>
       <c r="F189" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="190" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>63</v>
       </c>
@@ -6332,7 +6329,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>63</v>
       </c>
@@ -6346,27 +6343,27 @@
         <v>100</v>
       </c>
     </row>
-    <row r="192" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B192" s="2" t="s">
+        <v>809</v>
+      </c>
+      <c r="C192" s="2" t="s">
         <v>810</v>
       </c>
-      <c r="C192" s="2" t="s">
+      <c r="D192" s="2" t="s">
         <v>811</v>
-      </c>
-      <c r="D192" s="2" t="s">
-        <v>812</v>
       </c>
       <c r="F192" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G192" s="2" t="s">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="193" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
         <v>63</v>
       </c>
@@ -6383,7 +6380,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
         <v>63</v>
       </c>
@@ -6397,7 +6394,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="195" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
         <v>63</v>
       </c>
@@ -6411,7 +6408,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="196" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
         <v>63</v>
       </c>
@@ -6425,7 +6422,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="197" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
         <v>63</v>
       </c>
@@ -6439,7 +6436,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="198" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>63</v>
       </c>
@@ -6453,7 +6450,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>63</v>
       </c>
@@ -6467,7 +6464,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="200" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>63</v>
       </c>
@@ -6481,7 +6478,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="201" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="201" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A201" s="17" t="s">
         <v>63</v>
       </c>
@@ -6498,21 +6495,21 @@
       </c>
       <c r="G201" s="17"/>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B202" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="C202" s="2" t="s">
         <v>793</v>
-      </c>
-      <c r="C202" s="2" t="s">
-        <v>794</v>
       </c>
       <c r="F202" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="203" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
         <v>420</v>
       </c>
@@ -6529,7 +6526,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>420</v>
       </c>
@@ -6546,7 +6543,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>420</v>
       </c>
@@ -6560,7 +6557,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>420</v>
       </c>
@@ -6574,7 +6571,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>420</v>
       </c>
@@ -6588,7 +6585,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>420</v>
       </c>
@@ -6602,7 +6599,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="209" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>420</v>
       </c>
@@ -6622,7 +6619,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>420</v>
       </c>
@@ -6636,7 +6633,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>420</v>
       </c>
@@ -6650,7 +6647,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="212" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>420</v>
       </c>
@@ -6667,7 +6664,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="213" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>420</v>
       </c>
@@ -6682,7 +6679,7 @@
       </c>
       <c r="F213" s="3"/>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>420</v>
       </c>
@@ -6699,7 +6696,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>420</v>
       </c>
@@ -6716,7 +6713,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
         <v>420</v>
       </c>
@@ -6730,7 +6727,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
         <v>420</v>
       </c>
@@ -6744,7 +6741,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
         <v>420</v>
       </c>
@@ -6758,7 +6755,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>420</v>
       </c>
@@ -6772,7 +6769,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
         <v>420</v>
       </c>
@@ -6786,7 +6783,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="221" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
         <v>420</v>
       </c>
@@ -6803,7 +6800,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="222" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="222" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A222" s="2" t="s">
         <v>420</v>
       </c>
@@ -6817,7 +6814,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="223" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="223" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A223" s="17" t="s">
         <v>420</v>
       </c>
@@ -6834,7 +6831,7 @@
       </c>
       <c r="G223" s="17"/>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
         <v>93</v>
       </c>
@@ -6848,7 +6845,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
         <v>93</v>
       </c>
@@ -6865,7 +6862,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="226" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
         <v>93</v>
       </c>
@@ -6879,7 +6876,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="227" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
         <v>93</v>
       </c>
@@ -6896,7 +6893,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
         <v>93</v>
       </c>
@@ -6910,7 +6907,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
         <v>93</v>
       </c>
@@ -6924,7 +6921,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
         <v>93</v>
       </c>
@@ -6938,7 +6935,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="231" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
         <v>93</v>
       </c>
@@ -6952,7 +6949,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="232" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="232" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A232" s="17" t="s">
         <v>93</v>
       </c>
@@ -6969,7 +6966,7 @@
       </c>
       <c r="G232" s="17"/>
     </row>
-    <row r="233" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
         <v>70</v>
       </c>
@@ -6986,7 +6983,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="234" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
         <v>70</v>
       </c>
@@ -7003,7 +7000,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
         <v>70</v>
       </c>
@@ -7020,7 +7017,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="236" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="236" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A236" s="17" t="s">
         <v>70</v>
       </c>
@@ -7039,7 +7036,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
         <v>73</v>
       </c>
@@ -7053,21 +7050,21 @@
         <v>100</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B238" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="C238" s="2" t="s">
         <v>839</v>
-      </c>
-      <c r="C238" s="2" t="s">
-        <v>840</v>
       </c>
       <c r="F238" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
         <v>73</v>
       </c>
@@ -7081,7 +7078,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240" s="2" t="s">
         <v>73</v>
       </c>
@@ -7095,7 +7092,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A241" s="2" t="s">
         <v>73</v>
       </c>
@@ -7109,7 +7106,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="242" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A242" s="2" t="s">
         <v>73</v>
       </c>
@@ -7123,7 +7120,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A243" s="2" t="s">
         <v>73</v>
       </c>
@@ -7137,7 +7134,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244" s="2" t="s">
         <v>73</v>
       </c>
@@ -7151,7 +7148,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" s="2" t="s">
         <v>73</v>
       </c>
@@ -7165,7 +7162,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A246" s="2" t="s">
         <v>73</v>
       </c>
@@ -7179,7 +7176,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A247" s="2" t="s">
         <v>73</v>
       </c>
@@ -7193,7 +7190,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="248" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A248" s="2" t="s">
         <v>73</v>
       </c>
@@ -7210,21 +7207,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A249" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B249" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="C249" s="2" t="s">
         <v>795</v>
-      </c>
-      <c r="C249" s="2" t="s">
-        <v>796</v>
       </c>
       <c r="F249" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250" s="2" t="s">
         <v>73</v>
       </c>
@@ -7238,7 +7235,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" s="2" t="s">
         <v>73</v>
       </c>
@@ -7252,7 +7249,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A252" s="2" t="s">
         <v>73</v>
       </c>
@@ -7266,7 +7263,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A253" s="2" t="s">
         <v>73</v>
       </c>
@@ -7280,21 +7277,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B254" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="C254" s="2" t="s">
         <v>829</v>
-      </c>
-      <c r="C254" s="2" t="s">
-        <v>830</v>
       </c>
       <c r="F254" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255" s="2" t="s">
         <v>73</v>
       </c>
@@ -7311,21 +7308,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B256" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="C256" s="2" t="s">
         <v>831</v>
-      </c>
-      <c r="C256" s="2" t="s">
-        <v>832</v>
       </c>
       <c r="F256" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A257" s="2" t="s">
         <v>73</v>
       </c>
@@ -7339,21 +7336,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A258" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B258" s="2" t="s">
+        <v>813</v>
+      </c>
+      <c r="C258" s="2" t="s">
         <v>814</v>
-      </c>
-      <c r="C258" s="2" t="s">
-        <v>815</v>
       </c>
       <c r="F258" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A259" s="2" t="s">
         <v>73</v>
       </c>
@@ -7367,7 +7364,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A260" s="2" t="s">
         <v>73</v>
       </c>
@@ -7381,7 +7378,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A261" s="2" t="s">
         <v>73</v>
       </c>
@@ -7395,7 +7392,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A262" s="2" t="s">
         <v>73</v>
       </c>
@@ -7409,7 +7406,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A263" s="2" t="s">
         <v>73</v>
       </c>
@@ -7423,7 +7420,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="264" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A264" s="2" t="s">
         <v>73</v>
       </c>
@@ -7440,7 +7437,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A265" s="2" t="s">
         <v>73</v>
       </c>
@@ -7454,7 +7451,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A266" s="2" t="s">
         <v>73</v>
       </c>
@@ -7468,7 +7465,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
         <v>73</v>
       </c>
@@ -7482,7 +7479,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A268" s="2" t="s">
         <v>73</v>
       </c>
@@ -7496,7 +7493,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
         <v>73</v>
       </c>
@@ -7513,7 +7510,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A270" s="2" t="s">
         <v>73</v>
       </c>
@@ -7527,7 +7524,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A271" s="2" t="s">
         <v>73</v>
       </c>
@@ -7541,7 +7538,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="272" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
         <v>73</v>
       </c>
@@ -7555,7 +7552,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A273" s="2" t="s">
         <v>73</v>
       </c>
@@ -7569,7 +7566,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A274" s="2" t="s">
         <v>73</v>
       </c>
@@ -7583,7 +7580,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A275" s="2" t="s">
         <v>73</v>
       </c>
@@ -7597,7 +7594,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="276" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A276" s="2" t="s">
         <v>73</v>
       </c>
@@ -7614,7 +7611,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="277" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A277" s="2" t="s">
         <v>73</v>
       </c>
@@ -7631,7 +7628,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="278" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A278" s="2" t="s">
         <v>73</v>
       </c>
@@ -7648,7 +7645,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
         <v>73</v>
       </c>
@@ -7665,7 +7662,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="280" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
         <v>73</v>
       </c>
@@ -7679,7 +7676,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="281" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A281" s="2" t="s">
         <v>73</v>
       </c>
@@ -7693,7 +7690,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A282" s="2" t="s">
         <v>73</v>
       </c>
@@ -7707,7 +7704,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="283" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A283" s="2" t="s">
         <v>73</v>
       </c>
@@ -7724,7 +7721,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A284" s="2" t="s">
         <v>73</v>
       </c>
@@ -7738,7 +7735,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A285" s="2" t="s">
         <v>73</v>
       </c>
@@ -7752,24 +7749,24 @@
         <v>101</v>
       </c>
     </row>
-    <row r="286" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A286" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B286" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="C286" s="2" t="s">
         <v>772</v>
-      </c>
-      <c r="C286" s="2" t="s">
-        <v>773</v>
       </c>
       <c r="F286" s="16" t="s">
         <v>303</v>
       </c>
       <c r="G286" s="2" t="s">
-        <v>774</v>
-      </c>
-    </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.35">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A287" s="2" t="s">
         <v>73</v>
       </c>
@@ -7783,7 +7780,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A288" s="2" t="s">
         <v>73</v>
       </c>
@@ -7797,7 +7794,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A289" s="2" t="s">
         <v>73</v>
       </c>
@@ -7811,7 +7808,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
         <v>73</v>
       </c>
@@ -7825,7 +7822,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A291" s="2" t="s">
         <v>73</v>
       </c>
@@ -7839,7 +7836,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A292" s="2" t="s">
         <v>73</v>
       </c>
@@ -7853,7 +7850,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A293" s="2" t="s">
         <v>73</v>
       </c>
@@ -7867,7 +7864,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A294" s="2" t="s">
         <v>73</v>
       </c>
@@ -7884,7 +7881,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A295" s="2" t="s">
         <v>73</v>
       </c>
@@ -7898,7 +7895,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="296" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="296" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A296" s="2" t="s">
         <v>73</v>
       </c>
@@ -7912,7 +7909,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="297" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A297" s="2" t="s">
         <v>73</v>
       </c>
@@ -7929,7 +7926,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="298" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A298" s="2" t="s">
         <v>73</v>
       </c>
@@ -7946,7 +7943,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="299" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="299" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A299" s="17" t="s">
         <v>73</v>
       </c>
@@ -7963,7 +7960,7 @@
       </c>
       <c r="G299" s="17"/>
     </row>
-    <row r="300" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A300" s="2" t="s">
         <v>90</v>
       </c>
@@ -7980,7 +7977,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A301" s="2" t="s">
         <v>90</v>
       </c>
@@ -7997,7 +7994,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="302" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A302" s="2" t="s">
         <v>90</v>
       </c>
@@ -8014,21 +8011,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="303" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B303" s="2" t="s">
+        <v>796</v>
+      </c>
+      <c r="C303" s="2" t="s">
         <v>797</v>
       </c>
-      <c r="C303" s="2" t="s">
+      <c r="F303" s="25" t="s">
         <v>798</v>
       </c>
-      <c r="F303" s="25" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A304" s="2" t="s">
         <v>90</v>
       </c>
@@ -8042,7 +8039,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A305" s="2" t="s">
         <v>90</v>
       </c>
@@ -8059,7 +8056,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="306" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="306" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A306" s="17" t="s">
         <v>90</v>
       </c>
@@ -8087,13 +8084,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.54296875" customWidth="1"/>
-    <col min="2" max="2" width="52.26953125" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="52.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8101,7 +8098,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -8109,7 +8106,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -8117,7 +8114,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -8125,7 +8122,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>172</v>
       </c>
@@ -8133,7 +8130,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>413</v>
       </c>
@@ -8141,7 +8138,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>484</v>
       </c>
@@ -8149,7 +8146,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -8157,7 +8154,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -8165,7 +8162,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>275</v>
       </c>
@@ -8173,7 +8170,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -8181,7 +8178,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>404</v>
       </c>
@@ -8189,7 +8186,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>357</v>
       </c>
@@ -8197,7 +8194,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>63</v>
       </c>
@@ -8205,7 +8202,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>420</v>
       </c>
@@ -8213,7 +8210,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>93</v>
       </c>
@@ -8221,7 +8218,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>70</v>
       </c>
@@ -8229,7 +8226,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>73</v>
       </c>
@@ -8237,7 +8234,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>90</v>
       </c>

</xml_diff>

<commit_message>
In-progress file management and clean up
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -43,7 +43,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -98,6 +98,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -120,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -190,6 +196,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2919,9 +2926,9 @@
           <t>elec</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>ACXAGE</t>
+      <c r="B76" s="29" t="inlineStr">
+        <is>
+          <t>ASCAPEX</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2929,12 +2936,12 @@
           <t>Annual Sustaining CAPEX by Generator Age</t>
         </is>
       </c>
-      <c r="D76" s="26" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>Annual Sustaining CAPEX Base per Unit Capacity, Annual Sustaining CAPEX Age Slope, Annual Sustaining CAPEX Adder Over 30 Years, Annual Sustaining CAPEX Incremental Adder Over 40 Years</t>
         </is>
       </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>low</t>
         </is>
@@ -2963,19 +2970,19 @@
       </c>
     </row>
     <row r="78" ht="45" customHeight="1" s="27">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>ATfUF</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Retirement Schedule Length for Unviable Fleets</t>
+      <c r="B78" s="26" t="inlineStr">
+        <is>
+          <t>BBNPPTY</t>
+        </is>
+      </c>
+      <c r="C78" s="26" t="inlineStr">
+        <is>
+          <t>BAU Ban New Power Plants This Year</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
@@ -2992,12 +2999,12 @@
       </c>
       <c r="B79" s="26" t="inlineStr">
         <is>
-          <t>BBNPPTY</t>
+          <t>BBPPRTY</t>
         </is>
       </c>
       <c r="C79" s="26" t="inlineStr">
         <is>
-          <t>BAU Ban New Power Plants This Year</t>
+          <t>BAU Ban Power Plant Retrofits This Year</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
@@ -3014,17 +3021,22 @@
       </c>
       <c r="B80" s="26" t="inlineStr">
         <is>
-          <t>BBPPRTY</t>
+          <t>BCoESC</t>
         </is>
       </c>
       <c r="C80" s="26" t="inlineStr">
         <is>
-          <t>BAU Ban Power Plant Retrofits This Year</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>BAU Cost of Electricity Sector Capital</t>
+        </is>
+      </c>
+      <c r="D80" s="26" t="inlineStr">
+        <is>
+          <t>BAU Cost of Electricity Sector Capital for Power Plants, BAU Cost of Electricity Sector Capital for Other Investments</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3036,22 +3048,22 @@
       </c>
       <c r="B81" s="26" t="inlineStr">
         <is>
-          <t>BCoESC</t>
+          <t>BCpUC</t>
         </is>
       </c>
       <c r="C81" s="26" t="inlineStr">
         <is>
-          <t>BAU Cost of Electricity Sector Capital</t>
+          <t>Battery Cost per Unit Capacity</t>
         </is>
       </c>
       <c r="D81" s="26" t="inlineStr">
         <is>
-          <t>BAU Cost of Electricity Sector Capital for Power Plants, BAU Cost of Electricity Sector Capital for Other Investments</t>
-        </is>
-      </c>
-      <c r="F81" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>Battery Power Cost per Unit Capacity, Battery Energy Cost per Unit Capacity, Battery Balance of System Cost as Share of First Year Cost</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -3063,22 +3075,17 @@
       </c>
       <c r="B82" s="26" t="inlineStr">
         <is>
-          <t>BCpUC</t>
+          <t>BCRbQ</t>
         </is>
       </c>
       <c r="C82" s="26" t="inlineStr">
         <is>
-          <t>Battery Cost per Unit Capacity</t>
-        </is>
-      </c>
-      <c r="D82" s="26" t="inlineStr">
-        <is>
-          <t>Battery Power Cost per Unit Capacity, Battery Energy Cost per Unit Capacity, Battery Balance of System Cost as Share of First Year Cost</t>
-        </is>
-      </c>
-      <c r="F82" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>BAU Capacity Retirements before Quantization</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -3090,34 +3097,39 @@
       </c>
       <c r="B83" s="26" t="inlineStr">
         <is>
-          <t>BCRbQ</t>
+          <t>BDTPTUMCF</t>
         </is>
       </c>
       <c r="C83" s="26" t="inlineStr">
         <is>
-          <t>BAU Capacity Retirements before Quantization</t>
-        </is>
-      </c>
-      <c r="F83" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>Boolean Does This Plant Type Use Maximum Capacity Factor</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
     <row r="84" ht="30" customHeight="1" s="27">
-      <c r="A84" s="26" t="inlineStr">
+      <c r="A84" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B84" s="26" t="inlineStr">
-        <is>
-          <t>BDTPTUMCF</t>
-        </is>
-      </c>
-      <c r="C84" s="26" t="inlineStr">
-        <is>
-          <t>Boolean Does This Plant Type Use Maximum Capacity Factor</t>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>BEPQSD</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>BAU Elec Portfolio Qualifying Source Definitions</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>BAU RPS Qualifying Source Definitions, BAU CES Qualifying Source Definitions</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
@@ -3127,29 +3139,30 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>BEPQSD</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>BAU Elec Portfolio Qualifying Source Definitions</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>BAU RPS Qualifying Source Definitions, BAU CES Qualifying Source Definitions</t>
-        </is>
-      </c>
-      <c r="F85" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="B85" s="26" t="inlineStr">
+        <is>
+          <t>BEVGB</t>
+        </is>
+      </c>
+      <c r="C85" s="26" t="inlineStr">
+        <is>
+          <t>BAU EV Grid Balancing</t>
+        </is>
+      </c>
+      <c r="D85" s="26" t="inlineStr">
+        <is>
+          <t>Fraction of EVs Used for Grid Balancing on Average Day, Fraction of EV Battery Capacity Used for Grid Balancing when EV is Used for Grid Balancing</t>
+        </is>
+      </c>
+      <c r="E85" s="26" t="n"/>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -3161,23 +3174,17 @@
       </c>
       <c r="B86" s="26" t="inlineStr">
         <is>
-          <t>BEVGB</t>
+          <t>BGCL</t>
         </is>
       </c>
       <c r="C86" s="26" t="inlineStr">
         <is>
-          <t>BAU EV Grid Balancing</t>
-        </is>
-      </c>
-      <c r="D86" s="26" t="inlineStr">
-        <is>
-          <t>Fraction of EVs Used for Grid Balancing on Average Day, Fraction of EV Battery Capacity Used for Grid Balancing when EV is Used for Grid Balancing</t>
-        </is>
-      </c>
-      <c r="E86" s="26" t="n"/>
-      <c r="F86" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>BAU Gen Cap Lifetime</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3189,17 +3196,22 @@
       </c>
       <c r="B87" s="26" t="inlineStr">
         <is>
-          <t>BGCL</t>
+          <t>BGDPbES</t>
         </is>
       </c>
       <c r="C87" s="26" t="inlineStr">
         <is>
-          <t>BAU Gen Cap Lifetime</t>
-        </is>
-      </c>
-      <c r="F87" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>BAU Guaranteed Dispatch Percentage by Electricity Source</t>
+        </is>
+      </c>
+      <c r="F87" s="16" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G87" s="26" t="inlineStr">
+        <is>
+          <t>You are modeling a region where power plants are dispatched based on non-market rules rather than by least marginal cost</t>
         </is>
       </c>
     </row>
@@ -3211,22 +3223,22 @@
       </c>
       <c r="B88" s="26" t="inlineStr">
         <is>
-          <t>BGDPbES</t>
+          <t>BHRaSYC</t>
         </is>
       </c>
       <c r="C88" s="26" t="inlineStr">
         <is>
-          <t>BAU Guaranteed Dispatch Percentage by Electricity Source</t>
-        </is>
-      </c>
-      <c r="F88" s="16" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G88" s="26" t="inlineStr">
-        <is>
-          <t>You are modeling a region where power plants are dispatched based on non-market rules rather than by least marginal cost</t>
+          <t>BAU Heat Rates and Start Year Capacities</t>
+        </is>
+      </c>
+      <c r="D88" s="26" t="inlineStr">
+        <is>
+          <t>BAU Heat Rates, BAU Start Year Capacities</t>
+        </is>
+      </c>
+      <c r="F88" s="12" t="inlineStr">
+        <is>
+          <t>very high</t>
         </is>
       </c>
     </row>
@@ -3238,22 +3250,17 @@
       </c>
       <c r="B89" s="26" t="inlineStr">
         <is>
-          <t>BHRaSYC</t>
+          <t>BPHC</t>
         </is>
       </c>
       <c r="C89" s="26" t="inlineStr">
         <is>
-          <t>BAU Heat Rates and Start Year Capacities</t>
-        </is>
-      </c>
-      <c r="D89" s="26" t="inlineStr">
-        <is>
-          <t>BAU Heat Rates, BAU Start Year Capacities</t>
-        </is>
-      </c>
-      <c r="F89" s="12" t="inlineStr">
-        <is>
-          <t>very high</t>
+          <t>BAU Pumped Hydro Capacity</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -3265,17 +3272,22 @@
       </c>
       <c r="B90" s="26" t="inlineStr">
         <is>
-          <t>BPHC</t>
+          <t>BPMCCS</t>
         </is>
       </c>
       <c r="C90" s="26" t="inlineStr">
         <is>
-          <t>BAU Pumped Hydro Capacity</t>
-        </is>
-      </c>
-      <c r="F90" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>BAU Policy Mandated Capacity Construction Schedule</t>
+        </is>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G90" s="26" t="inlineStr">
+        <is>
+          <t>You know particular capacities of particular types of plants will come online in particular years (for example, they are already under construction), or you are modeling a region where power plant construction decisions are based on government mandates rather than being market-driven</t>
         </is>
       </c>
     </row>
@@ -3287,12 +3299,12 @@
       </c>
       <c r="B91" s="26" t="inlineStr">
         <is>
-          <t>BPMCCS</t>
+          <t>BPMCRS</t>
         </is>
       </c>
       <c r="C91" s="26" t="inlineStr">
         <is>
-          <t>BAU Policy Mandated Capacity Construction Schedule</t>
+          <t>BAU Policy Mandated Capacity Retrofit Schedule</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
@@ -3302,24 +3314,24 @@
       </c>
       <c r="G91" s="26" t="inlineStr">
         <is>
-          <t>You know particular capacities of particular types of plants will come online in particular years (for example, they are already under construction), or you are modeling a region where power plant construction decisions are based on government mandates rather than being market-driven</t>
+          <t>You know particular capacities of particular types of plants will be retrofit with CCUS in particular years (for example, they are already under construction), or you are modeling a region where power plant retrofit decisions are based on government mandates rather than being market-driven</t>
         </is>
       </c>
     </row>
     <row r="92" ht="75" customHeight="1" s="27">
-      <c r="A92" s="26" t="inlineStr">
+      <c r="A92" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B92" s="26" t="inlineStr">
-        <is>
-          <t>BPMCRS</t>
-        </is>
-      </c>
-      <c r="C92" s="26" t="inlineStr">
-        <is>
-          <t>BAU Policy Mandated Capacity Retrofit Schedule</t>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>BPMGBSA</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>BAU Policy Mandated Grid Battery Storage Additions</t>
         </is>
       </c>
       <c r="F92" s="16" t="inlineStr">
@@ -3329,34 +3341,29 @@
       </c>
       <c r="G92" s="26" t="inlineStr">
         <is>
-          <t>You know particular capacities of particular types of plants will be retrofit with CCUS in particular years (for example, they are already under construction), or you are modeling a region where power plant retrofit decisions are based on government mandates rather than being market-driven</t>
+          <t>You know particular battery capacity will come online in particular years (for example, they are already under construction), or you are modeling a region where power plant construction decisions are based on government mandates rather than being market-driven</t>
         </is>
       </c>
     </row>
     <row r="93" ht="90" customFormat="1" customHeight="1" s="26">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>BPMGBSA</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>BAU Policy Mandated Grid Battery Storage Additions</t>
-        </is>
-      </c>
-      <c r="F93" s="16" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G93" s="26" t="inlineStr">
-        <is>
-          <t>You know particular battery capacity will come online in particular years (for example, they are already under construction), or you are modeling a region where power plant construction decisions are based on government mandates rather than being market-driven</t>
+      <c r="B93" s="26" t="inlineStr">
+        <is>
+          <t>BPPEOUP</t>
+        </is>
+      </c>
+      <c r="C93" s="26" t="inlineStr">
+        <is>
+          <t>BAU Pwr Plnt Elec Own Use Perc</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3368,17 +3375,17 @@
       </c>
       <c r="B94" s="26" t="inlineStr">
         <is>
-          <t>BPPEOUP</t>
+          <t>BPSpUGBCD</t>
         </is>
       </c>
       <c r="C94" s="26" t="inlineStr">
         <is>
-          <t>BAU Pwr Plnt Elec Own Use Perc</t>
-        </is>
-      </c>
-      <c r="F94" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>BAU Percent Subsidy per Unit Grid Battery Capacity Deployed</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -3390,12 +3397,22 @@
       </c>
       <c r="B95" s="26" t="inlineStr">
         <is>
-          <t>BPSpUGBCD</t>
+          <t>BRPSDbS</t>
         </is>
       </c>
       <c r="C95" s="26" t="inlineStr">
         <is>
-          <t>BAU Percent Subsidy per Unit Grid Battery Capacity Deployed</t>
+          <t>BAU RPS Data by Subregion</t>
+        </is>
+      </c>
+      <c r="D95" s="26" t="inlineStr">
+        <is>
+          <t>BAU RPS Percentages by Subregion, BAU Electricity Shares by Subregion</t>
+        </is>
+      </c>
+      <c r="E95" s="26" t="inlineStr">
+        <is>
+          <t>RQSD</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
@@ -3412,22 +3429,12 @@
       </c>
       <c r="B96" s="26" t="inlineStr">
         <is>
-          <t>BRPSDbS</t>
+          <t>BSfGBP</t>
         </is>
       </c>
       <c r="C96" s="26" t="inlineStr">
         <is>
-          <t>BAU RPS Data by Subregion</t>
-        </is>
-      </c>
-      <c r="D96" s="26" t="inlineStr">
-        <is>
-          <t>BAU RPS Percentages by Subregion, BAU Electricity Shares by Subregion</t>
-        </is>
-      </c>
-      <c r="E96" s="26" t="inlineStr">
-        <is>
-          <t>RQSD</t>
+          <t>BAU Subsidy for Grid Battery Production</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
@@ -3444,12 +3451,12 @@
       </c>
       <c r="B97" s="26" t="inlineStr">
         <is>
-          <t>BSfGBP</t>
+          <t>BTaDLP</t>
         </is>
       </c>
       <c r="C97" s="26" t="inlineStr">
         <is>
-          <t>BAU Subsidy for Grid Battery Production</t>
+          <t>BAU Transmission and Distribution Loss Percentage</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
@@ -3466,17 +3473,17 @@
       </c>
       <c r="B98" s="26" t="inlineStr">
         <is>
-          <t>BTaDLP</t>
+          <t>BZECfNP</t>
         </is>
       </c>
       <c r="C98" s="26" t="inlineStr">
         <is>
-          <t>BAU Transmission and Distribution Loss Percentage</t>
-        </is>
-      </c>
-      <c r="F98" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>BAU Zero Emis Credit for Nuc Plants</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3488,12 +3495,17 @@
       </c>
       <c r="B99" s="26" t="inlineStr">
         <is>
-          <t>BZECfNP</t>
+          <t>CCaMC</t>
         </is>
       </c>
       <c r="C99" s="26" t="inlineStr">
         <is>
-          <t>BAU Zero Emis Credit for Nuc Plants</t>
+          <t>Capacity Construction and Maintenance Costs</t>
+        </is>
+      </c>
+      <c r="D99" s="26" t="inlineStr">
+        <is>
+          <t>Annual CapEx per Unit Capacity, BAU Construction Cost per Unit Capacity, Annual Fixed O&amp;M Cost per Unit Capacity, Variable O&amp;M Cost per Unit Elec Output, BAU Soft Costs per Unit Capacity, Annual CapEx per Unit Capacity, Spur Line Construction Cost per Unit Capacity, BAU CCS Retrofit Costs per Unit Capacity</t>
         </is>
       </c>
       <c r="F99" s="5" t="inlineStr">
@@ -3510,22 +3522,22 @@
       </c>
       <c r="B100" s="26" t="inlineStr">
         <is>
-          <t>CCaMC</t>
+          <t>CRbQ</t>
         </is>
       </c>
       <c r="C100" s="26" t="inlineStr">
         <is>
-          <t>Capacity Construction and Maintenance Costs</t>
-        </is>
-      </c>
-      <c r="D100" s="26" t="inlineStr">
-        <is>
-          <t>Annual CapEx per Unit Capacity, BAU Construction Cost per Unit Capacity, Annual Fixed O&amp;M Cost per Unit Capacity, Variable O&amp;M Cost per Unit Elec Output, BAU Soft Costs per Unit Capacity, Annual CapEx per Unit Capacity, Spur Line Construction Cost per Unit Capacity, BAU CCS Retrofit Costs per Unit Capacity</t>
-        </is>
-      </c>
-      <c r="F100" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>Capacity Retirements before Quantization</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
+        <is>
+          <t>n/a (policy lever)</t>
+        </is>
+      </c>
+      <c r="G100" s="26" t="inlineStr">
+        <is>
+          <t>You wish to switch from the BAU plant retirement schedule to an alternative schedule you have specified in input data (rather than using the early retirement policy lever, which accelerates retirements and is additive to the BAU retirements)</t>
         </is>
       </c>
     </row>
@@ -3537,22 +3549,17 @@
       </c>
       <c r="B101" s="26" t="inlineStr">
         <is>
-          <t>CRbQ</t>
+          <t>CRpUNL</t>
         </is>
       </c>
       <c r="C101" s="26" t="inlineStr">
         <is>
-          <t>Capacity Retirements before Quantization</t>
-        </is>
-      </c>
-      <c r="F101" s="6" t="inlineStr">
-        <is>
-          <t>n/a (policy lever)</t>
-        </is>
-      </c>
-      <c r="G101" s="26" t="inlineStr">
-        <is>
-          <t>You wish to switch from the BAU plant retirement schedule to an alternative schedule you have specified in input data (rather than using the early retirement policy lever, which accelerates retirements and is additive to the BAU retirements)</t>
+          <t>Cap Ret per Unit Net Loss</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3564,12 +3571,17 @@
       </c>
       <c r="B102" s="26" t="inlineStr">
         <is>
-          <t>CRpUNL</t>
+          <t>CSC</t>
         </is>
       </c>
       <c r="C102" s="26" t="inlineStr">
         <is>
-          <t>Cap Ret per Unit Net Loss</t>
+          <t>Capacity Supply Curve</t>
+        </is>
+      </c>
+      <c r="D102" s="26" t="inlineStr">
+        <is>
+          <t>Capacity Supply Curve Capacity Cost Multiplier vs Share of Exisiting Capacity Built This Year, Capacity Supply Curve Minimum Buildable Capacity for Plant Types with No Exisiting Capacity, Capacity Supply Curve Share of Cost Effective Capacity Built in a Single Year, Capacity Supply Curve Share of Cost Effective Hybrid Capacity Built in a Single Year</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
@@ -3586,17 +3598,12 @@
       </c>
       <c r="B103" s="26" t="inlineStr">
         <is>
-          <t>CSC</t>
+          <t>DCCpUIiPL</t>
         </is>
       </c>
       <c r="C103" s="26" t="inlineStr">
         <is>
-          <t>Capacity Supply Curve</t>
-        </is>
-      </c>
-      <c r="D103" s="26" t="inlineStr">
-        <is>
-          <t>Capacity Supply Curve Capacity Cost Multiplier vs Share of Exisiting Capacity Built This Year, Capacity Supply Curve Minimum Buildable Capacity for Plant Types with No Exisiting Capacity, Capacity Supply Curve Share of Cost Effective Capacity Built in a Single Year, Capacity Supply Curve Share of Cost Effective Hybrid Capacity Built in a Single Year</t>
+          <t>Distribution Construction Cost per Unit Increase in Peak Load</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
@@ -3613,17 +3620,17 @@
       </c>
       <c r="B104" s="26" t="inlineStr">
         <is>
-          <t>DCCpUIiPL</t>
+          <t>DCpUC</t>
         </is>
       </c>
       <c r="C104" s="26" t="inlineStr">
         <is>
-          <t>Distribution Construction Cost per Unit Increase in Peak Load</t>
-        </is>
-      </c>
-      <c r="F104" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>Decommissioning Cost per Unit Capacity</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -3635,12 +3642,12 @@
       </c>
       <c r="B105" s="26" t="inlineStr">
         <is>
-          <t>DCpUC</t>
+          <t>DPbES</t>
         </is>
       </c>
       <c r="C105" s="26" t="inlineStr">
         <is>
-          <t>Decommissioning Cost per Unit Capacity</t>
+          <t>Dispatch Priority by Electricity Source</t>
         </is>
       </c>
       <c r="F105" s="4" t="inlineStr">
@@ -3657,17 +3664,22 @@
       </c>
       <c r="B106" s="26" t="inlineStr">
         <is>
-          <t>DPbES</t>
+          <t>DRC</t>
         </is>
       </c>
       <c r="C106" s="26" t="inlineStr">
         <is>
-          <t>Dispatch Priority by Electricity Source</t>
-        </is>
-      </c>
-      <c r="F106" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>Demand Response Capacities</t>
+        </is>
+      </c>
+      <c r="D106" s="26" t="inlineStr">
+        <is>
+          <t>BAU Demand Response Capacity, Potential Additional Demand Response Capacity, Average DR Hours per DR Event</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -3679,98 +3691,98 @@
       </c>
       <c r="B107" s="26" t="inlineStr">
         <is>
-          <t>DRC</t>
+          <t>DRCo</t>
         </is>
       </c>
       <c r="C107" s="26" t="inlineStr">
         <is>
-          <t>Demand Response Capacities</t>
+          <t>Demand Response Costs</t>
         </is>
       </c>
       <c r="D107" s="26" t="inlineStr">
         <is>
-          <t>BAU Demand Response Capacity, Potential Additional Demand Response Capacity, Average DR Hours per DR Event</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="inlineStr">
+          <t>Annual Cost per Unit Demand Response Capacity, Share of DR by Provider</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="30" customHeight="1" s="27">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>elec</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>DUVT</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Deep Unviability Threshold</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" customFormat="1" s="26">
+      <c r="A109" s="26" t="inlineStr">
+        <is>
+          <t>elec</t>
+        </is>
+      </c>
+      <c r="B109" s="26" t="inlineStr">
+        <is>
+          <t>EIaE</t>
+        </is>
+      </c>
+      <c r="C109" s="26" t="inlineStr">
+        <is>
+          <t>Electricity Imports and Exports</t>
+        </is>
+      </c>
+      <c r="D109" s="26" t="inlineStr">
+        <is>
+          <t>BAU Imported Electricity, BAU Exported Electricity, Imported Electricity Price</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="30" customHeight="1" s="27">
-      <c r="A108" s="26" t="inlineStr">
+    <row r="110" ht="30" customHeight="1" s="27">
+      <c r="A110" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B108" s="26" t="inlineStr">
-        <is>
-          <t>DRCo</t>
-        </is>
-      </c>
-      <c r="C108" s="26" t="inlineStr">
-        <is>
-          <t>Demand Response Costs</t>
-        </is>
-      </c>
-      <c r="D108" s="26" t="inlineStr">
-        <is>
-          <t>Annual Cost per Unit Demand Response Capacity, Share of DR by Provider</t>
-        </is>
-      </c>
-      <c r="F108" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" customFormat="1" s="26">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>elec</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>DUVT</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Deep Unviability Threshold</t>
-        </is>
-      </c>
-      <c r="F109" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="30" customHeight="1" s="27">
-      <c r="A110" s="26" t="inlineStr">
-        <is>
-          <t>elec</t>
-        </is>
-      </c>
-      <c r="B110" s="26" t="inlineStr">
-        <is>
-          <t>EIaE</t>
-        </is>
-      </c>
-      <c r="C110" s="26" t="inlineStr">
-        <is>
-          <t>Electricity Imports and Exports</t>
-        </is>
-      </c>
-      <c r="D110" s="26" t="inlineStr">
-        <is>
-          <t>BAU Imported Electricity, BAU Exported Electricity, Imported Electricity Price</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>ELCCAfR</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ELCC Adjustment for Reliability</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>ELCC Adjustment for Reliability for Generation Sources, ELCC Adjustment for Reliability for Demand Altering Technologies</t>
+        </is>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3782,46 +3794,47 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ELCCAfR</t>
+          <t>EPQSD</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ELCC Adjustment for Reliability</t>
+          <t>Elec Portfolio Qualifying Source Definitions</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>ELCC Adjustment for Reliability for Generation Sources, ELCC Adjustment for Reliability for Demand Altering Technologies</t>
-        </is>
-      </c>
-      <c r="F111" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>RPS Qualifying Source Definitions, CES Qualifying Source Definitions</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
     <row r="112" customFormat="1" s="26">
-      <c r="A112" t="inlineStr">
+      <c r="A112" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>EPQSD</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Elec Portfolio Qualifying Source Definitions</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>RPS Qualifying Source Definitions, CES Qualifying Source Definitions</t>
-        </is>
-      </c>
+      <c r="B112" s="26" t="inlineStr">
+        <is>
+          <t>ESTRTE</t>
+        </is>
+      </c>
+      <c r="C112" s="26" t="inlineStr">
+        <is>
+          <t>Electricity Storage Technology Round-Trip Efficiency</t>
+        </is>
+      </c>
+      <c r="D112" s="26" t="inlineStr">
+        <is>
+          <t>Grid Battery Rount-Trip Efficiency, Pumped Hydro Round-Trip Efficiency</t>
+        </is>
+      </c>
+      <c r="E112" s="26" t="n"/>
       <c r="F112" s="4" t="inlineStr">
         <is>
           <t>low</t>
@@ -3829,27 +3842,21 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="26" t="inlineStr">
+      <c r="A113" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B113" s="26" t="inlineStr">
-        <is>
-          <t>ESTRTE</t>
-        </is>
-      </c>
-      <c r="C113" s="26" t="inlineStr">
-        <is>
-          <t>Electricity Storage Technology Round-Trip Efficiency</t>
-        </is>
-      </c>
-      <c r="D113" s="26" t="inlineStr">
-        <is>
-          <t>Grid Battery Rount-Trip Efficiency, Pumped Hydro Round-Trip Efficiency</t>
-        </is>
-      </c>
-      <c r="E113" s="26" t="n"/>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>FOAKCFoF</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>First of a Kind Capacity Fraction of Fleet</t>
+        </is>
+      </c>
       <c r="F113" s="4" t="inlineStr">
         <is>
           <t>low</t>
@@ -3857,24 +3864,24 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
+      <c r="A114" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>FOAKCFoF</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>First of a Kind Capacity Fraction of Fleet</t>
-        </is>
-      </c>
-      <c r="F114" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="B114" s="26" t="inlineStr">
+        <is>
+          <t>FoGBPD</t>
+        </is>
+      </c>
+      <c r="C114" s="26" t="inlineStr">
+        <is>
+          <t>Fraction of Grid Batteries Produced Domestically</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -3886,17 +3893,17 @@
       </c>
       <c r="B115" s="26" t="inlineStr">
         <is>
-          <t>FoGBPD</t>
+          <t>GBCGpUNR</t>
         </is>
       </c>
       <c r="C115" s="26" t="inlineStr">
         <is>
-          <t>Fraction of Grid Batteries Produced Domestically</t>
-        </is>
-      </c>
-      <c r="F115" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>Grid Battery Capacity Growth per Unit Net Revenue</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -3908,17 +3915,22 @@
       </c>
       <c r="B116" s="26" t="inlineStr">
         <is>
-          <t>GBCGpUNR</t>
+          <t>GBSC</t>
         </is>
       </c>
       <c r="C116" s="26" t="inlineStr">
         <is>
-          <t>Grid Battery Capacity Growth per Unit Net Revenue</t>
-        </is>
-      </c>
-      <c r="F116" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>Grid Battery Storage Capacities</t>
+        </is>
+      </c>
+      <c r="D116" s="26" t="inlineStr">
+        <is>
+          <t>Start Year Grid Battery Storage Capacity, Grid Battery Daily Storage Duration</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -3930,22 +3942,22 @@
       </c>
       <c r="B117" s="26" t="inlineStr">
         <is>
-          <t>GBSC</t>
+          <t>GDPbES</t>
         </is>
       </c>
       <c r="C117" s="26" t="inlineStr">
         <is>
-          <t>Grid Battery Storage Capacities</t>
-        </is>
-      </c>
-      <c r="D117" s="26" t="inlineStr">
-        <is>
-          <t>Start Year Grid Battery Storage Capacity, Grid Battery Daily Storage Duration</t>
-        </is>
-      </c>
-      <c r="F117" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>Guaranteed Dispatch Percentage by Electricity Source</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>n/a (policy lever)</t>
+        </is>
+      </c>
+      <c r="G117" s="26" t="inlineStr">
+        <is>
+          <t>You are modeling a region where power plants are dispatched based on non-market rules rather than by least marginal cost, and you are setting this policy lever to alter the BAU percentages</t>
         </is>
       </c>
     </row>
@@ -3957,39 +3969,34 @@
       </c>
       <c r="B118" s="26" t="inlineStr">
         <is>
-          <t>GDPbES</t>
+          <t>GHESLE</t>
         </is>
       </c>
       <c r="C118" s="26" t="inlineStr">
         <is>
-          <t>Guaranteed Dispatch Percentage by Electricity Source</t>
-        </is>
-      </c>
-      <c r="F118" s="6" t="inlineStr">
-        <is>
-          <t>n/a (policy lever)</t>
-        </is>
-      </c>
-      <c r="G118" s="26" t="inlineStr">
-        <is>
-          <t>You are modeling a region where power plants are dispatched based on non-market rules rather than by least marginal cost, and you are setting this policy lever to alter the BAU percentages</t>
+          <t>Green Hydrogen Electricity Supply Logit Exponent</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="26" t="inlineStr">
+      <c r="A119" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
       <c r="B119" s="26" t="inlineStr">
         <is>
-          <t>GHESLE</t>
+          <t>GHESS</t>
         </is>
       </c>
       <c r="C119" s="26" t="inlineStr">
         <is>
-          <t>Green Hydrogen Electricity Supply Logit Exponent</t>
+          <t>Green Hydrogen Electricity Supply Shareweights</t>
         </is>
       </c>
       <c r="F119" s="5" t="inlineStr">
@@ -4004,14 +4011,14 @@
           <t>elec</t>
         </is>
       </c>
-      <c r="B120" s="26" t="inlineStr">
-        <is>
-          <t>GHESS</t>
-        </is>
-      </c>
-      <c r="C120" s="26" t="inlineStr">
-        <is>
-          <t>Green Hydrogen Electricity Supply Shareweights</t>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>HCFoTC</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Hard Cap Fraction of Total Capacity</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
@@ -4021,24 +4028,24 @@
       </c>
     </row>
     <row r="121" ht="30" customFormat="1" customHeight="1" s="26">
-      <c r="A121" t="inlineStr">
+      <c r="A121" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>HCFoTC</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Hard Cap Fraction of Total Capacity</t>
-        </is>
-      </c>
-      <c r="F121" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="B121" s="26" t="inlineStr">
+        <is>
+          <t>HESBCpUEC</t>
+        </is>
+      </c>
+      <c r="C121" s="26" t="inlineStr">
+        <is>
+          <t>Hybrid Electricity Source Battery Capacity per Unit Electricity Capacity</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -4050,12 +4057,12 @@
       </c>
       <c r="B122" s="26" t="inlineStr">
         <is>
-          <t>HESBCpUEC</t>
+          <t>HOC</t>
         </is>
       </c>
       <c r="C122" s="26" t="inlineStr">
         <is>
-          <t>Hybrid Electricity Source Battery Capacity per Unit Electricity Capacity</t>
+          <t>Hydro Opportunity Cost</t>
         </is>
       </c>
       <c r="F122" s="4" t="inlineStr">
@@ -4065,19 +4072,19 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="26" t="inlineStr">
+      <c r="A123" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B123" s="26" t="inlineStr">
-        <is>
-          <t>HOC</t>
-        </is>
-      </c>
-      <c r="C123" s="26" t="inlineStr">
-        <is>
-          <t>Hydro Opportunity Cost</t>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>HSSfBA</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Half Saturation Share for Buildable Additions</t>
         </is>
       </c>
       <c r="F123" s="4" t="inlineStr">
@@ -4094,12 +4101,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>HSSfBA</t>
+          <t>HYECFCA</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Half Saturation Share for Buildable Additions</t>
+          <t>Historical Year Electricity Capacity Factor Calibration Adjustment</t>
         </is>
       </c>
       <c r="F124" s="4" t="inlineStr">
@@ -4109,19 +4116,19 @@
       </c>
     </row>
     <row r="125" ht="45" customFormat="1" customHeight="1" s="26">
-      <c r="A125" t="inlineStr">
+      <c r="A125" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>HYECFCA</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Historical Year Electricity Capacity Factor Calibration Adjustment</t>
+      <c r="B125" s="26" t="inlineStr">
+        <is>
+          <t>IiCFfNPdtTI</t>
+        </is>
+      </c>
+      <c r="C125" s="26" t="inlineStr">
+        <is>
+          <t>Increase in Capacity Factors for New Plants due to Technological Improvements</t>
         </is>
       </c>
       <c r="F125" s="4" t="inlineStr">
@@ -4138,17 +4145,17 @@
       </c>
       <c r="B126" s="26" t="inlineStr">
         <is>
-          <t>IiCFfNPdtTI</t>
+          <t>LFHVM</t>
         </is>
       </c>
       <c r="C126" s="26" t="inlineStr">
         <is>
-          <t>Increase in Capacity Factors for New Plants due to Technological Improvements</t>
-        </is>
-      </c>
-      <c r="F126" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>Load Factor Hourly Variance Multiplier</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -4160,12 +4167,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>KMPPC</t>
+          <t>MABAaSoF</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Typical Units Retired in a Peak Year</t>
+          <t>Max Annual Buildable Additions as Share of Fleet</t>
         </is>
       </c>
       <c r="F127" s="4" t="inlineStr">
@@ -4182,12 +4189,12 @@
       </c>
       <c r="B128" s="26" t="inlineStr">
         <is>
-          <t>LFHVM</t>
+          <t>MaMHEIaE</t>
         </is>
       </c>
       <c r="C128" s="26" t="inlineStr">
         <is>
-          <t>Load Factor Hourly Variance Multiplier</t>
+          <t>Max and Min Hourly Electriicty Imports and Exports</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
@@ -4197,19 +4204,19 @@
       </c>
     </row>
     <row r="129" ht="30" customFormat="1" customHeight="1" s="26">
-      <c r="A129" t="inlineStr">
+      <c r="A129" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>MABAaSoF</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>Max Annual Buildable Additions as Share of Fleet</t>
+      <c r="B129" s="26" t="inlineStr">
+        <is>
+          <t>MCF</t>
+        </is>
+      </c>
+      <c r="C129" s="26" t="inlineStr">
+        <is>
+          <t>Maximum Capacity Factor</t>
         </is>
       </c>
       <c r="F129" s="4" t="inlineStr">
@@ -4226,17 +4233,17 @@
       </c>
       <c r="B130" s="26" t="inlineStr">
         <is>
-          <t>MaMHEIaE</t>
+          <t>MLfPPR</t>
         </is>
       </c>
       <c r="C130" s="26" t="inlineStr">
         <is>
-          <t>Max and Min Hourly Electriicty Imports and Exports</t>
-        </is>
-      </c>
-      <c r="F130" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>Min Life for Pwr Plnt Rtmnts</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -4248,17 +4255,17 @@
       </c>
       <c r="B131" s="26" t="inlineStr">
         <is>
-          <t>MCF</t>
+          <t>MPCbS</t>
         </is>
       </c>
       <c r="C131" s="26" t="inlineStr">
         <is>
-          <t>Maximum Capacity Factor</t>
-        </is>
-      </c>
-      <c r="F131" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>Max Potential Capacity by Source</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -4270,12 +4277,12 @@
       </c>
       <c r="B132" s="26" t="inlineStr">
         <is>
-          <t>MLfPPR</t>
+          <t>MPPC</t>
         </is>
       </c>
       <c r="C132" s="26" t="inlineStr">
         <is>
-          <t>Min Life for Pwr Plnt Rtmnts</t>
+          <t>Minimum Power Plant Capacity</t>
         </is>
       </c>
       <c r="F132" s="4" t="inlineStr">
@@ -4285,117 +4292,127 @@
       </c>
     </row>
     <row r="133" ht="30" customHeight="1" s="27">
-      <c r="A133" s="26" t="inlineStr">
+      <c r="A133" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B133" s="26" t="inlineStr">
-        <is>
-          <t>MPCbS</t>
-        </is>
-      </c>
-      <c r="C133" s="26" t="inlineStr">
-        <is>
-          <t>Max Potential Capacity by Source</t>
-        </is>
-      </c>
-      <c r="F133" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>MSoCRiaSY</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Maximum Share of Capacity Retired in a Single Year</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
     <row r="134" ht="30" customHeight="1" s="27">
-      <c r="A134" s="26" t="inlineStr">
+      <c r="A134" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B134" s="26" t="inlineStr">
-        <is>
-          <t>MPPC</t>
-        </is>
-      </c>
-      <c r="C134" s="26" t="inlineStr">
-        <is>
-          <t>Minimum Power Plant Capacity</t>
-        </is>
-      </c>
-      <c r="F134" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>NSDoDC</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Normalized Standard Deviation of Dispatch Costs</t>
+        </is>
+      </c>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
     <row r="135" customFormat="1" s="26">
-      <c r="A135" t="inlineStr">
+      <c r="A135" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>MSoCRiaSY</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>Maximum Share of Capacity Retired in a Single Year</t>
-        </is>
-      </c>
-      <c r="F135" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="B135" s="26" t="inlineStr">
+        <is>
+          <t>PMCCS</t>
+        </is>
+      </c>
+      <c r="C135" s="26" t="inlineStr">
+        <is>
+          <t>Policy Mandated Capacity Construction Schedule</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>n/a (policy lever)</t>
+        </is>
+      </c>
+      <c r="G135" s="26" t="inlineStr">
+        <is>
+          <t>You are modeling a region where power plant construction decisions are based on government mandates rather than being market-driven, and you are setting this policy lever to alter the BAU mandates</t>
         </is>
       </c>
     </row>
     <row r="136" ht="60.75" customFormat="1" customHeight="1" s="26" thickBot="1">
-      <c r="A136" t="inlineStr">
+      <c r="A136" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>NSDoDC</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>Normalized Standard Deviation of Dispatch Costs</t>
-        </is>
-      </c>
-      <c r="F136" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="B136" s="26" t="inlineStr">
+        <is>
+          <t>PMCRS</t>
+        </is>
+      </c>
+      <c r="C136" s="26" t="inlineStr">
+        <is>
+          <t>Policy Mandated Capacity Retrofit Schedule</t>
+        </is>
+      </c>
+      <c r="F136" s="6" t="inlineStr">
+        <is>
+          <t>n/a (policy lever)</t>
+        </is>
+      </c>
+      <c r="G136" s="26" t="inlineStr">
+        <is>
+          <t>You are modeling a region where power plant CCUS retrofit decisions are based on government mandates rather than being market-driven, and you are setting this policy lever to alter the BAU mandates</t>
         </is>
       </c>
     </row>
     <row r="137" ht="30" customHeight="1" s="27">
-      <c r="A137" s="26" t="inlineStr">
+      <c r="A137" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B137" s="26" t="inlineStr">
-        <is>
-          <t>PMCCS</t>
-        </is>
-      </c>
-      <c r="C137" s="26" t="inlineStr">
-        <is>
-          <t>Policy Mandated Capacity Construction Schedule</t>
-        </is>
-      </c>
-      <c r="F137" s="6" t="inlineStr">
-        <is>
-          <t>n/a (policy lever)</t>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>PMGBSA</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Policy Mandated Grid Battery Storage Additions</t>
+        </is>
+      </c>
+      <c r="F137" s="16" t="inlineStr">
+        <is>
+          <t>optional</t>
         </is>
       </c>
       <c r="G137" s="26" t="inlineStr">
         <is>
-          <t>You are modeling a region where power plant construction decisions are based on government mandates rather than being market-driven, and you are setting this policy lever to alter the BAU mandates</t>
+          <t>You know particular battery capacity will come online in particular years (for example, they are already under construction), or you are modeling a region where power plant construction decisions are based on government mandates rather than being market-driven</t>
         </is>
       </c>
     </row>
@@ -4407,71 +4424,71 @@
       </c>
       <c r="B138" s="26" t="inlineStr">
         <is>
-          <t>PMCRS</t>
+          <t>RACP</t>
         </is>
       </c>
       <c r="C138" s="26" t="inlineStr">
         <is>
-          <t>Policy Mandated Capacity Retrofit Schedule</t>
-        </is>
-      </c>
-      <c r="F138" s="6" t="inlineStr">
-        <is>
-          <t>n/a (policy lever)</t>
-        </is>
-      </c>
-      <c r="G138" s="26" t="inlineStr">
-        <is>
-          <t>You are modeling a region where power plant CCUS retrofit decisions are based on government mandates rather than being market-driven, and you are setting this policy lever to alter the BAU mandates</t>
+          <t>RPS Alternative Compliance Payment</t>
+        </is>
+      </c>
+      <c r="D138" s="26" t="inlineStr">
+        <is>
+          <t>BAU RPS Alternative Compliance Payment, RPS Alternative Compliance Payment</t>
+        </is>
+      </c>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
     <row r="139" ht="75" customFormat="1" customHeight="1" s="26">
-      <c r="A139" t="inlineStr">
+      <c r="A139" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>PMGBSA</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>Policy Mandated Grid Battery Storage Additions</t>
-        </is>
-      </c>
-      <c r="F139" s="16" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G139" s="26" t="inlineStr">
-        <is>
-          <t>You know particular battery capacity will come online in particular years (for example, they are already under construction), or you are modeling a region where power plant construction decisions are based on government mandates rather than being market-driven</t>
+      <c r="B139" s="26" t="inlineStr">
+        <is>
+          <t>RAF</t>
+        </is>
+      </c>
+      <c r="C139" s="26" t="inlineStr">
+        <is>
+          <t>Regional Availability Factor</t>
+        </is>
+      </c>
+      <c r="D139" s="26" t="inlineStr">
+        <is>
+          <t>Regional Availability Factor for Generation, Regional Availability Factor for Capacity, Regional Availability Factor for Demand-Altering Technologies</t>
+        </is>
+      </c>
+      <c r="F139" s="14" t="inlineStr">
+        <is>
+          <t>to be determined via calibration</t>
         </is>
       </c>
     </row>
     <row r="140" ht="30" customHeight="1" s="27">
-      <c r="A140" s="26" t="inlineStr">
+      <c r="A140" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B140" s="26" t="inlineStr">
-        <is>
-          <t>RACP</t>
-        </is>
-      </c>
-      <c r="C140" s="26" t="inlineStr">
-        <is>
-          <t>RPS Alternative Compliance Payment</t>
-        </is>
-      </c>
-      <c r="D140" s="26" t="inlineStr">
-        <is>
-          <t>BAU RPS Alternative Compliance Payment, RPS Alternative Compliance Payment</t>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>RCDC</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Reliability Credit Derate Curve</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Reliability Credit Derate Curve Shape Parameter, Reliability Credit Derate Curve Scale Parameter</t>
         </is>
       </c>
       <c r="F140" s="5" t="inlineStr">
@@ -4488,49 +4505,44 @@
       </c>
       <c r="B141" s="26" t="inlineStr">
         <is>
-          <t>RAF</t>
+          <t>RLYr</t>
         </is>
       </c>
       <c r="C141" s="26" t="inlineStr">
         <is>
-          <t>Regional Availability Factor</t>
-        </is>
-      </c>
-      <c r="D141" s="26" t="inlineStr">
-        <is>
-          <t>Regional Availability Factor for Generation, Regional Availability Factor for Capacity, Regional Availability Factor for Demand-Altering Technologies</t>
-        </is>
-      </c>
-      <c r="F141" s="14" t="inlineStr">
-        <is>
-          <t>to be determined via calibration</t>
+          <t>Reliability Lookahead Years</t>
+        </is>
+      </c>
+      <c r="F141" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G141" s="24" t="inlineStr">
+        <is>
+          <t>You want the reliability mechanism to plan over a horizon other than the default 5 years (for example, to match the lead time of the marginal firm capacity resource in your region).</t>
         </is>
       </c>
     </row>
     <row r="142" ht="30" customFormat="1" customHeight="1" s="26">
-      <c r="A142" t="inlineStr">
+      <c r="A142" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>RCDC</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>Reliability Credit Derate Curve</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>Reliability Credit Derate Curve Shape Parameter, Reliability Credit Derate Curve Scale Parameter</t>
-        </is>
-      </c>
-      <c r="F142" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="B142" s="26" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="C142" s="26" t="inlineStr">
+        <is>
+          <t>Reserve Margin</t>
+        </is>
+      </c>
+      <c r="F142" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -4542,12 +4554,12 @@
       </c>
       <c r="B143" s="26" t="inlineStr">
         <is>
-          <t>RLYr</t>
+          <t>RPfFESCC</t>
         </is>
       </c>
       <c r="C143" s="26" t="inlineStr">
         <is>
-          <t>Reliability Lookahead Years</t>
+          <t>Repayment Period for Financed Electricity Sector Capital Costs</t>
         </is>
       </c>
       <c r="F143" s="4" t="inlineStr">
@@ -4555,80 +4567,80 @@
           <t>low</t>
         </is>
       </c>
-      <c r="G143" s="24" t="inlineStr">
-        <is>
-          <t>You want the reliability mechanism to plan over a horizon other than the default 5 years (for example, to match the lead time of the marginal firm capacity resource in your region).</t>
-        </is>
-      </c>
     </row>
     <row r="144" ht="30" customHeight="1" s="27">
-      <c r="A144" s="26" t="inlineStr">
+      <c r="A144" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B144" s="26" t="inlineStr">
-        <is>
-          <t>RM</t>
-        </is>
-      </c>
-      <c r="C144" s="26" t="inlineStr">
-        <is>
-          <t>Reserve Margin</t>
-        </is>
-      </c>
-      <c r="F144" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>RPSDbS</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>RPS Data by Subregion</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>RPS Percentages by Subregion, CES Percentages by Subregion</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
     <row r="145" ht="30" customFormat="1" customHeight="1" s="26">
-      <c r="A145" s="26" t="inlineStr">
+      <c r="A145" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B145" s="26" t="inlineStr">
-        <is>
-          <t>RPfFESCC</t>
-        </is>
-      </c>
-      <c r="C145" s="26" t="inlineStr">
-        <is>
-          <t>Repayment Period for Financed Electricity Sector Capital Costs</t>
-        </is>
-      </c>
-      <c r="F145" s="4" t="inlineStr">
+      <c r="B145" s="29" t="inlineStr">
+        <is>
+          <t>RSLfUF</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Retirement Schedule Length for Unviable Fleets</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
     </row>
     <row r="146" ht="45" customHeight="1" s="27">
-      <c r="A146" t="inlineStr">
+      <c r="A146" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>RPSDbS</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>RPS Data by Subregion</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>RPS Percentages by Subregion, CES Percentages by Subregion</t>
-        </is>
-      </c>
-      <c r="F146" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+      <c r="B146" s="26" t="inlineStr">
+        <is>
+          <t>SES</t>
+        </is>
+      </c>
+      <c r="C146" s="26" t="inlineStr">
+        <is>
+          <t>Seasonal Electricity Storage</t>
+        </is>
+      </c>
+      <c r="D146" s="26" t="inlineStr">
+        <is>
+          <t>Seasonal Electricity Storage Capacity, Seasonal Electricity Storage Annual Charge and Discharge Cycles, Seasonal Electricity Storage Round Trip Efficiency</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
@@ -4640,49 +4652,44 @@
       </c>
       <c r="B147" s="26" t="inlineStr">
         <is>
-          <t>SES</t>
+          <t>SHELF</t>
         </is>
       </c>
       <c r="C147" s="26" t="inlineStr">
         <is>
-          <t>Seasonal Electricity Storage</t>
+          <t>Seasonal Hourly Equipment Load Factors</t>
         </is>
       </c>
       <c r="D147" s="26" t="inlineStr">
         <is>
-          <t>Seasonal Electricity Storage Capacity, Seasonal Electricity Storage Annual Charge and Discharge Cycles, Seasonal Electricity Storage Round Trip Efficiency</t>
-        </is>
-      </c>
-      <c r="F147" s="5" t="inlineStr">
+          <t>Seasonal Hourly Equipment Load Factors, Days per Timeslice</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" customFormat="1" s="26">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>elec</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>SoCtICoS</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Share of Capacity that Is Cost of Service</t>
+        </is>
+      </c>
+      <c r="F148" s="5" t="inlineStr">
         <is>
           <t>medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="148" customFormat="1" s="26">
-      <c r="A148" s="26" t="inlineStr">
-        <is>
-          <t>elec</t>
-        </is>
-      </c>
-      <c r="B148" s="26" t="inlineStr">
-        <is>
-          <t>SHELF</t>
-        </is>
-      </c>
-      <c r="C148" s="26" t="inlineStr">
-        <is>
-          <t>Seasonal Hourly Equipment Load Factors</t>
-        </is>
-      </c>
-      <c r="D148" s="26" t="inlineStr">
-        <is>
-          <t>Seasonal Hourly Equipment Load Factors, Days per Timeslice</t>
-        </is>
-      </c>
-      <c r="F148" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
         </is>
       </c>
     </row>
@@ -4692,19 +4699,19 @@
           <t>elec</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>SoCtICoS</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Share of Capacity that Is Cost of Service</t>
-        </is>
-      </c>
-      <c r="F149" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="B149" s="26" t="inlineStr">
+        <is>
+          <t>SoCtMbCtbDP</t>
+        </is>
+      </c>
+      <c r="C149" s="26" t="inlineStr">
+        <is>
+          <t>Share of Costs that Must be Covered to be Deemed Profitable</t>
+        </is>
+      </c>
+      <c r="F149" s="14" t="inlineStr">
+        <is>
+          <t>to be determined via calibration</t>
         </is>
       </c>
     </row>
@@ -4714,41 +4721,46 @@
           <t>elec</t>
         </is>
       </c>
-      <c r="B150" s="26" t="inlineStr">
-        <is>
-          <t>SoCtMbCtbDP</t>
-        </is>
-      </c>
-      <c r="C150" s="26" t="inlineStr">
-        <is>
-          <t>Share of Costs that Must be Covered to be Deemed Profitable</t>
-        </is>
-      </c>
-      <c r="F150" s="14" t="inlineStr">
-        <is>
-          <t>to be determined via calibration</t>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>SoEDtICoS</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Share of Electricity Demand that Is Cost of Service</t>
+        </is>
+      </c>
+      <c r="F150" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
     <row r="151" ht="30" customHeight="1" s="27">
-      <c r="A151" t="inlineStr">
+      <c r="A151" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>SoEDtICoS</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>Share of Electricity Demand that Is Cost of Service</t>
-        </is>
-      </c>
-      <c r="F151" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="B151" s="26" t="inlineStr">
+        <is>
+          <t>SoESCaOMCbIC</t>
+        </is>
+      </c>
+      <c r="C151" s="26" t="inlineStr">
+        <is>
+          <t>Share of Electricity Sector Capital and OM Costs by ISIC Code</t>
+        </is>
+      </c>
+      <c r="D151" s="26" t="inlineStr">
+        <is>
+          <t>Share of Electricity Sector Capital Costs by ISIC Code, Share of Electricity Sector Fixed OM Costs by ISIC Code, Share of Electricity Sector Variable OM Costs by ISIC Code</t>
+        </is>
+      </c>
+      <c r="F151" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -4760,44 +4772,39 @@
       </c>
       <c r="B152" s="26" t="inlineStr">
         <is>
-          <t>SoESCaOMCbIC</t>
+          <t>SoFCtMbCtPR</t>
         </is>
       </c>
       <c r="C152" s="26" t="inlineStr">
         <is>
-          <t>Share of Electricity Sector Capital and OM Costs by ISIC Code</t>
-        </is>
-      </c>
-      <c r="D152" s="26" t="inlineStr">
-        <is>
-          <t>Share of Electricity Sector Capital Costs by ISIC Code, Share of Electricity Sector Fixed OM Costs by ISIC Code, Share of Electricity Sector Variable OM Costs by ISIC Code</t>
-        </is>
-      </c>
-      <c r="F152" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>Share of Forward Costs that Must be Covered to Prevent Retirement</t>
+        </is>
+      </c>
+      <c r="F152" s="14" t="inlineStr">
+        <is>
+          <t>to be determined via calibration</t>
         </is>
       </c>
     </row>
     <row r="153" customFormat="1" s="26">
-      <c r="A153" s="26" t="inlineStr">
+      <c r="A153" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B153" s="26" t="inlineStr">
-        <is>
-          <t>SoFCtMbCtPR</t>
-        </is>
-      </c>
-      <c r="C153" s="26" t="inlineStr">
-        <is>
-          <t>Share of Forward Costs that Must be Covered to Prevent Retirement</t>
-        </is>
-      </c>
-      <c r="F153" s="14" t="inlineStr">
-        <is>
-          <t>to be determined via calibration</t>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SoFCtMbCtPRCoS</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Share of Forward Costs that Must Be Covered to Prevent Retirement for Cost of Service Plants</t>
+        </is>
+      </c>
+      <c r="F153" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -4809,12 +4816,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>SoFCtMbCtPRCoS</t>
+          <t>SoFCtMbCtPRM</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Share of Forward Costs that Must Be Covered to Prevent Retirement for Cost of Service Plants</t>
+          <t>Share of Forward Costs that Must Be Covered to Prevent Retirement for Merchant Plants</t>
         </is>
       </c>
       <c r="F154" s="4" t="inlineStr">
@@ -4824,19 +4831,19 @@
       </c>
     </row>
     <row r="155" ht="30" customHeight="1" s="27">
-      <c r="A155" t="inlineStr">
+      <c r="A155" s="26" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>SoFCtMbCtPRM</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>Share of Forward Costs that Must Be Covered to Prevent Retirement for Merchant Plants</t>
+      <c r="B155" s="26" t="inlineStr">
+        <is>
+          <t>SoTaDCCbIC</t>
+        </is>
+      </c>
+      <c r="C155" s="26" t="inlineStr">
+        <is>
+          <t>Share of Transmission and Distribution Capital Costs by ISIC Code</t>
         </is>
       </c>
       <c r="F155" s="4" t="inlineStr">
@@ -4853,12 +4860,12 @@
       </c>
       <c r="B156" s="26" t="inlineStr">
         <is>
-          <t>SoTaDCCbIC</t>
+          <t>SoTaDOMCbIC</t>
         </is>
       </c>
       <c r="C156" s="26" t="inlineStr">
         <is>
-          <t>Share of Transmission and Distribution Capital Costs by ISIC Code</t>
+          <t>Share of Transmission and Distribution OM Costs by ISIC Code</t>
         </is>
       </c>
       <c r="F156" s="4" t="inlineStr">
@@ -4875,12 +4882,12 @@
       </c>
       <c r="B157" s="26" t="inlineStr">
         <is>
-          <t>SoTaDOMCbIC</t>
+          <t>STfESCE</t>
         </is>
       </c>
       <c r="C157" s="26" t="inlineStr">
         <is>
-          <t>Share of Transmission and Distribution OM Costs by ISIC Code</t>
+          <t>Smoothing Time for Electricity Sector Capital Expenditures</t>
         </is>
       </c>
       <c r="F157" s="4" t="inlineStr">
@@ -4897,17 +4904,17 @@
       </c>
       <c r="B158" s="26" t="inlineStr">
         <is>
-          <t>STfESCE</t>
+          <t>SYPEL</t>
         </is>
       </c>
       <c r="C158" s="26" t="inlineStr">
         <is>
-          <t>Smoothing Time for Electricity Sector Capital Expenditures</t>
-        </is>
-      </c>
-      <c r="F158" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>Start Year Peak Electricity Load</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
     </row>
@@ -4919,12 +4926,17 @@
       </c>
       <c r="B159" s="26" t="inlineStr">
         <is>
-          <t>SYPEL</t>
+          <t>SYSHECF</t>
         </is>
       </c>
       <c r="C159" s="26" t="inlineStr">
         <is>
-          <t>Start Year Peak Electricity Load</t>
+          <t>Start Year Seasonal Expected Hourly Capacity Factors</t>
+        </is>
+      </c>
+      <c r="E159" s="26" t="inlineStr">
+        <is>
+          <t>MCF</t>
         </is>
       </c>
       <c r="F159" s="3" t="inlineStr">
@@ -4941,17 +4953,17 @@
       </c>
       <c r="B160" s="26" t="inlineStr">
         <is>
-          <t>SYSHECF</t>
+          <t>SYTaDC</t>
         </is>
       </c>
       <c r="C160" s="26" t="inlineStr">
         <is>
-          <t>Start Year Seasonal Expected Hourly Capacity Factors</t>
-        </is>
-      </c>
-      <c r="E160" s="26" t="inlineStr">
-        <is>
-          <t>MCF</t>
+          <t>Start Year Transmission and Distribution Costs</t>
+        </is>
+      </c>
+      <c r="D160" s="26" t="inlineStr">
+        <is>
+          <t>Start Year Transmission Capital Costs, Start Year Distribution Capital Costs, Start Year Transmission OM Costs, Start Year Distribution OM Costs</t>
         </is>
       </c>
       <c r="F160" s="3" t="inlineStr">
@@ -4968,22 +4980,17 @@
       </c>
       <c r="B161" s="26" t="inlineStr">
         <is>
-          <t>SYTaDC</t>
+          <t>TACFMfPBTY</t>
         </is>
       </c>
       <c r="C161" s="26" t="inlineStr">
         <is>
-          <t>Start Year Transmission and Distribution Costs</t>
-        </is>
-      </c>
-      <c r="D161" s="26" t="inlineStr">
-        <is>
-          <t>Start Year Transmission Capital Costs, Start Year Distribution Capital Costs, Start Year Transmission OM Costs, Start Year Distribution OM Costs</t>
-        </is>
-      </c>
-      <c r="F161" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>Time Adjusted Capacity Factor Multiplier for Plants Built This Year</t>
+        </is>
+      </c>
+      <c r="F161" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>
@@ -4995,39 +5002,39 @@
       </c>
       <c r="B162" s="26" t="inlineStr">
         <is>
-          <t>TACFMfPBTY</t>
+          <t>TCCpUNEC</t>
         </is>
       </c>
       <c r="C162" s="26" t="inlineStr">
         <is>
-          <t>Time Adjusted Capacity Factor Multiplier for Plants Built This Year</t>
-        </is>
-      </c>
-      <c r="F162" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>Transmission Construction Cost per Unit New Electricity Capacity</t>
+        </is>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
     </row>
     <row r="163" ht="60" customHeight="1" s="27">
-      <c r="A163" s="26" t="inlineStr">
+      <c r="A163" t="inlineStr">
         <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B163" s="26" t="inlineStr">
-        <is>
-          <t>TCCpUNEC</t>
-        </is>
-      </c>
-      <c r="C163" s="26" t="inlineStr">
-        <is>
-          <t>Transmission Construction Cost per Unit New Electricity Capacity</t>
-        </is>
-      </c>
-      <c r="F163" s="5" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="B163" s="29" t="inlineStr">
+        <is>
+          <t>TURiaPY</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Typical Units Retired in a Peak Year</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cement breakout: acronym-key rating fixes from the regional-adaptability audit
CPSW and MASCM raised to importance high for new-country adaptation (entry
gates reflect region-specific commercialization landscapes; SCM supply needs
country-specific ash/slag/pozzolan data), with update-condition notes added.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/InputData/acronym-key.xlsx
+++ b/InputData/acronym-key.xlsx
@@ -6380,7 +6380,12 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>to be determined via calibration</t>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Entry-gate years reflect the region-specific commercialization landscape for CCS, electric kilns, and alternative chemistries.</t>
         </is>
       </c>
     </row>
@@ -6801,7 +6806,12 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Regional SCM supply (fly ash, slag, pozzolans) requires country-specific data from ash/slag associations or national statistics.</t>
         </is>
       </c>
     </row>

</xml_diff>